<commit_message>
docs: add sparse accuracy comparison sheet
Add a formatted Accuracy worksheet with PPL, Commonsense, MMLU, and GSM8K comparisons against Dense. Validation: reopened and rendered both worksheets and found no formula errors.
</commit_message>
<xml_diff>
--- a/docs/hybrid_sparse_performance.xlsx
+++ b/docs/hybrid_sparse_performance.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="Rb60abf710f7443f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="Rd09d9b84c9e64e89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R7f704ca729164a00"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,11 +14,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="200" formatCode="0.00"/>
     <x:numFmt numFmtId="201" formatCode="0.000x"/>
+    <x:numFmt numFmtId="202" formatCode="0%"/>
+    <x:numFmt numFmtId="203" formatCode="0.0000"/>
+    <x:numFmt numFmtId="204" formatCode="0.00%"/>
+    <x:numFmt numFmtId="205" formatCode="0.00 &quot;pp&quot;"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -50,8 +55,14 @@
       <x:color rgb="FF475569"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1E3A5F"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -83,8 +94,13 @@
         <x:fgColor rgb="FFF8FAFC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEFF6FF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="10">
+  <x:borders count="16">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -167,11 +183,53 @@
         <x:color rgb="FFCBD5E1"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="49">
+  <x:cellXfs count="89">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -278,6 +336,114 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="4" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="4" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="4" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="4" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="4" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="4" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="4" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="4" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="4" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="4" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="4" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="4" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="6" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="6" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="6" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="6" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -741,4 +907,432 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="27" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="27" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="19" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="19" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>Qwen1.5-MoE Sparse Accuracy Comparison</x:v>
+      </x:c>
+      <x:c r="B1" s="3"/>
+      <x:c r="C1" s="3"/>
+      <x:c r="D1" s="3"/>
+      <x:c r="E1" s="3"/>
+      <x:c r="F1" s="3"/>
+      <x:c r="G1" s="3"/>
+      <x:c r="H1" s="3"/>
+      <x:c r="I1" s="3"/>
+      <x:c r="J1" s="3"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Qwen/Qwen1.5-MoE-A2.7B | Wanda | 128 WikiText2 calibration samples | routed experts only</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+      <x:c r="I2" s="6"/>
+      <x:c r="J2" s="6"/>
+    </x:row>
+    <x:row r="4" ht="36" customHeight="1">
+      <x:c r="A4" s="18" t="str">
+        <x:v>Configuration</x:v>
+      </x:c>
+      <x:c r="B4" s="19" t="str">
+        <x:v>Sparse pattern</x:v>
+      </x:c>
+      <x:c r="C4" s="19" t="str">
+        <x:v>Block shape</x:v>
+      </x:c>
+      <x:c r="D4" s="19" t="str">
+        <x:v>Sparsity</x:v>
+      </x:c>
+      <x:c r="E4" s="19" t="str">
+        <x:v>WikiText2 PPL</x:v>
+      </x:c>
+      <x:c r="F4" s="19" t="str">
+        <x:v>PPL delta vs Dense</x:v>
+      </x:c>
+      <x:c r="G4" s="19" t="str">
+        <x:v>Commonsense avg</x:v>
+      </x:c>
+      <x:c r="H4" s="19" t="str">
+        <x:v>Commonsense delta</x:v>
+      </x:c>
+      <x:c r="I4" s="19" t="str">
+        <x:v>MMLU 5-shot</x:v>
+      </x:c>
+      <x:c r="J4" s="20" t="str">
+        <x:v>GSM8K 5-shot flexible</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="66" t="str">
+        <x:v>Dense</x:v>
+      </x:c>
+      <x:c r="B5" s="66" t="str">
+        <x:v>Dense</x:v>
+      </x:c>
+      <x:c r="C5" s="66" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="D5" s="67" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="68" t="n">
+        <x:v>7.2173</x:v>
+      </x:c>
+      <x:c r="F5" s="68" t="n">
+        <x:f>E5-$E$5</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G5" s="69" t="n">
+        <x:v>0.6639</x:v>
+      </x:c>
+      <x:c r="H5" s="70" t="n">
+        <x:f>(G5-$G$5)*100</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I5" s="69" t="n">
+        <x:v>0.6124</x:v>
+      </x:c>
+      <x:c r="J5" s="69" t="n">
+        <x:v>0.6065</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="30" t="str">
+        <x:v>SlideSparse 6:8</x:v>
+      </x:c>
+      <x:c r="B6" s="30" t="str">
+        <x:v>6:8 element sparse</x:v>
+      </x:c>
+      <x:c r="C6" s="30" t="str">
+        <x:v>Vector</x:v>
+      </x:c>
+      <x:c r="D6" s="50" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="E6" s="53" t="n">
+        <x:v>7.3003</x:v>
+      </x:c>
+      <x:c r="F6" s="53" t="n">
+        <x:f>E6-$E$5</x:f>
+        <x:v>0.08300000000000018</x:v>
+      </x:c>
+      <x:c r="G6" s="56" t="n">
+        <x:v>0.659506</x:v>
+      </x:c>
+      <x:c r="H6" s="59" t="n">
+        <x:f>(G6-$G$5)*100</x:f>
+        <x:v>-0.4394000000000009</x:v>
+      </x:c>
+      <x:c r="I6" s="56" t="n">
+        <x:v>0.6087</x:v>
+      </x:c>
+      <x:c r="J6" s="56" t="n">
+        <x:v>0.6035</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="30" t="str">
+        <x:v>Hybrid Block Sparse 1x4</x:v>
+      </x:c>
+      <x:c r="B7" s="30" t="str">
+        <x:v>1-of-2 blocks use 2:4</x:v>
+      </x:c>
+      <x:c r="C7" s="30" t="str">
+        <x:v>1 x 4</x:v>
+      </x:c>
+      <x:c r="D7" s="50" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="E7" s="53" t="n">
+        <x:v>7.3666</x:v>
+      </x:c>
+      <x:c r="F7" s="53" t="n">
+        <x:f>E7-$E$5</x:f>
+        <x:v>0.1493000000000002</x:v>
+      </x:c>
+      <x:c r="G7" s="56" t="n">
+        <x:v>0.660879</x:v>
+      </x:c>
+      <x:c r="H7" s="59" t="n">
+        <x:f>(G7-$G$5)*100</x:f>
+        <x:v>-0.30210000000000514</x:v>
+      </x:c>
+      <x:c r="I7" s="56"/>
+      <x:c r="J7" s="56"/>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="30" t="str">
+        <x:v>Hybrid Block Sparse 4x4</x:v>
+      </x:c>
+      <x:c r="B8" s="30" t="str">
+        <x:v>1-of-2 blocks use 2:4</x:v>
+      </x:c>
+      <x:c r="C8" s="30" t="str">
+        <x:v>4 x 4</x:v>
+      </x:c>
+      <x:c r="D8" s="50" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="E8" s="53" t="n">
+        <x:v>7.4606</x:v>
+      </x:c>
+      <x:c r="F8" s="53" t="n">
+        <x:f>E8-$E$5</x:f>
+        <x:v>0.24330000000000052</x:v>
+      </x:c>
+      <x:c r="G8" s="56" t="n">
+        <x:v>0.659993</x:v>
+      </x:c>
+      <x:c r="H8" s="59" t="n">
+        <x:f>(G8-$G$5)*100</x:f>
+        <x:v>-0.3906999999999994</x:v>
+      </x:c>
+      <x:c r="I8" s="56"/>
+      <x:c r="J8" s="56"/>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="30" t="str">
+        <x:v>Hybrid Block Sparse 16x16</x:v>
+      </x:c>
+      <x:c r="B9" s="30" t="str">
+        <x:v>1-of-2 blocks use 2:4</x:v>
+      </x:c>
+      <x:c r="C9" s="30" t="str">
+        <x:v>16 x 16</x:v>
+      </x:c>
+      <x:c r="D9" s="50" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="E9" s="53" t="n">
+        <x:v>7.5743</x:v>
+      </x:c>
+      <x:c r="F9" s="53" t="n">
+        <x:f>E9-$E$5</x:f>
+        <x:v>0.3570000000000002</x:v>
+      </x:c>
+      <x:c r="G9" s="56" t="n">
+        <x:v>0.659448</x:v>
+      </x:c>
+      <x:c r="H9" s="59" t="n">
+        <x:f>(G9-$G$5)*100</x:f>
+        <x:v>-0.44520000000000115</x:v>
+      </x:c>
+      <x:c r="I9" s="56"/>
+      <x:c r="J9" s="56"/>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="30" t="str">
+        <x:v>Hybrid Block Sparse 64x64</x:v>
+      </x:c>
+      <x:c r="B10" s="30" t="str">
+        <x:v>1-of-2 blocks use 2:4</x:v>
+      </x:c>
+      <x:c r="C10" s="30" t="str">
+        <x:v>64 x 64</x:v>
+      </x:c>
+      <x:c r="D10" s="50" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="E10" s="53" t="n">
+        <x:v>7.6273</x:v>
+      </x:c>
+      <x:c r="F10" s="53" t="n">
+        <x:f>E10-$E$5</x:f>
+        <x:v>0.41000000000000014</x:v>
+      </x:c>
+      <x:c r="G10" s="56" t="n">
+        <x:v>0.6569</x:v>
+      </x:c>
+      <x:c r="H10" s="59" t="n">
+        <x:f>(G10-$G$5)*100</x:f>
+        <x:v>-0.7000000000000006</x:v>
+      </x:c>
+      <x:c r="I10" s="56"/>
+      <x:c r="J10" s="56"/>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="30" t="str">
+        <x:v>HB-N:M 50%</x:v>
+      </x:c>
+      <x:c r="B11" s="30" t="str">
+        <x:v>All blocks use 2:4</x:v>
+      </x:c>
+      <x:c r="C11" s="30" t="str">
+        <x:v>16 x 16</x:v>
+      </x:c>
+      <x:c r="D11" s="50" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E11" s="53" t="n">
+        <x:v>8.54</x:v>
+      </x:c>
+      <x:c r="F11" s="53" t="n">
+        <x:f>E11-$E$5</x:f>
+        <x:v>1.3226999999999993</x:v>
+      </x:c>
+      <x:c r="G11" s="56" t="n">
+        <x:v>0.6394</x:v>
+      </x:c>
+      <x:c r="H11" s="59" t="n">
+        <x:f>(G11-$G$5)*100</x:f>
+        <x:v>-2.4500000000000077</x:v>
+      </x:c>
+      <x:c r="I11" s="56" t="n">
+        <x:v>0.5583</x:v>
+      </x:c>
+      <x:c r="J11" s="56" t="n">
+        <x:v>0.4049</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="31" t="str">
+        <x:v>HB-N:M 75%</x:v>
+      </x:c>
+      <x:c r="B12" s="31" t="str">
+        <x:v>1-of-2 blocks kept + 2:4</x:v>
+      </x:c>
+      <x:c r="C12" s="31" t="str">
+        <x:v>16 x 16</x:v>
+      </x:c>
+      <x:c r="D12" s="51" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="E12" s="54" t="n">
+        <x:v>218.85</x:v>
+      </x:c>
+      <x:c r="F12" s="54" t="n">
+        <x:f>E12-$E$5</x:f>
+        <x:v>211.6327</x:v>
+      </x:c>
+      <x:c r="G12" s="57" t="n">
+        <x:v>0.3984</x:v>
+      </x:c>
+      <x:c r="H12" s="60" t="n">
+        <x:f>(G12-$G$5)*100</x:f>
+        <x:v>-26.550000000000008</x:v>
+      </x:c>
+      <x:c r="I12" s="57" t="n">
+        <x:v>0.2522</x:v>
+      </x:c>
+      <x:c r="J12" s="57" t="n">
+        <x:v>0.0114</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="83" t="str">
+        <x:v>Sources: qwen1_5_moe_structured_sparsity_accuracy.md and qwen1_5_moe_hybrid_block_sparse_results.md. Blank cells indicate metrics that were not evaluated. Lower PPL and higher accuracy are better.</x:v>
+      </x:c>
+      <x:c r="B14" s="84"/>
+      <x:c r="C14" s="84"/>
+      <x:c r="D14" s="84"/>
+      <x:c r="E14" s="84"/>
+      <x:c r="F14" s="84"/>
+      <x:c r="G14" s="84"/>
+      <x:c r="H14" s="84"/>
+      <x:c r="I14" s="84"/>
+      <x:c r="J14" s="85"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="86"/>
+      <x:c r="B15" s="87"/>
+      <x:c r="C15" s="87"/>
+      <x:c r="D15" s="87"/>
+      <x:c r="E15" s="87"/>
+      <x:c r="F15" s="87"/>
+      <x:c r="G15" s="87"/>
+      <x:c r="H15" s="87"/>
+      <x:c r="I15" s="87"/>
+      <x:c r="J15" s="88"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A2:J2"/>
+    <x:mergeCell ref="A14:J15"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="E5:E12">
+    <x:cfRule type="colorScale" priority="1">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="num" val="9"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFBBF7D0"/>
+        <x:color rgb="FFFEF3C7"/>
+        <x:color rgb="FFFECACA"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="F6:F12">
+    <x:cfRule type="colorScale" priority="2">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="num" val="0.5"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFFEF3C7"/>
+        <x:color rgb="FFFED7AA"/>
+        <x:color rgb="FFFECACA"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G5:G12">
+    <x:cfRule type="colorScale" priority="3">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="num" val="0.64"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFFECACA"/>
+        <x:color rgb="FFFEF3C7"/>
+        <x:color rgb="FFBBF7D0"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="H6:H12">
+    <x:cfRule type="colorScale" priority="4">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="num" val="-1"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFFECACA"/>
+        <x:color rgb="FFFEF3C7"/>
+        <x:color rgb="FFBBF7D0"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="I5:J12">
+    <x:cfRule type="colorScale" priority="5">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFFECACA"/>
+        <x:color rgb="FFFEF3C7"/>
+        <x:color rgb="FFBBF7D0"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record persistent metadata results
Add a dedicated workbook sheet for persistent scheduling and lane-ready metadata benchmarks, including the target-shape NCU comparison. Mark both experiments complete in the optimization checklist.
</commit_message>
<xml_diff>
--- a/docs/hybrid_sparse_performance.xlsx
+++ b/docs/hybrid_sparse_performance.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="Rd09d9b84c9e64e89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R7f704ca729164a00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R96df9866cc324aa9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="Rb44229c2d6864b12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R9288c611de1d4fcd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,15 +15,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="8">
     <x:numFmt numFmtId="200" formatCode="0.00"/>
     <x:numFmt numFmtId="201" formatCode="0.000x"/>
     <x:numFmt numFmtId="202" formatCode="0%"/>
     <x:numFmt numFmtId="203" formatCode="0.0000"/>
     <x:numFmt numFmtId="204" formatCode="0.00%"/>
     <x:numFmt numFmtId="205" formatCode="0.00 &quot;pp&quot;"/>
+    <x:numFmt numFmtId="206" formatCode="0.000"/>
+    <x:numFmt numFmtId="207" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -61,8 +64,37 @@
       <x:color rgb="FF1E3A5F"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="22"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF0B4F71"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF4B5C75"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -99,8 +131,28 @@
         <x:fgColor rgb="FFEFF6FF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1B2D5C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EDF9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF24466F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F7FB"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="16">
+  <x:borders count="17">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -225,11 +277,25 @@
         <x:color rgb="FFCBD5E1"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD6DFEA"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD6DFEA"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD6DFEA"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD6DFEA"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="89">
+  <x:cellXfs count="112">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -444,6 +510,51 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -456,7 +567,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -1335,4 +1446,545 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="21" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="21" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="21" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="23" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="38" customHeight="1">
+      <x:c r="A1" s="91" t="str">
+        <x:v>Persistent Scheduler + Lane-Ready Metadata</x:v>
+      </x:c>
+      <x:c r="B1" s="91"/>
+      <x:c r="C1" s="91"/>
+      <x:c r="D1" s="91"/>
+      <x:c r="E1" s="91"/>
+      <x:c r="F1" s="91"/>
+      <x:c r="G1" s="91"/>
+    </x:row>
+    <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="94" t="str">
+        <x:v>NVIDIA H20 | BF16 input/output | FP32 accumulation | 64 x 64 weight blocks | 1-of-2 blocks use 2:4 | L2 flush disabled</x:v>
+      </x:c>
+      <x:c r="B2" s="94"/>
+      <x:c r="C2" s="94"/>
+      <x:c r="D2" s="94"/>
+      <x:c r="E2" s="94"/>
+      <x:c r="F2" s="94"/>
+      <x:c r="G2" s="94"/>
+    </x:row>
+    <x:row r="4" ht="38" customHeight="1">
+      <x:c r="A4" s="99" t="str">
+        <x:v>Shape (M x N x K)</x:v>
+      </x:c>
+      <x:c r="B4" s="99" t="str">
+        <x:v>Fused STSM (us)</x:v>
+      </x:c>
+      <x:c r="C4" s="99" t="str">
+        <x:v>Persistent 3 CTA/SM (us)</x:v>
+      </x:c>
+      <x:c r="D4" s="99" t="str">
+        <x:v>Lane-ready (us)</x:v>
+      </x:c>
+      <x:c r="E4" s="99" t="str">
+        <x:v>DeepGEMM (us)</x:v>
+      </x:c>
+      <x:c r="F4" s="99" t="str">
+        <x:v>Speedup vs STSM</x:v>
+      </x:c>
+      <x:c r="G4" s="99" t="str">
+        <x:v>Speedup over DeepGEMM</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="101" t="str">
+        <x:v>128 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B5" s="103" t="n">
+        <x:v>18.62</x:v>
+      </x:c>
+      <x:c r="C5" s="103" t="n">
+        <x:v>17.28</x:v>
+      </x:c>
+      <x:c r="D5" s="103" t="n">
+        <x:v>14.69</x:v>
+      </x:c>
+      <x:c r="E5" s="103" t="n">
+        <x:v>9.9</x:v>
+      </x:c>
+      <x:c r="F5" s="104" t="n">
+        <x:f>B5/D5</x:f>
+        <x:v>1.2675289312457456</x:v>
+      </x:c>
+      <x:c r="G5" s="104" t="n">
+        <x:f>E5/D5</x:f>
+        <x:v>0.673927842069435</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="101" t="str">
+        <x:v>128 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B6" s="103" t="n">
+        <x:v>12.83</x:v>
+      </x:c>
+      <x:c r="C6" s="103" t="n">
+        <x:v>12.28</x:v>
+      </x:c>
+      <x:c r="D6" s="103" t="n">
+        <x:v>10.88</x:v>
+      </x:c>
+      <x:c r="E6" s="103" t="n">
+        <x:v>8.61</x:v>
+      </x:c>
+      <x:c r="F6" s="104" t="n">
+        <x:f>B6/D6</x:f>
+        <x:v>1.1792279411764706</x:v>
+      </x:c>
+      <x:c r="G6" s="104" t="n">
+        <x:f>E6/D6</x:f>
+        <x:v>0.791360294117647</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="101" t="str">
+        <x:v>256 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B7" s="103" t="n">
+        <x:v>24.26</x:v>
+      </x:c>
+      <x:c r="C7" s="103" t="n">
+        <x:v>23.7</x:v>
+      </x:c>
+      <x:c r="D7" s="103" t="n">
+        <x:v>22.07</x:v>
+      </x:c>
+      <x:c r="E7" s="103" t="n">
+        <x:v>13.89</x:v>
+      </x:c>
+      <x:c r="F7" s="104" t="n">
+        <x:f>B7/D7</x:f>
+        <x:v>1.099229723606706</x:v>
+      </x:c>
+      <x:c r="G7" s="104" t="n">
+        <x:f>E7/D7</x:f>
+        <x:v>0.6293611236973267</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="101" t="str">
+        <x:v>256 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B8" s="103" t="n">
+        <x:v>17.92</x:v>
+      </x:c>
+      <x:c r="C8" s="103" t="n">
+        <x:v>17.57</x:v>
+      </x:c>
+      <x:c r="D8" s="103" t="n">
+        <x:v>16.57</x:v>
+      </x:c>
+      <x:c r="E8" s="103" t="n">
+        <x:v>13.36</x:v>
+      </x:c>
+      <x:c r="F8" s="104" t="n">
+        <x:f>B8/D8</x:f>
+        <x:v>1.0814725407362704</x:v>
+      </x:c>
+      <x:c r="G8" s="104" t="n">
+        <x:f>E8/D8</x:f>
+        <x:v>0.8062764031382015</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="101" t="str">
+        <x:v>512 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B9" s="103" t="n">
+        <x:v>32.54</x:v>
+      </x:c>
+      <x:c r="C9" s="103" t="n">
+        <x:v>97.46</x:v>
+      </x:c>
+      <x:c r="D9" s="103" t="n">
+        <x:v>30.75</x:v>
+      </x:c>
+      <x:c r="E9" s="103" t="n">
+        <x:v>26.45</x:v>
+      </x:c>
+      <x:c r="F9" s="104" t="n">
+        <x:f>B9/D9</x:f>
+        <x:v>1.058211382113821</x:v>
+      </x:c>
+      <x:c r="G9" s="104" t="n">
+        <x:f>E9/D9</x:f>
+        <x:v>0.8601626016260162</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="101" t="str">
+        <x:v>512 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B10" s="103" t="n">
+        <x:v>90.97</x:v>
+      </x:c>
+      <x:c r="C10" s="103" t="n">
+        <x:v>37.07</x:v>
+      </x:c>
+      <x:c r="D10" s="103" t="n">
+        <x:v>34.13</x:v>
+      </x:c>
+      <x:c r="E10" s="103" t="n">
+        <x:v>26.57</x:v>
+      </x:c>
+      <x:c r="F10" s="104" t="n">
+        <x:f>B10/D10</x:f>
+        <x:v>2.665397011426897</x:v>
+      </x:c>
+      <x:c r="G10" s="104" t="n">
+        <x:f>E10/D10</x:f>
+        <x:v>0.778493993554058</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="101" t="str">
+        <x:v>1024 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B11" s="103" t="n">
+        <x:v>104.84</x:v>
+      </x:c>
+      <x:c r="C11" s="103" t="n">
+        <x:v>116.67</x:v>
+      </x:c>
+      <x:c r="D11" s="103" t="n">
+        <x:v>97.8</x:v>
+      </x:c>
+      <x:c r="E11" s="103" t="n">
+        <x:v>98.57</x:v>
+      </x:c>
+      <x:c r="F11" s="104" t="n">
+        <x:f>B11/D11</x:f>
+        <x:v>1.0719836400817997</x:v>
+      </x:c>
+      <x:c r="G11" s="104" t="n">
+        <x:f>E11/D11</x:f>
+        <x:v>1.0078732106339467</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="101" t="str">
+        <x:v>1024 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B12" s="103" t="n">
+        <x:v>104.48</x:v>
+      </x:c>
+      <x:c r="C12" s="103" t="n">
+        <x:v>112.97</x:v>
+      </x:c>
+      <x:c r="D12" s="103" t="n">
+        <x:v>98.75</x:v>
+      </x:c>
+      <x:c r="E12" s="103" t="n">
+        <x:v>97.22</x:v>
+      </x:c>
+      <x:c r="F12" s="104" t="n">
+        <x:f>B12/D12</x:f>
+        <x:v>1.0580253164556963</x:v>
+      </x:c>
+      <x:c r="G12" s="104" t="n">
+        <x:f>E12/D12</x:f>
+        <x:v>0.984506329113924</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="101" t="str">
+        <x:v>2048 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B13" s="103" t="n">
+        <x:v>193.1</x:v>
+      </x:c>
+      <x:c r="C13" s="103" t="n">
+        <x:v>280.45</x:v>
+      </x:c>
+      <x:c r="D13" s="103" t="n">
+        <x:v>142.21</x:v>
+      </x:c>
+      <x:c r="E13" s="103" t="n">
+        <x:v>194.62</x:v>
+      </x:c>
+      <x:c r="F13" s="104" t="n">
+        <x:f>B13/D13</x:f>
+        <x:v>1.3578510653259264</x:v>
+      </x:c>
+      <x:c r="G13" s="104" t="n">
+        <x:f>E13/D13</x:f>
+        <x:v>1.3685394838618943</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="101" t="str">
+        <x:v>2048 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B14" s="103" t="n">
+        <x:v>95.17</x:v>
+      </x:c>
+      <x:c r="C14" s="103" t="n">
+        <x:v>129.61</x:v>
+      </x:c>
+      <x:c r="D14" s="103" t="n">
+        <x:v>91.3</x:v>
+      </x:c>
+      <x:c r="E14" s="103" t="n">
+        <x:v>93.03</x:v>
+      </x:c>
+      <x:c r="F14" s="104" t="n">
+        <x:f>B14/D14</x:f>
+        <x:v>1.0423877327491786</x:v>
+      </x:c>
+      <x:c r="G14" s="104" t="n">
+        <x:f>E14/D14</x:f>
+        <x:v>1.01894852135816</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="101" t="str">
+        <x:v>4096 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B15" s="103" t="n">
+        <x:v>172.46</x:v>
+      </x:c>
+      <x:c r="C15" s="103" t="n">
+        <x:v>265.21</x:v>
+      </x:c>
+      <x:c r="D15" s="103" t="n">
+        <x:v>172.96</x:v>
+      </x:c>
+      <x:c r="E15" s="103" t="n">
+        <x:v>184.29</x:v>
+      </x:c>
+      <x:c r="F15" s="104" t="n">
+        <x:f>B15/D15</x:f>
+        <x:v>0.997109158186864</x:v>
+      </x:c>
+      <x:c r="G15" s="104" t="n">
+        <x:f>E15/D15</x:f>
+        <x:v>1.0655064754856614</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="101" t="str">
+        <x:v>4096 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B16" s="103" t="n">
+        <x:v>174.23</x:v>
+      </x:c>
+      <x:c r="C16" s="103" t="n">
+        <x:v>269.04</x:v>
+      </x:c>
+      <x:c r="D16" s="103" t="n">
+        <x:v>167.28</x:v>
+      </x:c>
+      <x:c r="E16" s="103" t="n">
+        <x:v>182.11</x:v>
+      </x:c>
+      <x:c r="F16" s="104" t="n">
+        <x:f>B16/D16</x:f>
+        <x:v>1.041547106647537</x:v>
+      </x:c>
+      <x:c r="G16" s="104" t="n">
+        <x:f>E16/D16</x:f>
+        <x:v>1.0886537541846006</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="101" t="str">
+        <x:v>512 x 4096 x 4096</x:v>
+      </x:c>
+      <x:c r="B17" s="103" t="n">
+        <x:v>150.21</x:v>
+      </x:c>
+      <x:c r="C17" s="103" t="n">
+        <x:v>174.89</x:v>
+      </x:c>
+      <x:c r="D17" s="103" t="n">
+        <x:v>133.34</x:v>
+      </x:c>
+      <x:c r="E17" s="103" t="n">
+        <x:v>131.48</x:v>
+      </x:c>
+      <x:c r="F17" s="104" t="n">
+        <x:f>B17/D17</x:f>
+        <x:v>1.1265186740662967</x:v>
+      </x:c>
+      <x:c r="G17" s="104" t="n">
+        <x:f>E17/D17</x:f>
+        <x:v>0.9860506974651266</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="105" t="str">
+        <x:v>NCU comparison at 512 x 4096 x 4096</x:v>
+      </x:c>
+      <x:c r="B21" s="105"/>
+      <x:c r="C21" s="105"/>
+      <x:c r="D21" s="105"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="106" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B22" s="106" t="str">
+        <x:v>Persistent 3 CTA/SM</x:v>
+      </x:c>
+      <x:c r="C22" s="106" t="str">
+        <x:v>Lane-ready</x:v>
+      </x:c>
+      <x:c r="D22" s="106" t="str">
+        <x:v>Change</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="100" t="str">
+        <x:v>NCU duration (us)</x:v>
+      </x:c>
+      <x:c r="B23" s="107" t="n">
+        <x:v>192.448</x:v>
+      </x:c>
+      <x:c r="C23" s="107" t="n">
+        <x:v>161.632</x:v>
+      </x:c>
+      <x:c r="D23" s="108" t="n">
+        <x:f>C23/B23-1</x:f>
+        <x:v>-0.16012637179913536</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="100" t="str">
+        <x:v>Registers / thread</x:v>
+      </x:c>
+      <x:c r="B24" s="107" t="n">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="C24" s="107" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="D24" s="108" t="n">
+        <x:f>C24/B24-1</x:f>
+        <x:v>-0.34782608695652173</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="100" t="str">
+        <x:v>Dynamic shared memory (KB / CTA)</x:v>
+      </x:c>
+      <x:c r="B25" s="107" t="n">
+        <x:v>74.752</x:v>
+      </x:c>
+      <x:c r="C25" s="107" t="n">
+        <x:v>58.368</x:v>
+      </x:c>
+      <x:c r="D25" s="108" t="n">
+        <x:f>C25/B25-1</x:f>
+        <x:v>-0.2191780821917807</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="100" t="str">
+        <x:v>Active warps (% peak)</x:v>
+      </x:c>
+      <x:c r="B26" s="107" t="n">
+        <x:v>22.923226</x:v>
+      </x:c>
+      <x:c r="C26" s="107" t="n">
+        <x:v>34.313097</x:v>
+      </x:c>
+      <x:c r="D26" s="108" t="n">
+        <x:f>C26/B26-1</x:f>
+        <x:v>0.4968703357895612</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="100" t="str">
+        <x:v>Tensor pipe active (% peak)</x:v>
+      </x:c>
+      <x:c r="B27" s="107" t="n">
+        <x:v>14.900994</x:v>
+      </x:c>
+      <x:c r="C27" s="107" t="n">
+        <x:v>18.759332</x:v>
+      </x:c>
+      <x:c r="D27" s="108" t="n">
+        <x:f>C27/B27-1</x:f>
+        <x:v>0.25893158536940564</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="100" t="str">
+        <x:v>Warp instructions</x:v>
+      </x:c>
+      <x:c r="B28" s="107" t="n">
+        <x:v>21270725</x:v>
+      </x:c>
+      <x:c r="C28" s="107" t="n">
+        <x:v>14163518</x:v>
+      </x:c>
+      <x:c r="D28" s="108" t="n">
+        <x:f>C28/B28-1</x:f>
+        <x:v>-0.3341309240752255</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="38" customHeight="1">
+      <x:c r="A30" s="111" t="str">
+        <x:v>Benchmark note: all eight GPUs reported 96-100% utilization during the standard sweep, so isolated target-shape measurements and NCU deltas are more reliable than individual sweep outliers.</x:v>
+      </x:c>
+      <x:c r="B30" s="111"/>
+      <x:c r="C30" s="111"/>
+      <x:c r="D30" s="111"/>
+      <x:c r="E30" s="111"/>
+      <x:c r="F30" s="111"/>
+      <x:c r="G30" s="111"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A2:G2"/>
+    <x:mergeCell ref="A21:D21"/>
+    <x:mergeCell ref="A30:G30"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="G5:G17">
+    <x:cfRule type="colorScale" priority="1">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF9B9BC"/>
+        <x:color rgb="FFFFF0BF"/>
+        <x:color rgb="FFB8EDC9"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="F5:F17">
+    <x:cfRule type="colorScale" priority="2">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF9B9BC"/>
+        <x:color rgb="FFFFF0BF"/>
+        <x:color rgb="FFB8EDC9"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add cuBLAS Tensor Core baseline
Add a dedicated workbook sheet comparing lane-ready sparse GEMM with DeepGEMM and strict BF16 cuBLASLt. Record the FP32 accumulation configuration and NCU-confirmed HGMMA Tensor Core instruction.
</commit_message>
<xml_diff>
--- a/docs/hybrid_sparse_performance.xlsx
+++ b/docs/hybrid_sparse_performance.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R96df9866cc324aa9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="Rb44229c2d6864b12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R9288c611de1d4fcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R72c9142762364690"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="Rd0826a93bc5c423a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="Rb403a3f305284785"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="Rf46480aab8934609"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -94,7 +95,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="16">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -129,6 +130,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFEFF6FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1B2D5C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EDF9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF24466F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F7FB"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -295,7 +316,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="112">
+  <x:cellXfs count="128">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -554,6 +575,36 @@
     <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1987,4 +2038,510 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="27" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="21" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="21" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="23" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="23" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="38" customHeight="1">
+      <x:c r="A1" s="114" t="str">
+        <x:v>cuBLAS Tensor Core Baseline</x:v>
+      </x:c>
+      <x:c r="B1" s="114"/>
+      <x:c r="C1" s="114"/>
+      <x:c r="D1" s="114"/>
+      <x:c r="E1" s="114"/>
+      <x:c r="F1" s="114"/>
+      <x:c r="G1" s="114"/>
+    </x:row>
+    <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="117" t="str">
+        <x:v>NVIDIA H20 | BF16 input/output | FP32 compute and accumulation | cuBLASLt Tensor Core heuristic | L2 flush disabled</x:v>
+      </x:c>
+      <x:c r="B2" s="117"/>
+      <x:c r="C2" s="117"/>
+      <x:c r="D2" s="117"/>
+      <x:c r="E2" s="117"/>
+      <x:c r="F2" s="117"/>
+      <x:c r="G2" s="117"/>
+    </x:row>
+    <x:row r="4" ht="38" customHeight="1">
+      <x:c r="A4" s="122" t="str">
+        <x:v>Shape (M x N x K)</x:v>
+      </x:c>
+      <x:c r="B4" s="122" t="str">
+        <x:v>Lane-ready sparse (us)</x:v>
+      </x:c>
+      <x:c r="C4" s="122" t="str">
+        <x:v>DeepGEMM (us)</x:v>
+      </x:c>
+      <x:c r="D4" s="122" t="str">
+        <x:v>cuBLASLt (us)</x:v>
+      </x:c>
+      <x:c r="E4" s="122" t="str">
+        <x:v>Speedup over DeepGEMM</x:v>
+      </x:c>
+      <x:c r="F4" s="122" t="str">
+        <x:v>Speedup over cuBLASLt</x:v>
+      </x:c>
+      <x:c r="G4" s="122" t="str">
+        <x:v>cuBLASLt vs DeepGEMM</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="101" t="str">
+        <x:v>128 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B5" s="103" t="n">
+        <x:v>15.43</x:v>
+      </x:c>
+      <x:c r="C5" s="103" t="n">
+        <x:v>10.1</x:v>
+      </x:c>
+      <x:c r="D5" s="103" t="n">
+        <x:v>8.41</x:v>
+      </x:c>
+      <x:c r="E5" s="104" t="n">
+        <x:f>C5/B5</x:f>
+        <x:v>0.6545690213869086</x:v>
+      </x:c>
+      <x:c r="F5" s="104" t="n">
+        <x:f>D5/B5</x:f>
+        <x:v>0.5450421257290992</x:v>
+      </x:c>
+      <x:c r="G5" s="104" t="n">
+        <x:f>C5/D5</x:f>
+        <x:v>1.2009512485136742</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="101" t="str">
+        <x:v>128 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B6" s="103" t="n">
+        <x:v>11.52</x:v>
+      </x:c>
+      <x:c r="C6" s="103" t="n">
+        <x:v>9.09</x:v>
+      </x:c>
+      <x:c r="D6" s="103" t="n">
+        <x:v>8.22</x:v>
+      </x:c>
+      <x:c r="E6" s="104" t="n">
+        <x:f>C6/B6</x:f>
+        <x:v>0.7890625</x:v>
+      </x:c>
+      <x:c r="F6" s="104" t="n">
+        <x:f>D6/B6</x:f>
+        <x:v>0.7135416666666667</x:v>
+      </x:c>
+      <x:c r="G6" s="104" t="n">
+        <x:f>C6/D6</x:f>
+        <x:v>1.105839416058394</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="101" t="str">
+        <x:v>256 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B7" s="103" t="n">
+        <x:v>22.92</x:v>
+      </x:c>
+      <x:c r="C7" s="103" t="n">
+        <x:v>14.08</x:v>
+      </x:c>
+      <x:c r="D7" s="103" t="n">
+        <x:v>13.92</x:v>
+      </x:c>
+      <x:c r="E7" s="104" t="n">
+        <x:f>C7/B7</x:f>
+        <x:v>0.6143106457242582</x:v>
+      </x:c>
+      <x:c r="F7" s="104" t="n">
+        <x:f>D7/B7</x:f>
+        <x:v>0.6073298429319371</x:v>
+      </x:c>
+      <x:c r="G7" s="104" t="n">
+        <x:f>C7/D7</x:f>
+        <x:v>1.0114942528735633</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="101" t="str">
+        <x:v>256 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B8" s="103" t="n">
+        <x:v>16.93</x:v>
+      </x:c>
+      <x:c r="C8" s="103" t="n">
+        <x:v>13.73</x:v>
+      </x:c>
+      <x:c r="D8" s="103" t="n">
+        <x:v>13.89</x:v>
+      </x:c>
+      <x:c r="E8" s="104" t="n">
+        <x:f>C8/B8</x:f>
+        <x:v>0.8109864146485529</x:v>
+      </x:c>
+      <x:c r="F8" s="104" t="n">
+        <x:f>D8/B8</x:f>
+        <x:v>0.8204370939161253</x:v>
+      </x:c>
+      <x:c r="G8" s="104" t="n">
+        <x:f>C8/D8</x:f>
+        <x:v>0.9884809215262779</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="101" t="str">
+        <x:v>512 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B9" s="103" t="n">
+        <x:v>32.29</x:v>
+      </x:c>
+      <x:c r="C9" s="103" t="n">
+        <x:v>30.15</x:v>
+      </x:c>
+      <x:c r="D9" s="103" t="n">
+        <x:v>30.16</x:v>
+      </x:c>
+      <x:c r="E9" s="104" t="n">
+        <x:f>C9/B9</x:f>
+        <x:v>0.933725611644472</x:v>
+      </x:c>
+      <x:c r="F9" s="104" t="n">
+        <x:f>D9/B9</x:f>
+        <x:v>0.9340353050480025</x:v>
+      </x:c>
+      <x:c r="G9" s="104" t="n">
+        <x:f>C9/D9</x:f>
+        <x:v>0.9996684350132625</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="101" t="str">
+        <x:v>512 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B10" s="103" t="n">
+        <x:v>32.03</x:v>
+      </x:c>
+      <x:c r="C10" s="103" t="n">
+        <x:v>25.56</x:v>
+      </x:c>
+      <x:c r="D10" s="103" t="n">
+        <x:v>25.15</x:v>
+      </x:c>
+      <x:c r="E10" s="104" t="n">
+        <x:f>C10/B10</x:f>
+        <x:v>0.7980018732438339</x:v>
+      </x:c>
+      <x:c r="F10" s="104" t="n">
+        <x:f>D10/B10</x:f>
+        <x:v>0.7852013737121448</x:v>
+      </x:c>
+      <x:c r="G10" s="104" t="n">
+        <x:f>C10/D10</x:f>
+        <x:v>1.0163021868787276</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="101" t="str">
+        <x:v>1024 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B11" s="103" t="n">
+        <x:v>97.36</x:v>
+      </x:c>
+      <x:c r="C11" s="103" t="n">
+        <x:v>98.5</x:v>
+      </x:c>
+      <x:c r="D11" s="103" t="n">
+        <x:v>98.15</x:v>
+      </x:c>
+      <x:c r="E11" s="104" t="n">
+        <x:f>C11/B11</x:f>
+        <x:v>1.011709120788825</x:v>
+      </x:c>
+      <x:c r="F11" s="104" t="n">
+        <x:f>D11/B11</x:f>
+        <x:v>1.008114215283484</x:v>
+      </x:c>
+      <x:c r="G11" s="104" t="n">
+        <x:f>C11/D11</x:f>
+        <x:v>1.0035659704533877</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="101" t="str">
+        <x:v>1024 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B12" s="103" t="n">
+        <x:v>99.29</x:v>
+      </x:c>
+      <x:c r="C12" s="103" t="n">
+        <x:v>97.68</x:v>
+      </x:c>
+      <x:c r="D12" s="103" t="n">
+        <x:v>96.27</x:v>
+      </x:c>
+      <x:c r="E12" s="104" t="n">
+        <x:f>C12/B12</x:f>
+        <x:v>0.9837848725954276</x:v>
+      </x:c>
+      <x:c r="F12" s="104" t="n">
+        <x:f>D12/B12</x:f>
+        <x:v>0.9695840467317957</x:v>
+      </x:c>
+      <x:c r="G12" s="104" t="n">
+        <x:f>C12/D12</x:f>
+        <x:v>1.014646307260829</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="101" t="str">
+        <x:v>2048 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B13" s="103" t="n">
+        <x:v>191.6</x:v>
+      </x:c>
+      <x:c r="C13" s="103" t="n">
+        <x:v>194.5</x:v>
+      </x:c>
+      <x:c r="D13" s="103" t="n">
+        <x:v>196.1</x:v>
+      </x:c>
+      <x:c r="E13" s="104" t="n">
+        <x:f>C13/B13</x:f>
+        <x:v>1.0151356993736953</x:v>
+      </x:c>
+      <x:c r="F13" s="104" t="n">
+        <x:f>D13/B13</x:f>
+        <x:v>1.0234864300626305</x:v>
+      </x:c>
+      <x:c r="G13" s="104" t="n">
+        <x:f>C13/D13</x:f>
+        <x:v>0.9918408975012749</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="101" t="str">
+        <x:v>2048 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B14" s="103" t="n">
+        <x:v>91.28</x:v>
+      </x:c>
+      <x:c r="C14" s="103" t="n">
+        <x:v>93.36</x:v>
+      </x:c>
+      <x:c r="D14" s="103" t="n">
+        <x:v>91.35</x:v>
+      </x:c>
+      <x:c r="E14" s="104" t="n">
+        <x:f>C14/B14</x:f>
+        <x:v>1.0227870289219982</x:v>
+      </x:c>
+      <x:c r="F14" s="104" t="n">
+        <x:f>D14/B14</x:f>
+        <x:v>1.0007668711656441</x:v>
+      </x:c>
+      <x:c r="G14" s="104" t="n">
+        <x:f>C14/D14</x:f>
+        <x:v>1.0220032840722497</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="101" t="str">
+        <x:v>4096 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B15" s="103" t="n">
+        <x:v>174.99</x:v>
+      </x:c>
+      <x:c r="C15" s="103" t="n">
+        <x:v>182.95</x:v>
+      </x:c>
+      <x:c r="D15" s="103" t="n">
+        <x:v>185.86</x:v>
+      </x:c>
+      <x:c r="E15" s="104" t="n">
+        <x:f>C15/B15</x:f>
+        <x:v>1.045488313617921</x:v>
+      </x:c>
+      <x:c r="F15" s="104" t="n">
+        <x:f>D15/B15</x:f>
+        <x:v>1.0621178353048746</x:v>
+      </x:c>
+      <x:c r="G15" s="104" t="n">
+        <x:f>C15/D15</x:f>
+        <x:v>0.9843430539115462</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="101" t="str">
+        <x:v>4096 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B16" s="103" t="n">
+        <x:v>168.31</x:v>
+      </x:c>
+      <x:c r="C16" s="103" t="n">
+        <x:v>182</x:v>
+      </x:c>
+      <x:c r="D16" s="103" t="n">
+        <x:v>175.71</x:v>
+      </x:c>
+      <x:c r="E16" s="104" t="n">
+        <x:f>C16/B16</x:f>
+        <x:v>1.0813380072485295</x:v>
+      </x:c>
+      <x:c r="F16" s="104" t="n">
+        <x:f>D16/B16</x:f>
+        <x:v>1.0439664904046106</x:v>
+      </x:c>
+      <x:c r="G16" s="104" t="n">
+        <x:f>C16/D16</x:f>
+        <x:v>1.035797621080189</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="101" t="str">
+        <x:v>512 x 4096 x 4096</x:v>
+      </x:c>
+      <x:c r="B17" s="103" t="n">
+        <x:v>133.58</x:v>
+      </x:c>
+      <x:c r="C17" s="103" t="n">
+        <x:v>131.28</x:v>
+      </x:c>
+      <x:c r="D17" s="103" t="n">
+        <x:v>130.85</x:v>
+      </x:c>
+      <x:c r="E17" s="104" t="n">
+        <x:f>C17/B17</x:f>
+        <x:v>0.9827818535708938</x:v>
+      </x:c>
+      <x:c r="F17" s="104" t="n">
+        <x:f>D17/B17</x:f>
+        <x:v>0.979562808803713</x:v>
+      </x:c>
+      <x:c r="G17" s="104" t="n">
+        <x:f>C17/D17</x:f>
+        <x:v>1.0032862055789071</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="123" t="str">
+        <x:v>cuBLASLt configuration and NCU confirmation</x:v>
+      </x:c>
+      <x:c r="B21" s="123"/>
+      <x:c r="C21" s="123"/>
+      <x:c r="D21" s="123"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="124" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B22" s="124" t="str">
+        <x:v>Observed value</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="100" t="str">
+        <x:v>Input / output dtype</x:v>
+      </x:c>
+      <x:c r="B23" s="100" t="str">
+        <x:v>BF16 / BF16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="100" t="str">
+        <x:v>Compute / accumulator type</x:v>
+      </x:c>
+      <x:c r="B24" s="100" t="str">
+        <x:v>CUBLAS_COMPUTE_32F / FP32</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="100" t="str">
+        <x:v>Algorithm selection</x:v>
+      </x:c>
+      <x:c r="B25" s="100" t="str">
+        <x:v>cuBLASLt Tensor Core heuristic</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="100" t="str">
+        <x:v>Observed SASS</x:v>
+      </x:c>
+      <x:c r="B26" s="100" t="str">
+        <x:v>HGMMA.64x112x16.F32.BF16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="100" t="str">
+        <x:v>Tensor pipe active (% peak)</x:v>
+      </x:c>
+      <x:c r="B27" s="107" t="n">
+        <x:v>24.390369</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="100" t="str">
+        <x:v>Target-shape NCU duration (us)</x:v>
+      </x:c>
+      <x:c r="B28" s="107" t="n">
+        <x:v>143.968</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="38" customHeight="1">
+      <x:c r="A30" s="127" t="str">
+        <x:v>Speedup is baseline latency divided by lane-ready sparse latency. Values above 1.0x mean the sparse kernel is faster. NCU duration includes profiling replay overhead and should not be compared directly with benchmark latency.</x:v>
+      </x:c>
+      <x:c r="B30" s="127"/>
+      <x:c r="C30" s="127"/>
+      <x:c r="D30" s="127"/>
+      <x:c r="E30" s="127"/>
+      <x:c r="F30" s="127"/>
+      <x:c r="G30" s="127"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A2:G2"/>
+    <x:mergeCell ref="A21:D21"/>
+    <x:mergeCell ref="A30:G30"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="E5:E17">
+    <x:cfRule type="colorScale" priority="1">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF9B9BC"/>
+        <x:color rgb="FFFFF0BF"/>
+        <x:color rgb="FFB8EDC9"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="F5:F17">
+    <x:cfRule type="colorScale" priority="2">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF9B9BC"/>
+        <x:color rgb="FFFFF0BF"/>
+        <x:color rgb="FFB8EDC9"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record 128x32 stage-three experiment
Add benchmark and NCU comparisons to the performance workbook and mark the strategy as evaluated but not selected.
</commit_message>
<xml_diff>
--- a/docs/hybrid_sparse_performance.xlsx
+++ b/docs/hybrid_sparse_performance.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R72c9142762364690"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="Rd0826a93bc5c423a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="Rb403a3f305284785"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="Rf46480aab8934609"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R612d3501b96049c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R4b8546eb9b9443ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R3eac93cc1bb8460b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="R6dd60ac6ee124a46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="R08256476ce4545a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +27,7 @@
     <x:numFmt numFmtId="206" formatCode="0.000"/>
     <x:numFmt numFmtId="207" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="12">
+  <x:fonts count="21">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -94,8 +95,58 @@
       <x:color rgb="FF4B5C75"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="20"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF075985"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF475569"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="20"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF075985"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF475569"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="20">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -172,8 +223,28 @@
         <x:fgColor rgb="FFF4F7FB"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1D3265"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD8ECF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF294F7A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF1F5F9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="17">
+  <x:borders count="20">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -312,11 +383,32 @@
         <x:color rgb="FFD6DFEA"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7E0EA"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD7E0EA"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7E0EA"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD7E0EA"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFA8B7C7"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="128">
+  <x:cellXfs count="166">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -605,6 +697,66 @@
     <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="11" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="11" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="18" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="17" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="17" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="17" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="17" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="17" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="17" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2544,4 +2696,522 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="35" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="152" t="str">
+        <x:v>128 x 32 Weight Tile + Three-Stage TMA</x:v>
+      </x:c>
+      <x:c r="B1" s="152"/>
+      <x:c r="C1" s="152"/>
+      <x:c r="D1" s="152"/>
+      <x:c r="E1" s="152"/>
+      <x:c r="F1" s="152"/>
+      <x:c r="G1" s="152"/>
+      <x:c r="H1" s="152"/>
+      <x:c r="I1" s="152"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="153" t="str">
+        <x:v>NVIDIA H20 | BF16 input/output | FP32 accumulation | 1-of-2 blocks use 2:4 | L2 flush disabled</x:v>
+      </x:c>
+      <x:c r="B2" s="153"/>
+      <x:c r="C2" s="153"/>
+      <x:c r="D2" s="153"/>
+      <x:c r="E2" s="153"/>
+      <x:c r="F2" s="153"/>
+      <x:c r="G2" s="153"/>
+      <x:c r="H2" s="153"/>
+      <x:c r="I2" s="153"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="154"/>
+      <x:c r="B3" s="154"/>
+      <x:c r="C3" s="154"/>
+      <x:c r="D3" s="154"/>
+      <x:c r="E3" s="154"/>
+      <x:c r="F3" s="154"/>
+      <x:c r="G3" s="154"/>
+      <x:c r="H3" s="154"/>
+      <x:c r="I3" s="154"/>
+    </x:row>
+    <x:row r="4" ht="36" customHeight="1">
+      <x:c r="A4" s="155" t="str">
+        <x:v>Shape (M x N x K)</x:v>
+      </x:c>
+      <x:c r="B4" s="155" t="str">
+        <x:v>Sparse latency (us)</x:v>
+      </x:c>
+      <x:c r="C4" s="155" t="str">
+        <x:v>Dense latency (us)</x:v>
+      </x:c>
+      <x:c r="D4" s="155" t="str">
+        <x:v>Reduce (us)</x:v>
+      </x:c>
+      <x:c r="E4" s="155" t="str">
+        <x:v>Total (us)</x:v>
+      </x:c>
+      <x:c r="F4" s="155" t="str">
+        <x:v>DeepGEMM (us)</x:v>
+      </x:c>
+      <x:c r="G4" s="155" t="str">
+        <x:v>Speedup over DeepGEMM</x:v>
+      </x:c>
+      <x:c r="H4" s="155" t="str">
+        <x:v>Stage-2 total (us)</x:v>
+      </x:c>
+      <x:c r="I4" s="155" t="str">
+        <x:v>Change vs Stage-2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="156" t="str">
+        <x:v>512 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B5" s="157" t="n">
+        <x:v>29.15</x:v>
+      </x:c>
+      <x:c r="C5" s="157" t="n">
+        <x:v>21.98</x:v>
+      </x:c>
+      <x:c r="D5" s="157" t="n">
+        <x:v>9.56</x:v>
+      </x:c>
+      <x:c r="E5" s="157" t="n">
+        <x:v>60.7</x:v>
+      </x:c>
+      <x:c r="F5" s="157" t="n">
+        <x:v>25.19</x:v>
+      </x:c>
+      <x:c r="G5" s="158" t="n">
+        <x:f>F5/E5</x:f>
+        <x:v>0.41499176276771005</x:v>
+      </x:c>
+      <x:c r="H5" s="157" t="n">
+        <x:v>60.64</x:v>
+      </x:c>
+      <x:c r="I5" s="159" t="n">
+        <x:f>E5/H5-1</x:f>
+        <x:v>0.0009894459102903763</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="156" t="str">
+        <x:v>1024 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B6" s="157" t="n">
+        <x:v>58.11</x:v>
+      </x:c>
+      <x:c r="C6" s="157" t="n">
+        <x:v>41.62</x:v>
+      </x:c>
+      <x:c r="D6" s="157" t="n">
+        <x:v>10.84</x:v>
+      </x:c>
+      <x:c r="E6" s="157" t="n">
+        <x:v>110.57</x:v>
+      </x:c>
+      <x:c r="F6" s="157" t="n">
+        <x:v>48.99</x:v>
+      </x:c>
+      <x:c r="G6" s="158" t="n">
+        <x:f>F6/E6</x:f>
+        <x:v>0.4430677398932803</x:v>
+      </x:c>
+      <x:c r="H6" s="157" t="n">
+        <x:v>108.5</x:v>
+      </x:c>
+      <x:c r="I6" s="159" t="n">
+        <x:f>E6/H6-1</x:f>
+        <x:v>0.019078341013824884</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="156" t="str">
+        <x:v>2048 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B7" s="157" t="n">
+        <x:v>104.37</x:v>
+      </x:c>
+      <x:c r="C7" s="157" t="n">
+        <x:v>63.69</x:v>
+      </x:c>
+      <x:c r="D7" s="157" t="n">
+        <x:v>16.56</x:v>
+      </x:c>
+      <x:c r="E7" s="157" t="n">
+        <x:v>184.62</x:v>
+      </x:c>
+      <x:c r="F7" s="157" t="n">
+        <x:v>94.78</x:v>
+      </x:c>
+      <x:c r="G7" s="158" t="n">
+        <x:f>F7/E7</x:f>
+        <x:v>0.5133788321958618</x:v>
+      </x:c>
+      <x:c r="H7" s="157" t="n">
+        <x:v>202.41</x:v>
+      </x:c>
+      <x:c r="I7" s="159" t="n">
+        <x:f>E7/H7-1</x:f>
+        <x:v>-0.08789091448050979</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="160" t="str">
+        <x:v>4096 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B8" s="161" t="n">
+        <x:v>185.78</x:v>
+      </x:c>
+      <x:c r="C8" s="161" t="n">
+        <x:v>106.27</x:v>
+      </x:c>
+      <x:c r="D8" s="161" t="n">
+        <x:v>37.99</x:v>
+      </x:c>
+      <x:c r="E8" s="161" t="n">
+        <x:v>330.04</x:v>
+      </x:c>
+      <x:c r="F8" s="161" t="n">
+        <x:v>183.01</x:v>
+      </x:c>
+      <x:c r="G8" s="162" t="n">
+        <x:f>F8/E8</x:f>
+        <x:v>0.5545085444188582</x:v>
+      </x:c>
+      <x:c r="H8" s="161" t="n">
+        <x:v>329.27</x:v>
+      </x:c>
+      <x:c r="I8" s="163" t="n">
+        <x:f>E8/H8-1</x:f>
+        <x:v>0.0023385063929299843</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="154"/>
+      <x:c r="B9" s="154"/>
+      <x:c r="C9" s="154"/>
+      <x:c r="D9" s="154"/>
+      <x:c r="E9" s="154"/>
+      <x:c r="F9" s="154"/>
+      <x:c r="G9" s="154"/>
+      <x:c r="H9" s="154"/>
+      <x:c r="I9" s="154"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="154"/>
+      <x:c r="B10" s="154"/>
+      <x:c r="C10" s="154"/>
+      <x:c r="D10" s="154"/>
+      <x:c r="E10" s="154"/>
+      <x:c r="F10" s="154"/>
+      <x:c r="G10" s="154"/>
+      <x:c r="H10" s="154"/>
+      <x:c r="I10" s="154"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="164" t="str">
+        <x:v>NCU: Sparse Kernel at 1024 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B11" s="164"/>
+      <x:c r="C11" s="164"/>
+      <x:c r="D11" s="164"/>
+      <x:c r="E11" s="154"/>
+      <x:c r="F11" s="154"/>
+      <x:c r="G11" s="154"/>
+      <x:c r="H11" s="154"/>
+      <x:c r="I11" s="154"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="155" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B12" s="155" t="str">
+        <x:v>Stage 2</x:v>
+      </x:c>
+      <x:c r="C12" s="155" t="str">
+        <x:v>Stage 3</x:v>
+      </x:c>
+      <x:c r="D12" s="155" t="str">
+        <x:v>Change</x:v>
+      </x:c>
+      <x:c r="E12" s="154"/>
+      <x:c r="F12" s="154"/>
+      <x:c r="G12" s="154"/>
+      <x:c r="H12" s="154"/>
+      <x:c r="I12" s="154"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="156" t="str">
+        <x:v>NCU duration (us)</x:v>
+      </x:c>
+      <x:c r="B13" s="157" t="n">
+        <x:v>84.29</x:v>
+      </x:c>
+      <x:c r="C13" s="157" t="n">
+        <x:v>83.58</x:v>
+      </x:c>
+      <x:c r="D13" s="159" t="n">
+        <x:f>C13/B13-1</x:f>
+        <x:v>-0.008423300510143616</x:v>
+      </x:c>
+      <x:c r="E13" s="154"/>
+      <x:c r="F13" s="154"/>
+      <x:c r="G13" s="154"/>
+      <x:c r="H13" s="154"/>
+      <x:c r="I13" s="154"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="156" t="str">
+        <x:v>Memory throughput (% peak)</x:v>
+      </x:c>
+      <x:c r="B14" s="157" t="n">
+        <x:v>10.58</x:v>
+      </x:c>
+      <x:c r="C14" s="157" t="n">
+        <x:v>10.98</x:v>
+      </x:c>
+      <x:c r="D14" s="159" t="n">
+        <x:f>C14/B14-1</x:f>
+        <x:v>0.03780718336483946</x:v>
+      </x:c>
+      <x:c r="E14" s="154"/>
+      <x:c r="F14" s="154"/>
+      <x:c r="G14" s="154"/>
+      <x:c r="H14" s="154"/>
+      <x:c r="I14" s="154"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="156" t="str">
+        <x:v>DRAM throughput (% peak)</x:v>
+      </x:c>
+      <x:c r="B15" s="157" t="n">
+        <x:v>1.78</x:v>
+      </x:c>
+      <x:c r="C15" s="157" t="n">
+        <x:v>1.79</x:v>
+      </x:c>
+      <x:c r="D15" s="159" t="n">
+        <x:f>C15/B15-1</x:f>
+        <x:v>0.00561797752808979</x:v>
+      </x:c>
+      <x:c r="E15" s="154"/>
+      <x:c r="F15" s="154"/>
+      <x:c r="G15" s="154"/>
+      <x:c r="H15" s="154"/>
+      <x:c r="I15" s="154"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="156" t="str">
+        <x:v>SM busy (%)</x:v>
+      </x:c>
+      <x:c r="B16" s="157" t="n">
+        <x:v>20.6</x:v>
+      </x:c>
+      <x:c r="C16" s="157" t="n">
+        <x:v>21.16</x:v>
+      </x:c>
+      <x:c r="D16" s="159" t="n">
+        <x:f>C16/B16-1</x:f>
+        <x:v>0.027184466019417375</x:v>
+      </x:c>
+      <x:c r="E16" s="154"/>
+      <x:c r="F16" s="154"/>
+      <x:c r="G16" s="154"/>
+      <x:c r="H16" s="154"/>
+      <x:c r="I16" s="154"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="156" t="str">
+        <x:v>Eligible warps / scheduler</x:v>
+      </x:c>
+      <x:c r="B17" s="157" t="n">
+        <x:v>0.22</x:v>
+      </x:c>
+      <x:c r="C17" s="157" t="n">
+        <x:v>0.22</x:v>
+      </x:c>
+      <x:c r="D17" s="159" t="n">
+        <x:f>C17/B17-1</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="154"/>
+      <x:c r="F17" s="154"/>
+      <x:c r="G17" s="154"/>
+      <x:c r="H17" s="154"/>
+      <x:c r="I17" s="154"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="156" t="str">
+        <x:v>Registers / thread</x:v>
+      </x:c>
+      <x:c r="B18" s="157" t="n">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="C18" s="157" t="n">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="D18" s="159" t="n">
+        <x:f>C18/B18-1</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="154"/>
+      <x:c r="F18" s="154"/>
+      <x:c r="G18" s="154"/>
+      <x:c r="H18" s="154"/>
+      <x:c r="I18" s="154"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="156" t="str">
+        <x:v>Dynamic shared memory (KB / CTA)</x:v>
+      </x:c>
+      <x:c r="B19" s="157" t="n">
+        <x:v>16.42</x:v>
+      </x:c>
+      <x:c r="C19" s="157" t="n">
+        <x:v>24.62</x:v>
+      </x:c>
+      <x:c r="D19" s="159" t="n">
+        <x:f>C19/B19-1</x:f>
+        <x:v>0.4993909866017052</x:v>
+      </x:c>
+      <x:c r="E19" s="154"/>
+      <x:c r="F19" s="154"/>
+      <x:c r="G19" s="154"/>
+      <x:c r="H19" s="154"/>
+      <x:c r="I19" s="154"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="156" t="str">
+        <x:v>Theoretical occupancy (%)</x:v>
+      </x:c>
+      <x:c r="B20" s="157" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C20" s="157" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D20" s="159" t="n">
+        <x:f>C20/B20-1</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E20" s="154"/>
+      <x:c r="F20" s="154"/>
+      <x:c r="G20" s="154"/>
+      <x:c r="H20" s="154"/>
+      <x:c r="I20" s="154"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="156" t="str">
+        <x:v>Achieved occupancy (%)</x:v>
+      </x:c>
+      <x:c r="B21" s="157" t="n">
+        <x:v>14.19</x:v>
+      </x:c>
+      <x:c r="C21" s="157" t="n">
+        <x:v>14.23</x:v>
+      </x:c>
+      <x:c r="D21" s="159" t="n">
+        <x:f>C21/B21-1</x:f>
+        <x:v>0.0028188865398168783</x:v>
+      </x:c>
+      <x:c r="E21" s="154"/>
+      <x:c r="F21" s="154"/>
+      <x:c r="G21" s="154"/>
+      <x:c r="H21" s="154"/>
+      <x:c r="I21" s="154"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="160" t="str">
+        <x:v>Long scoreboard stall (%)</x:v>
+      </x:c>
+      <x:c r="B22" s="161" t="n">
+        <x:v>59.6</x:v>
+      </x:c>
+      <x:c r="C22" s="161" t="n">
+        <x:v>57.8</x:v>
+      </x:c>
+      <x:c r="D22" s="163" t="n">
+        <x:f>C22/B22-1</x:f>
+        <x:v>-0.030201342281879318</x:v>
+      </x:c>
+      <x:c r="E22" s="154"/>
+      <x:c r="F22" s="154"/>
+      <x:c r="G22" s="154"/>
+      <x:c r="H22" s="154"/>
+      <x:c r="I22" s="154"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="154"/>
+      <x:c r="B23" s="154"/>
+      <x:c r="C23" s="154"/>
+      <x:c r="D23" s="154"/>
+      <x:c r="E23" s="154"/>
+      <x:c r="F23" s="154"/>
+      <x:c r="G23" s="154"/>
+      <x:c r="H23" s="154"/>
+      <x:c r="I23" s="154"/>
+    </x:row>
+    <x:row r="24" ht="34" customHeight="1">
+      <x:c r="A24" s="165" t="str">
+        <x:v>Decision: keep the three-stage kernel as an experimental version; do not dispatch M &gt; 512 to it because the end-to-end latency did not improve consistently.</x:v>
+      </x:c>
+      <x:c r="B24" s="165"/>
+      <x:c r="C24" s="165"/>
+      <x:c r="D24" s="165"/>
+      <x:c r="E24" s="165"/>
+      <x:c r="F24" s="165"/>
+      <x:c r="G24" s="165"/>
+      <x:c r="H24" s="165"/>
+      <x:c r="I24" s="165"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:I1"/>
+    <x:mergeCell ref="A2:I2"/>
+    <x:mergeCell ref="A11:D11"/>
+    <x:mergeCell ref="A24:I24"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="G5:G8">
+    <x:cfRule type="colorScale" priority="1">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF8B4B4"/>
+        <x:color rgb="FFFEF3C7"/>
+        <x:color rgb="FFB7EFC5"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="I5:I8">
+    <x:cfRule type="colorScale" priority="2">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFB7EFC5"/>
+        <x:color rgb="FFFEF3C7"/>
+        <x:color rgb="FFF8B4B4"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record merge K2 kernel experiment
Add the standard sweep and NCU comparison to the performance workbook, and mark merge_k2 as evaluated but not selected.
</commit_message>
<xml_diff>
--- a/docs/hybrid_sparse_performance.xlsx
+++ b/docs/hybrid_sparse_performance.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R612d3501b96049c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R4b8546eb9b9443ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R3eac93cc1bb8460b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="R6dd60ac6ee124a46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="R08256476ce4545a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="Rfa37073b19cc40c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R46a966e28ff04cbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R3112d3eebf00486d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="Rbcab98cc148d474d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="Rebafcfb0eeea4773"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="R6ae6e6906c8b40fa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +18,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="8">
+  <x:numFmts count="9">
     <x:numFmt numFmtId="200" formatCode="0.00"/>
     <x:numFmt numFmtId="201" formatCode="0.000x"/>
     <x:numFmt numFmtId="202" formatCode="0%"/>
@@ -26,6 +27,7 @@
     <x:numFmt numFmtId="205" formatCode="0.00 &quot;pp&quot;"/>
     <x:numFmt numFmtId="206" formatCode="0.000"/>
     <x:numFmt numFmtId="207" formatCode="0.0%"/>
+    <x:numFmt numFmtId="208" formatCode="#,##0"/>
   </x:numFmts>
   <x:fonts count="21">
     <x:font>
@@ -146,7 +148,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="20">
+  <x:fills count="24">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -221,6 +223,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF4F7FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1D3265"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD8ECF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF294F7A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF1F5F9"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -408,7 +430,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="166">
+  <x:cellXfs count="183">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -757,6 +779,37 @@
     <x:xf numFmtId="207" fontId="17" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="19" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="20" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="22" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="17" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -3214,4 +3267,652 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="35" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="17" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="17" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="168" t="str">
+        <x:v>Merge Two K Blocks per WGMMA Group</x:v>
+      </x:c>
+      <x:c r="B1" s="168"/>
+      <x:c r="C1" s="168"/>
+      <x:c r="D1" s="168"/>
+      <x:c r="E1" s="168"/>
+      <x:c r="F1" s="168"/>
+      <x:c r="G1" s="168"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="171" t="str">
+        <x:v>NVIDIA H20 | BF16 input/output | FP32 accumulation | 64 x 64 weight blocks | lane-ready metadata | L2 flush disabled</x:v>
+      </x:c>
+      <x:c r="B2" s="171"/>
+      <x:c r="C2" s="171"/>
+      <x:c r="D2" s="171"/>
+      <x:c r="E2" s="171"/>
+      <x:c r="F2" s="171"/>
+      <x:c r="G2" s="171"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="154"/>
+      <x:c r="B3" s="154"/>
+      <x:c r="C3" s="154"/>
+      <x:c r="D3" s="154"/>
+      <x:c r="E3" s="154"/>
+      <x:c r="F3" s="154"/>
+      <x:c r="G3" s="154"/>
+    </x:row>
+    <x:row r="4" ht="36" customHeight="1">
+      <x:c r="A4" s="178" t="str">
+        <x:v>Shape (M x N x K)</x:v>
+      </x:c>
+      <x:c r="B4" s="178" t="str">
+        <x:v>Lane-ready (us)</x:v>
+      </x:c>
+      <x:c r="C4" s="178" t="str">
+        <x:v>Merge K2 (us)</x:v>
+      </x:c>
+      <x:c r="D4" s="178" t="str">
+        <x:v>DeepGEMM (us)</x:v>
+      </x:c>
+      <x:c r="E4" s="178" t="str">
+        <x:v>cuBLASLt (us)</x:v>
+      </x:c>
+      <x:c r="F4" s="178" t="str">
+        <x:v>Speedup over DeepGEMM</x:v>
+      </x:c>
+      <x:c r="G4" s="178" t="str">
+        <x:v>Change vs Lane-ready</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="156" t="str">
+        <x:v>128 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B5" s="157" t="n">
+        <x:v>15.02</x:v>
+      </x:c>
+      <x:c r="C5" s="157" t="n">
+        <x:v>19.73</x:v>
+      </x:c>
+      <x:c r="D5" s="157" t="n">
+        <x:v>9.86</x:v>
+      </x:c>
+      <x:c r="E5" s="157" t="n">
+        <x:v>8.22</x:v>
+      </x:c>
+      <x:c r="F5" s="158" t="n">
+        <x:f>D5/C5</x:f>
+        <x:v>0.4997465788139888</x:v>
+      </x:c>
+      <x:c r="G5" s="159" t="n">
+        <x:f>C5/B5-1</x:f>
+        <x:v>0.3135818908122503</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="156" t="str">
+        <x:v>128 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B6" s="157" t="n">
+        <x:v>11.23</x:v>
+      </x:c>
+      <x:c r="C6" s="157" t="n">
+        <x:v>14.35</x:v>
+      </x:c>
+      <x:c r="D6" s="157" t="n">
+        <x:v>8.87</x:v>
+      </x:c>
+      <x:c r="E6" s="157" t="n">
+        <x:v>8.03</x:v>
+      </x:c>
+      <x:c r="F6" s="158" t="n">
+        <x:f>D6/C6</x:f>
+        <x:v>0.6181184668989547</x:v>
+      </x:c>
+      <x:c r="G6" s="159" t="n">
+        <x:f>C6/B6-1</x:f>
+        <x:v>0.27782724844167395</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="156" t="str">
+        <x:v>256 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B7" s="157" t="n">
+        <x:v>22.96</x:v>
+      </x:c>
+      <x:c r="C7" s="157" t="n">
+        <x:v>24.72</x:v>
+      </x:c>
+      <x:c r="D7" s="157" t="n">
+        <x:v>14.93</x:v>
+      </x:c>
+      <x:c r="E7" s="157" t="n">
+        <x:v>14.72</x:v>
+      </x:c>
+      <x:c r="F7" s="158" t="n">
+        <x:f>D7/C7</x:f>
+        <x:v>0.6039644012944984</x:v>
+      </x:c>
+      <x:c r="G7" s="159" t="n">
+        <x:f>C7/B7-1</x:f>
+        <x:v>0.07665505226480818</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="156" t="str">
+        <x:v>256 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B8" s="157" t="n">
+        <x:v>17.94</x:v>
+      </x:c>
+      <x:c r="C8" s="157" t="n">
+        <x:v>19.18</x:v>
+      </x:c>
+      <x:c r="D8" s="157" t="n">
+        <x:v>14.45</x:v>
+      </x:c>
+      <x:c r="E8" s="157" t="n">
+        <x:v>14.53</x:v>
+      </x:c>
+      <x:c r="F8" s="158" t="n">
+        <x:f>D8/C8</x:f>
+        <x:v>0.7533889468196038</x:v>
+      </x:c>
+      <x:c r="G8" s="159" t="n">
+        <x:f>C8/B8-1</x:f>
+        <x:v>0.06911928651059074</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="156" t="str">
+        <x:v>512 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B9" s="157" t="n">
+        <x:v>30.53</x:v>
+      </x:c>
+      <x:c r="C9" s="157" t="n">
+        <x:v>30.43</x:v>
+      </x:c>
+      <x:c r="D9" s="157" t="n">
+        <x:v>25.79</x:v>
+      </x:c>
+      <x:c r="E9" s="157" t="n">
+        <x:v>25.94</x:v>
+      </x:c>
+      <x:c r="F9" s="158" t="n">
+        <x:f>D9/C9</x:f>
+        <x:v>0.847518895826487</x:v>
+      </x:c>
+      <x:c r="G9" s="159" t="n">
+        <x:f>C9/B9-1</x:f>
+        <x:v>-0.0032754667540124682</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="156" t="str">
+        <x:v>512 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B10" s="157" t="n">
+        <x:v>31.06</x:v>
+      </x:c>
+      <x:c r="C10" s="157" t="n">
+        <x:v>34.24</x:v>
+      </x:c>
+      <x:c r="D10" s="157" t="n">
+        <x:v>24.84</x:v>
+      </x:c>
+      <x:c r="E10" s="157" t="n">
+        <x:v>24.78</x:v>
+      </x:c>
+      <x:c r="F10" s="158" t="n">
+        <x:f>D10/C10</x:f>
+        <x:v>0.7254672897196262</x:v>
+      </x:c>
+      <x:c r="G10" s="159" t="n">
+        <x:f>C10/B10-1</x:f>
+        <x:v>0.10238248551191265</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="156" t="str">
+        <x:v>1024 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B11" s="157" t="n">
+        <x:v>49.94</x:v>
+      </x:c>
+      <x:c r="C11" s="157" t="n">
+        <x:v>51.51</x:v>
+      </x:c>
+      <x:c r="D11" s="157" t="n">
+        <x:v>48.84</x:v>
+      </x:c>
+      <x:c r="E11" s="157" t="n">
+        <x:v>48.81</x:v>
+      </x:c>
+      <x:c r="F11" s="158" t="n">
+        <x:f>D11/C11</x:f>
+        <x:v>0.9481654047757718</x:v>
+      </x:c>
+      <x:c r="G11" s="159" t="n">
+        <x:f>C11/B11-1</x:f>
+        <x:v>0.0314377252703244</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="156" t="str">
+        <x:v>1024 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B12" s="157" t="n">
+        <x:v>49.78</x:v>
+      </x:c>
+      <x:c r="C12" s="157" t="n">
+        <x:v>52.4</x:v>
+      </x:c>
+      <x:c r="D12" s="157" t="n">
+        <x:v>47.06</x:v>
+      </x:c>
+      <x:c r="E12" s="157" t="n">
+        <x:v>46.03</x:v>
+      </x:c>
+      <x:c r="F12" s="158" t="n">
+        <x:f>D12/C12</x:f>
+        <x:v>0.8980916030534352</x:v>
+      </x:c>
+      <x:c r="G12" s="159" t="n">
+        <x:f>C12/B12-1</x:f>
+        <x:v>0.05263157894736836</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="156" t="str">
+        <x:v>2048 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B13" s="157" t="n">
+        <x:v>92.71</x:v>
+      </x:c>
+      <x:c r="C13" s="157" t="n">
+        <x:v>95.69</x:v>
+      </x:c>
+      <x:c r="D13" s="157" t="n">
+        <x:v>94.5</x:v>
+      </x:c>
+      <x:c r="E13" s="157" t="n">
+        <x:v>94.02</x:v>
+      </x:c>
+      <x:c r="F13" s="158" t="n">
+        <x:f>D13/C13</x:f>
+        <x:v>0.9875640087783467</x:v>
+      </x:c>
+      <x:c r="G13" s="159" t="n">
+        <x:f>C13/B13-1</x:f>
+        <x:v>0.032143242368676495</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="156" t="str">
+        <x:v>2048 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B14" s="157" t="n">
+        <x:v>90.78</x:v>
+      </x:c>
+      <x:c r="C14" s="157" t="n">
+        <x:v>92.31</x:v>
+      </x:c>
+      <x:c r="D14" s="157" t="n">
+        <x:v>92.39</x:v>
+      </x:c>
+      <x:c r="E14" s="157" t="n">
+        <x:v>90.5</x:v>
+      </x:c>
+      <x:c r="F14" s="158" t="n">
+        <x:f>D14/C14</x:f>
+        <x:v>1.0008666450005417</x:v>
+      </x:c>
+      <x:c r="G14" s="159" t="n">
+        <x:f>C14/B14-1</x:f>
+        <x:v>0.016853932584269593</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="156" t="str">
+        <x:v>4096 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B15" s="157" t="n">
+        <x:v>170.26</x:v>
+      </x:c>
+      <x:c r="C15" s="157" t="n">
+        <x:v>173.35</x:v>
+      </x:c>
+      <x:c r="D15" s="157" t="n">
+        <x:v>182.62</x:v>
+      </x:c>
+      <x:c r="E15" s="157" t="n">
+        <x:v>185.71</x:v>
+      </x:c>
+      <x:c r="F15" s="158" t="n">
+        <x:f>D15/C15</x:f>
+        <x:v>1.0534756273435246</x:v>
+      </x:c>
+      <x:c r="G15" s="159" t="n">
+        <x:f>C15/B15-1</x:f>
+        <x:v>0.01814871373193938</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="160" t="str">
+        <x:v>4096 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B16" s="161" t="n">
+        <x:v>168.81</x:v>
+      </x:c>
+      <x:c r="C16" s="161" t="n">
+        <x:v>169.53</x:v>
+      </x:c>
+      <x:c r="D16" s="161" t="n">
+        <x:v>182.29</x:v>
+      </x:c>
+      <x:c r="E16" s="161" t="n">
+        <x:v>175.79</x:v>
+      </x:c>
+      <x:c r="F16" s="162" t="n">
+        <x:f>D16/C16</x:f>
+        <x:v>1.0752669144104288</x:v>
+      </x:c>
+      <x:c r="G16" s="163" t="n">
+        <x:f>C16/B16-1</x:f>
+        <x:v>0.004265150168828891</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="154"/>
+      <x:c r="B17" s="154"/>
+      <x:c r="C17" s="154"/>
+      <x:c r="D17" s="154"/>
+      <x:c r="E17" s="154"/>
+      <x:c r="F17" s="154"/>
+      <x:c r="G17" s="154"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="154"/>
+      <x:c r="B18" s="154"/>
+      <x:c r="C18" s="154"/>
+      <x:c r="D18" s="154"/>
+      <x:c r="E18" s="154"/>
+      <x:c r="F18" s="154"/>
+      <x:c r="G18" s="154"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="177" t="str">
+        <x:v>NCU: 1024 x 1408 x 2048 Lane-Ready Kernel</x:v>
+      </x:c>
+      <x:c r="B19" s="177"/>
+      <x:c r="C19" s="177"/>
+      <x:c r="D19" s="177"/>
+      <x:c r="E19" s="154"/>
+      <x:c r="F19" s="154"/>
+      <x:c r="G19" s="154"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="178" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B20" s="178" t="str">
+        <x:v>Baseline</x:v>
+      </x:c>
+      <x:c r="C20" s="178" t="str">
+        <x:v>Merge K2</x:v>
+      </x:c>
+      <x:c r="D20" s="178" t="str">
+        <x:v>Change</x:v>
+      </x:c>
+      <x:c r="E20" s="154"/>
+      <x:c r="F20" s="154"/>
+      <x:c r="G20" s="154"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="156" t="str">
+        <x:v>NCU duration (us)</x:v>
+      </x:c>
+      <x:c r="B21" s="157" t="n">
+        <x:v>62.24</x:v>
+      </x:c>
+      <x:c r="C21" s="157" t="n">
+        <x:v>65.31</x:v>
+      </x:c>
+      <x:c r="D21" s="159" t="n">
+        <x:f>C21/B21-1</x:f>
+        <x:v>0.049325192802056606</x:v>
+      </x:c>
+      <x:c r="E21" s="154"/>
+      <x:c r="F21" s="154"/>
+      <x:c r="G21" s="154"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="156" t="str">
+        <x:v>SM busy (%)</x:v>
+      </x:c>
+      <x:c r="B22" s="157" t="n">
+        <x:v>68.91</x:v>
+      </x:c>
+      <x:c r="C22" s="157" t="n">
+        <x:v>62.23</x:v>
+      </x:c>
+      <x:c r="D22" s="159" t="n">
+        <x:f>C22/B22-1</x:f>
+        <x:v>-0.09693803511827026</x:v>
+      </x:c>
+      <x:c r="E22" s="154"/>
+      <x:c r="F22" s="154"/>
+      <x:c r="G22" s="154"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="156" t="str">
+        <x:v>Memory throughput (% peak)</x:v>
+      </x:c>
+      <x:c r="B23" s="157" t="n">
+        <x:v>22.06</x:v>
+      </x:c>
+      <x:c r="C23" s="157" t="n">
+        <x:v>21.43</x:v>
+      </x:c>
+      <x:c r="D23" s="159" t="n">
+        <x:f>C23/B23-1</x:f>
+        <x:v>-0.02855847688123292</x:v>
+      </x:c>
+      <x:c r="E23" s="154"/>
+      <x:c r="F23" s="154"/>
+      <x:c r="G23" s="154"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="156" t="str">
+        <x:v>DRAM throughput (% peak)</x:v>
+      </x:c>
+      <x:c r="B24" s="157" t="n">
+        <x:v>3.49</x:v>
+      </x:c>
+      <x:c r="C24" s="157" t="n">
+        <x:v>3.32</x:v>
+      </x:c>
+      <x:c r="D24" s="159" t="n">
+        <x:f>C24/B24-1</x:f>
+        <x:v>-0.04871060171919783</x:v>
+      </x:c>
+      <x:c r="E24" s="154"/>
+      <x:c r="F24" s="154"/>
+      <x:c r="G24" s="154"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="156" t="str">
+        <x:v>Eligible warps / scheduler</x:v>
+      </x:c>
+      <x:c r="B25" s="157" t="n">
+        <x:v>0.28</x:v>
+      </x:c>
+      <x:c r="C25" s="157" t="n">
+        <x:v>0.27</x:v>
+      </x:c>
+      <x:c r="D25" s="159" t="n">
+        <x:f>C25/B25-1</x:f>
+        <x:v>-0.0357142857142857</x:v>
+      </x:c>
+      <x:c r="E25" s="154"/>
+      <x:c r="F25" s="154"/>
+      <x:c r="G25" s="154"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="156" t="str">
+        <x:v>Warp cycles / issued instruction</x:v>
+      </x:c>
+      <x:c r="B26" s="157" t="n">
+        <x:v>24.13</x:v>
+      </x:c>
+      <x:c r="C26" s="157" t="n">
+        <x:v>21.37</x:v>
+      </x:c>
+      <x:c r="D26" s="159" t="n">
+        <x:f>C26/B26-1</x:f>
+        <x:v>-0.11438043928719432</x:v>
+      </x:c>
+      <x:c r="E26" s="154"/>
+      <x:c r="F26" s="154"/>
+      <x:c r="G26" s="154"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="156" t="str">
+        <x:v>Registers / thread</x:v>
+      </x:c>
+      <x:c r="B27" s="157" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C27" s="157" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="D27" s="159" t="n">
+        <x:f>C27/B27-1</x:f>
+        <x:v>0.050000000000000044</x:v>
+      </x:c>
+      <x:c r="E27" s="154"/>
+      <x:c r="F27" s="154"/>
+      <x:c r="G27" s="154"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="156" t="str">
+        <x:v>Achieved occupancy (%)</x:v>
+      </x:c>
+      <x:c r="B28" s="157" t="n">
+        <x:v>30.93</x:v>
+      </x:c>
+      <x:c r="C28" s="157" t="n">
+        <x:v>29.96</x:v>
+      </x:c>
+      <x:c r="D28" s="159" t="n">
+        <x:f>C28/B28-1</x:f>
+        <x:v>-0.03136113805366958</x:v>
+      </x:c>
+      <x:c r="E28" s="154"/>
+      <x:c r="F28" s="154"/>
+      <x:c r="G28" s="154"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="156" t="str">
+        <x:v>CTA barrier stall (%)</x:v>
+      </x:c>
+      <x:c r="B29" s="157" t="n">
+        <x:v>67.1</x:v>
+      </x:c>
+      <x:c r="C29" s="157" t="n">
+        <x:v>57.5</x:v>
+      </x:c>
+      <x:c r="D29" s="159" t="n">
+        <x:f>C29/B29-1</x:f>
+        <x:v>-0.1430700447093889</x:v>
+      </x:c>
+      <x:c r="E29" s="154"/>
+      <x:c r="F29" s="154"/>
+      <x:c r="G29" s="154"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="160" t="str">
+        <x:v>Executed instructions</x:v>
+      </x:c>
+      <x:c r="B30" s="179" t="n">
+        <x:v>5105987</x:v>
+      </x:c>
+      <x:c r="C30" s="179" t="n">
+        <x:v>6231332</x:v>
+      </x:c>
+      <x:c r="D30" s="163" t="n">
+        <x:f>C30/B30-1</x:f>
+        <x:v>0.22039715338092325</x:v>
+      </x:c>
+      <x:c r="E30" s="154"/>
+      <x:c r="F30" s="154"/>
+      <x:c r="G30" s="154"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="154"/>
+      <x:c r="B31" s="154"/>
+      <x:c r="C31" s="154"/>
+      <x:c r="D31" s="154"/>
+      <x:c r="E31" s="154"/>
+      <x:c r="F31" s="154"/>
+      <x:c r="G31" s="154"/>
+    </x:row>
+    <x:row r="32" ht="38" customHeight="1">
+      <x:c r="A32" s="182" t="str">
+        <x:v>Decision: preserve the implementation but do not select it. Barrier stalls fell, but two-stage buffer reuse became coarser and instruction count increased, so end-to-end latency regressed on most shapes.</x:v>
+      </x:c>
+      <x:c r="B32" s="182"/>
+      <x:c r="C32" s="182"/>
+      <x:c r="D32" s="182"/>
+      <x:c r="E32" s="182"/>
+      <x:c r="F32" s="182"/>
+      <x:c r="G32" s="182"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A2:G2"/>
+    <x:mergeCell ref="A19:D19"/>
+    <x:mergeCell ref="A32:G32"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="F5:F16">
+    <x:cfRule type="colorScale" priority="1">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF8B4B4"/>
+        <x:color rgb="FFFEF3C7"/>
+        <x:color rgb="FFB7EFC5"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G5:G16">
+    <x:cfRule type="colorScale" priority="2">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFB7EFC5"/>
+        <x:color rgb="FFFEF3C7"/>
+        <x:color rgb="FFF8B4B4"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record TMA pipeline stage experiment
Add median latency and fixed-shape NCU occupancy results for the 3-, 4-, and 5-stage 64 x 64 kernels. Record Stage 3 as the selected depth because Stage 4 and Stage 5 lose CTA residency.
</commit_message>
<xml_diff>
--- a/docs/hybrid_sparse_performance.xlsx
+++ b/docs/hybrid_sparse_performance.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="Rfa37073b19cc40c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R46a966e28ff04cbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R3112d3eebf00486d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="Rbcab98cc148d474d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="Rebafcfb0eeea4773"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="R6ae6e6906c8b40fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="Re9730e67123e4611"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R5fbaa80d48ed430a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="Rb1608c13041242d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="R79160dfc86dc4aad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="R257808f6a9f44a41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="R0aecc7acd3c74a17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="Rf48d9f1c90634b3b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -29,7 +30,7 @@
     <x:numFmt numFmtId="207" formatCode="0.0%"/>
     <x:numFmt numFmtId="208" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="21">
+  <x:fonts count="22">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -147,8 +148,14 @@
       <x:color rgb="FF475569"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF166534"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="24">
+  <x:fills count="29">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -258,6 +265,31 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF294F7A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF1F5F9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1D3265"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD8ECF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF294F7A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F3E8"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -430,7 +462,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="183">
+  <x:cellXfs count="205">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -810,6 +842,46 @@
     <x:xf numFmtId="0" fontId="17" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="20" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="20" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="26" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="27" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="27" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="27" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="27" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="27" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="27" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -3915,4 +3987,998 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="19" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="19" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="19" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="185" t="str">
+        <x:v>64 x 64 Weight Block: TMA Pipeline Depth</x:v>
+      </x:c>
+      <x:c r="B1" s="185"/>
+      <x:c r="C1" s="185"/>
+      <x:c r="D1" s="185"/>
+      <x:c r="E1" s="185"/>
+      <x:c r="F1" s="185"/>
+      <x:c r="G1" s="185"/>
+      <x:c r="H1" s="185"/>
+      <x:c r="I1" s="185"/>
+      <x:c r="J1" s="185"/>
+      <x:c r="K1" s="185"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="188" t="str">
+        <x:v>NVIDIA H20 | BF16 input/output | FP32 accumulation | stage count is the only kernel variable | L2 flush disabled | latency is the median of 3 runs</x:v>
+      </x:c>
+      <x:c r="B2" s="188"/>
+      <x:c r="C2" s="188"/>
+      <x:c r="D2" s="188"/>
+      <x:c r="E2" s="188"/>
+      <x:c r="F2" s="188"/>
+      <x:c r="G2" s="188"/>
+      <x:c r="H2" s="188"/>
+      <x:c r="I2" s="188"/>
+      <x:c r="J2" s="188"/>
+      <x:c r="K2" s="188"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="154"/>
+      <x:c r="B3" s="154"/>
+      <x:c r="C3" s="154"/>
+      <x:c r="D3" s="154"/>
+      <x:c r="E3" s="154"/>
+      <x:c r="F3" s="154"/>
+      <x:c r="G3" s="154"/>
+      <x:c r="H3" s="154"/>
+      <x:c r="I3" s="154"/>
+      <x:c r="J3" s="154"/>
+      <x:c r="K3" s="154"/>
+    </x:row>
+    <x:row r="4" ht="42" customHeight="1">
+      <x:c r="A4" s="195" t="str">
+        <x:v>Shape (M x N x K)</x:v>
+      </x:c>
+      <x:c r="B4" s="195" t="str">
+        <x:v>Stage 2 (us)</x:v>
+      </x:c>
+      <x:c r="C4" s="195" t="str">
+        <x:v>Stage 3 (us)</x:v>
+      </x:c>
+      <x:c r="D4" s="195" t="str">
+        <x:v>Stage 4 (us)</x:v>
+      </x:c>
+      <x:c r="E4" s="195" t="str">
+        <x:v>Stage 5 (us)</x:v>
+      </x:c>
+      <x:c r="F4" s="195" t="str">
+        <x:v>DeepGEMM (us)</x:v>
+      </x:c>
+      <x:c r="G4" s="195" t="str">
+        <x:v>cuBLASLt (us)</x:v>
+      </x:c>
+      <x:c r="H4" s="195" t="str">
+        <x:v>Best stage</x:v>
+      </x:c>
+      <x:c r="I4" s="195" t="str">
+        <x:v>Best latency (us)</x:v>
+      </x:c>
+      <x:c r="J4" s="195" t="str">
+        <x:v>Speedup vs Stage 2</x:v>
+      </x:c>
+      <x:c r="K4" s="195" t="str">
+        <x:v>Speedup over DeepGEMM</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="156" t="str">
+        <x:v>128 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B5" s="157" t="n">
+        <x:v>16.37</x:v>
+      </x:c>
+      <x:c r="C5" s="157" t="n">
+        <x:v>16.03</x:v>
+      </x:c>
+      <x:c r="D5" s="157" t="n">
+        <x:v>15.99</x:v>
+      </x:c>
+      <x:c r="E5" s="157" t="n">
+        <x:v>15.39</x:v>
+      </x:c>
+      <x:c r="F5" s="157" t="n">
+        <x:v>9.99</x:v>
+      </x:c>
+      <x:c r="G5" s="157" t="n">
+        <x:v>8.23</x:v>
+      </x:c>
+      <x:c r="H5" s="200" t="str">
+        <x:v>Stage 5</x:v>
+      </x:c>
+      <x:c r="I5" s="157" t="n">
+        <x:f>MIN(B5:E5)</x:f>
+        <x:v>15.39</x:v>
+      </x:c>
+      <x:c r="J5" s="158" t="n">
+        <x:f>B5/I5</x:f>
+        <x:v>1.06367771280052</x:v>
+      </x:c>
+      <x:c r="K5" s="158" t="n">
+        <x:f>F5/I5</x:f>
+        <x:v>0.6491228070175439</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="156" t="str">
+        <x:v>128 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B6" s="157" t="n">
+        <x:v>11.17</x:v>
+      </x:c>
+      <x:c r="C6" s="157" t="n">
+        <x:v>11.52</x:v>
+      </x:c>
+      <x:c r="D6" s="157" t="n">
+        <x:v>11.59</x:v>
+      </x:c>
+      <x:c r="E6" s="157" t="n">
+        <x:v>11.84</x:v>
+      </x:c>
+      <x:c r="F6" s="157" t="n">
+        <x:v>9.31</x:v>
+      </x:c>
+      <x:c r="G6" s="157" t="n">
+        <x:v>8.4</x:v>
+      </x:c>
+      <x:c r="H6" s="200" t="str">
+        <x:v>Stage 2</x:v>
+      </x:c>
+      <x:c r="I6" s="157" t="n">
+        <x:f>MIN(B6:E6)</x:f>
+        <x:v>11.17</x:v>
+      </x:c>
+      <x:c r="J6" s="158" t="n">
+        <x:f>B6/I6</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K6" s="158" t="n">
+        <x:f>F6/I6</x:f>
+        <x:v>0.8334825425246196</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="156" t="str">
+        <x:v>256 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B7" s="157" t="n">
+        <x:v>46.6</x:v>
+      </x:c>
+      <x:c r="C7" s="157" t="n">
+        <x:v>46.91</x:v>
+      </x:c>
+      <x:c r="D7" s="157" t="n">
+        <x:v>46.69</x:v>
+      </x:c>
+      <x:c r="E7" s="157" t="n">
+        <x:v>46.59</x:v>
+      </x:c>
+      <x:c r="F7" s="157" t="n">
+        <x:v>14.11</x:v>
+      </x:c>
+      <x:c r="G7" s="157" t="n">
+        <x:v>13.94</x:v>
+      </x:c>
+      <x:c r="H7" s="200" t="str">
+        <x:v>Stage 5</x:v>
+      </x:c>
+      <x:c r="I7" s="157" t="n">
+        <x:f>MIN(B7:E7)</x:f>
+        <x:v>46.59</x:v>
+      </x:c>
+      <x:c r="J7" s="158" t="n">
+        <x:f>B7/I7</x:f>
+        <x:v>1.0002146383344064</x:v>
+      </x:c>
+      <x:c r="K7" s="158" t="n">
+        <x:f>F7/I7</x:f>
+        <x:v>0.3028546898476068</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="156" t="str">
+        <x:v>256 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B8" s="157" t="n">
+        <x:v>16.93</x:v>
+      </x:c>
+      <x:c r="C8" s="157" t="n">
+        <x:v>17.17</x:v>
+      </x:c>
+      <x:c r="D8" s="157" t="n">
+        <x:v>17.24</x:v>
+      </x:c>
+      <x:c r="E8" s="157" t="n">
+        <x:v>17.4</x:v>
+      </x:c>
+      <x:c r="F8" s="157" t="n">
+        <x:v>13.61</x:v>
+      </x:c>
+      <x:c r="G8" s="157" t="n">
+        <x:v>13.48</x:v>
+      </x:c>
+      <x:c r="H8" s="200" t="str">
+        <x:v>Stage 2</x:v>
+      </x:c>
+      <x:c r="I8" s="157" t="n">
+        <x:f>MIN(B8:E8)</x:f>
+        <x:v>16.93</x:v>
+      </x:c>
+      <x:c r="J8" s="158" t="n">
+        <x:f>B8/I8</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K8" s="158" t="n">
+        <x:f>F8/I8</x:f>
+        <x:v>0.8038984051978736</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="156" t="str">
+        <x:v>512 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B9" s="157" t="n">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="C9" s="157" t="n">
+        <x:v>53.94</x:v>
+      </x:c>
+      <x:c r="D9" s="157" t="n">
+        <x:v>89.33</x:v>
+      </x:c>
+      <x:c r="E9" s="157" t="n">
+        <x:v>90.07</x:v>
+      </x:c>
+      <x:c r="F9" s="157" t="n">
+        <x:v>50.06</x:v>
+      </x:c>
+      <x:c r="G9" s="157" t="n">
+        <x:v>50.26</x:v>
+      </x:c>
+      <x:c r="H9" s="200" t="str">
+        <x:v>Stage 3</x:v>
+      </x:c>
+      <x:c r="I9" s="157" t="n">
+        <x:f>MIN(B9:E9)</x:f>
+        <x:v>53.94</x:v>
+      </x:c>
+      <x:c r="J9" s="158" t="n">
+        <x:f>B9/I9</x:f>
+        <x:v>1.0011123470522802</x:v>
+      </x:c>
+      <x:c r="K9" s="158" t="n">
+        <x:f>F9/I9</x:f>
+        <x:v>0.92806822395254</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="156" t="str">
+        <x:v>512 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B10" s="157" t="n">
+        <x:v>31.35</x:v>
+      </x:c>
+      <x:c r="C10" s="157" t="n">
+        <x:v>30.97</x:v>
+      </x:c>
+      <x:c r="D10" s="157" t="n">
+        <x:v>31.1</x:v>
+      </x:c>
+      <x:c r="E10" s="157" t="n">
+        <x:v>31.12</x:v>
+      </x:c>
+      <x:c r="F10" s="157" t="n">
+        <x:v>24.75</x:v>
+      </x:c>
+      <x:c r="G10" s="157" t="n">
+        <x:v>24.71</x:v>
+      </x:c>
+      <x:c r="H10" s="200" t="str">
+        <x:v>Stage 3</x:v>
+      </x:c>
+      <x:c r="I10" s="157" t="n">
+        <x:f>MIN(B10:E10)</x:f>
+        <x:v>30.97</x:v>
+      </x:c>
+      <x:c r="J10" s="158" t="n">
+        <x:f>B10/I10</x:f>
+        <x:v>1.012269938650307</x:v>
+      </x:c>
+      <x:c r="K10" s="158" t="n">
+        <x:f>F10/I10</x:f>
+        <x:v>0.7991604778818211</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="156" t="str">
+        <x:v>1024 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B11" s="157" t="n">
+        <x:v>49.28</x:v>
+      </x:c>
+      <x:c r="C11" s="157" t="n">
+        <x:v>48.83</x:v>
+      </x:c>
+      <x:c r="D11" s="157" t="n">
+        <x:v>59.94</x:v>
+      </x:c>
+      <x:c r="E11" s="157" t="n">
+        <x:v>59.93</x:v>
+      </x:c>
+      <x:c r="F11" s="157" t="n">
+        <x:v>48.9</x:v>
+      </x:c>
+      <x:c r="G11" s="157" t="n">
+        <x:v>48.88</x:v>
+      </x:c>
+      <x:c r="H11" s="200" t="str">
+        <x:v>Stage 3</x:v>
+      </x:c>
+      <x:c r="I11" s="157" t="n">
+        <x:f>MIN(B11:E11)</x:f>
+        <x:v>48.83</x:v>
+      </x:c>
+      <x:c r="J11" s="158" t="n">
+        <x:f>B11/I11</x:f>
+        <x:v>1.009215646119189</x:v>
+      </x:c>
+      <x:c r="K11" s="158" t="n">
+        <x:f>F11/I11</x:f>
+        <x:v>1.0014335449518739</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="156" t="str">
+        <x:v>1024 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B12" s="157" t="n">
+        <x:v>49.69</x:v>
+      </x:c>
+      <x:c r="C12" s="157" t="n">
+        <x:v>49.45</x:v>
+      </x:c>
+      <x:c r="D12" s="157" t="n">
+        <x:v>57.51</x:v>
+      </x:c>
+      <x:c r="E12" s="157" t="n">
+        <x:v>57.86</x:v>
+      </x:c>
+      <x:c r="F12" s="157" t="n">
+        <x:v>47.22</x:v>
+      </x:c>
+      <x:c r="G12" s="157" t="n">
+        <x:v>46.4</x:v>
+      </x:c>
+      <x:c r="H12" s="200" t="str">
+        <x:v>Stage 3</x:v>
+      </x:c>
+      <x:c r="I12" s="157" t="n">
+        <x:f>MIN(B12:E12)</x:f>
+        <x:v>49.45</x:v>
+      </x:c>
+      <x:c r="J12" s="158" t="n">
+        <x:f>B12/I12</x:f>
+        <x:v>1.0048533872598584</x:v>
+      </x:c>
+      <x:c r="K12" s="158" t="n">
+        <x:f>F12/I12</x:f>
+        <x:v>0.9549039433771486</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="156" t="str">
+        <x:v>2048 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B13" s="157" t="n">
+        <x:v>91.94</x:v>
+      </x:c>
+      <x:c r="C13" s="157" t="n">
+        <x:v>90.03</x:v>
+      </x:c>
+      <x:c r="D13" s="157" t="n">
+        <x:v>117.48</x:v>
+      </x:c>
+      <x:c r="E13" s="157" t="n">
+        <x:v>117.81</x:v>
+      </x:c>
+      <x:c r="F13" s="157" t="n">
+        <x:v>94.76</x:v>
+      </x:c>
+      <x:c r="G13" s="157" t="n">
+        <x:v>94.25</x:v>
+      </x:c>
+      <x:c r="H13" s="200" t="str">
+        <x:v>Stage 3</x:v>
+      </x:c>
+      <x:c r="I13" s="157" t="n">
+        <x:f>MIN(B13:E13)</x:f>
+        <x:v>90.03</x:v>
+      </x:c>
+      <x:c r="J13" s="158" t="n">
+        <x:f>B13/I13</x:f>
+        <x:v>1.021215150505387</x:v>
+      </x:c>
+      <x:c r="K13" s="158" t="n">
+        <x:f>F13/I13</x:f>
+        <x:v>1.0525380428745974</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="156" t="str">
+        <x:v>2048 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B14" s="157" t="n">
+        <x:v>90.18</x:v>
+      </x:c>
+      <x:c r="C14" s="157" t="n">
+        <x:v>89.09</x:v>
+      </x:c>
+      <x:c r="D14" s="157" t="n">
+        <x:v>117.8</x:v>
+      </x:c>
+      <x:c r="E14" s="157" t="n">
+        <x:v>121.84</x:v>
+      </x:c>
+      <x:c r="F14" s="157" t="n">
+        <x:v>92.34</x:v>
+      </x:c>
+      <x:c r="G14" s="157" t="n">
+        <x:v>90.36</x:v>
+      </x:c>
+      <x:c r="H14" s="200" t="str">
+        <x:v>Stage 3</x:v>
+      </x:c>
+      <x:c r="I14" s="157" t="n">
+        <x:f>MIN(B14:E14)</x:f>
+        <x:v>89.09</x:v>
+      </x:c>
+      <x:c r="J14" s="158" t="n">
+        <x:f>B14/I14</x:f>
+        <x:v>1.01223481872264</x:v>
+      </x:c>
+      <x:c r="K14" s="158" t="n">
+        <x:f>F14/I14</x:f>
+        <x:v>1.036479964081266</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="156" t="str">
+        <x:v>4096 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B15" s="157" t="n">
+        <x:v>170.44</x:v>
+      </x:c>
+      <x:c r="C15" s="157" t="n">
+        <x:v>166.66</x:v>
+      </x:c>
+      <x:c r="D15" s="157" t="n">
+        <x:v>232.46</x:v>
+      </x:c>
+      <x:c r="E15" s="157" t="n">
+        <x:v>233.05</x:v>
+      </x:c>
+      <x:c r="F15" s="157" t="n">
+        <x:v>182.6</x:v>
+      </x:c>
+      <x:c r="G15" s="157" t="n">
+        <x:v>185.57</x:v>
+      </x:c>
+      <x:c r="H15" s="200" t="str">
+        <x:v>Stage 3</x:v>
+      </x:c>
+      <x:c r="I15" s="157" t="n">
+        <x:f>MIN(B15:E15)</x:f>
+        <x:v>166.66</x:v>
+      </x:c>
+      <x:c r="J15" s="158" t="n">
+        <x:f>B15/I15</x:f>
+        <x:v>1.0226809072362895</x:v>
+      </x:c>
+      <x:c r="K15" s="158" t="n">
+        <x:f>F15/I15</x:f>
+        <x:v>1.09564382575303</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="160" t="str">
+        <x:v>4096 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B16" s="161" t="n">
+        <x:v>167.74</x:v>
+      </x:c>
+      <x:c r="C16" s="161" t="n">
+        <x:v>163.84</x:v>
+      </x:c>
+      <x:c r="D16" s="161" t="n">
+        <x:v>249.41</x:v>
+      </x:c>
+      <x:c r="E16" s="161" t="n">
+        <x:v>250.5</x:v>
+      </x:c>
+      <x:c r="F16" s="161" t="n">
+        <x:v>182.18</x:v>
+      </x:c>
+      <x:c r="G16" s="161" t="n">
+        <x:v>175.72</x:v>
+      </x:c>
+      <x:c r="H16" s="201" t="str">
+        <x:v>Stage 3</x:v>
+      </x:c>
+      <x:c r="I16" s="161" t="n">
+        <x:f>MIN(B16:E16)</x:f>
+        <x:v>163.84</x:v>
+      </x:c>
+      <x:c r="J16" s="162" t="n">
+        <x:f>B16/I16</x:f>
+        <x:v>1.0238037109375</x:v>
+      </x:c>
+      <x:c r="K16" s="162" t="n">
+        <x:f>F16/I16</x:f>
+        <x:v>1.1119384765625</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="154"/>
+      <x:c r="B17" s="154"/>
+      <x:c r="C17" s="154"/>
+      <x:c r="D17" s="154"/>
+      <x:c r="E17" s="154"/>
+      <x:c r="F17" s="154"/>
+      <x:c r="G17" s="154"/>
+      <x:c r="H17" s="154"/>
+      <x:c r="I17" s="154"/>
+      <x:c r="J17" s="154"/>
+      <x:c r="K17" s="154"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="154"/>
+      <x:c r="B18" s="154"/>
+      <x:c r="C18" s="154"/>
+      <x:c r="D18" s="154"/>
+      <x:c r="E18" s="154"/>
+      <x:c r="F18" s="154"/>
+      <x:c r="G18" s="154"/>
+      <x:c r="H18" s="154"/>
+      <x:c r="I18" s="154"/>
+      <x:c r="J18" s="154"/>
+      <x:c r="K18" s="154"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="194" t="str">
+        <x:v>NCU: M=1024, N=1408, K=2048</x:v>
+      </x:c>
+      <x:c r="B19" s="194"/>
+      <x:c r="C19" s="194"/>
+      <x:c r="D19" s="194"/>
+      <x:c r="E19" s="194"/>
+      <x:c r="F19" s="194"/>
+      <x:c r="G19" s="194"/>
+      <x:c r="H19" s="194"/>
+      <x:c r="I19" s="194"/>
+      <x:c r="J19" s="194"/>
+      <x:c r="K19" s="194"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="195" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B20" s="195" t="str">
+        <x:v>Stage 2</x:v>
+      </x:c>
+      <x:c r="C20" s="195" t="str">
+        <x:v>Stage 3</x:v>
+      </x:c>
+      <x:c r="D20" s="195" t="str">
+        <x:v>Stage 4</x:v>
+      </x:c>
+      <x:c r="E20" s="195" t="str">
+        <x:v>Stage 5</x:v>
+      </x:c>
+      <x:c r="F20" s="195" t="str">
+        <x:v>Observation</x:v>
+      </x:c>
+      <x:c r="G20" s="195"/>
+      <x:c r="H20" s="195"/>
+      <x:c r="I20" s="195"/>
+      <x:c r="J20" s="195"/>
+      <x:c r="K20" s="195"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="156" t="str">
+        <x:v>NCU duration (us)</x:v>
+      </x:c>
+      <x:c r="B21" s="157" t="n">
+        <x:v>62.24</x:v>
+      </x:c>
+      <x:c r="C21" s="157" t="n">
+        <x:v>60.93</x:v>
+      </x:c>
+      <x:c r="D21" s="157" t="n">
+        <x:v>67.9</x:v>
+      </x:c>
+      <x:c r="E21" s="157" t="n">
+        <x:v>68.32</x:v>
+      </x:c>
+      <x:c r="F21" s="156" t="str">
+        <x:v>Stage 3 is 2.1% faster than Stage 2</x:v>
+      </x:c>
+      <x:c r="G21" s="156"/>
+      <x:c r="H21" s="156"/>
+      <x:c r="I21" s="156"/>
+      <x:c r="J21" s="156"/>
+      <x:c r="K21" s="156"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="156" t="str">
+        <x:v>SM busy (%)</x:v>
+      </x:c>
+      <x:c r="B22" s="157" t="n">
+        <x:v>68.91</x:v>
+      </x:c>
+      <x:c r="C22" s="157" t="n">
+        <x:v>71.13</x:v>
+      </x:c>
+      <x:c r="D22" s="157" t="n">
+        <x:v>65.56</x:v>
+      </x:c>
+      <x:c r="E22" s="157" t="n">
+        <x:v>66.38</x:v>
+      </x:c>
+      <x:c r="F22" s="156" t="str">
+        <x:v>Stage 3 has the highest SM activity</x:v>
+      </x:c>
+      <x:c r="G22" s="156"/>
+      <x:c r="H22" s="156"/>
+      <x:c r="I22" s="156"/>
+      <x:c r="J22" s="156"/>
+      <x:c r="K22" s="156"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="156" t="str">
+        <x:v>Memory throughput (% peak)</x:v>
+      </x:c>
+      <x:c r="B23" s="157" t="n">
+        <x:v>22.06</x:v>
+      </x:c>
+      <x:c r="C23" s="157" t="n">
+        <x:v>22.94</x:v>
+      </x:c>
+      <x:c r="D23" s="157" t="n">
+        <x:v>19.49</x:v>
+      </x:c>
+      <x:c r="E23" s="157" t="n">
+        <x:v>18.27</x:v>
+      </x:c>
+      <x:c r="F23" s="156" t="str">
+        <x:v>Deeper stages do not improve bandwidth use</x:v>
+      </x:c>
+      <x:c r="G23" s="156"/>
+      <x:c r="H23" s="156"/>
+      <x:c r="I23" s="156"/>
+      <x:c r="J23" s="156"/>
+      <x:c r="K23" s="156"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="156" t="str">
+        <x:v>DRAM throughput (% peak)</x:v>
+      </x:c>
+      <x:c r="B24" s="157" t="n">
+        <x:v>3.49</x:v>
+      </x:c>
+      <x:c r="C24" s="157" t="n">
+        <x:v>3.56</x:v>
+      </x:c>
+      <x:c r="D24" s="157" t="n">
+        <x:v>3.19</x:v>
+      </x:c>
+      <x:c r="E24" s="157" t="n">
+        <x:v>3.18</x:v>
+      </x:c>
+      <x:c r="F24" s="156" t="str">
+        <x:v>Kernel is not DRAM-bandwidth bound</x:v>
+      </x:c>
+      <x:c r="G24" s="156"/>
+      <x:c r="H24" s="156"/>
+      <x:c r="I24" s="156"/>
+      <x:c r="J24" s="156"/>
+      <x:c r="K24" s="156"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="156" t="str">
+        <x:v>Eligible warps / scheduler</x:v>
+      </x:c>
+      <x:c r="B25" s="157" t="n">
+        <x:v>0.28</x:v>
+      </x:c>
+      <x:c r="C25" s="157" t="n">
+        <x:v>0.29</x:v>
+      </x:c>
+      <x:c r="D25" s="157" t="n">
+        <x:v>0.24</x:v>
+      </x:c>
+      <x:c r="E25" s="157" t="n">
+        <x:v>0.24</x:v>
+      </x:c>
+      <x:c r="F25" s="156" t="str">
+        <x:v>Stage 4/5 expose less schedulable work</x:v>
+      </x:c>
+      <x:c r="G25" s="156"/>
+      <x:c r="H25" s="156"/>
+      <x:c r="I25" s="156"/>
+      <x:c r="J25" s="156"/>
+      <x:c r="K25" s="156"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="156" t="str">
+        <x:v>Warp cycles / issued instruction</x:v>
+      </x:c>
+      <x:c r="B26" s="157" t="n">
+        <x:v>24.13</x:v>
+      </x:c>
+      <x:c r="C26" s="157" t="n">
+        <x:v>23.76</x:v>
+      </x:c>
+      <x:c r="D26" s="157" t="n">
+        <x:v>19.62</x:v>
+      </x:c>
+      <x:c r="E26" s="157" t="n">
+        <x:v>19.69</x:v>
+      </x:c>
+      <x:c r="F26" s="156" t="str">
+        <x:v>Lower value does not offset reduced residency</x:v>
+      </x:c>
+      <x:c r="G26" s="156"/>
+      <x:c r="H26" s="156"/>
+      <x:c r="I26" s="156"/>
+      <x:c r="J26" s="156"/>
+      <x:c r="K26" s="156"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="156" t="str">
+        <x:v>Registers / thread</x:v>
+      </x:c>
+      <x:c r="B27" s="157" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C27" s="157" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="D27" s="157" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="E27" s="157" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F27" s="156" t="str">
+        <x:v>Register pressure is unchanged</x:v>
+      </x:c>
+      <x:c r="G27" s="156"/>
+      <x:c r="H27" s="156"/>
+      <x:c r="I27" s="156"/>
+      <x:c r="J27" s="156"/>
+      <x:c r="K27" s="156"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="156" t="str">
+        <x:v>Dynamic shared memory (KB/CTA)</x:v>
+      </x:c>
+      <x:c r="B28" s="157" t="n">
+        <x:v>50.18</x:v>
+      </x:c>
+      <x:c r="C28" s="157" t="n">
+        <x:v>66.56</x:v>
+      </x:c>
+      <x:c r="D28" s="157" t="n">
+        <x:v>82.94</x:v>
+      </x:c>
+      <x:c r="E28" s="157" t="n">
+        <x:v>99.33</x:v>
+      </x:c>
+      <x:c r="F28" s="156" t="str">
+        <x:v>Each extra stage costs about 16 KB</x:v>
+      </x:c>
+      <x:c r="G28" s="156"/>
+      <x:c r="H28" s="156"/>
+      <x:c r="I28" s="156"/>
+      <x:c r="J28" s="156"/>
+      <x:c r="K28" s="156"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="156" t="str">
+        <x:v>Shared-memory block limit</x:v>
+      </x:c>
+      <x:c r="B29" s="157" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C29" s="157" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D29" s="157" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E29" s="157" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F29" s="156" t="str">
+        <x:v>Stage 4 crosses the 2 CTA/SM threshold</x:v>
+      </x:c>
+      <x:c r="G29" s="156"/>
+      <x:c r="H29" s="156"/>
+      <x:c r="I29" s="156"/>
+      <x:c r="J29" s="156"/>
+      <x:c r="K29" s="156"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="156" t="str">
+        <x:v>Theoretical occupancy (%)</x:v>
+      </x:c>
+      <x:c r="B30" s="157" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C30" s="157" t="n">
+        <x:v>37.5</x:v>
+      </x:c>
+      <x:c r="D30" s="157" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="E30" s="157" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F30" s="156" t="str">
+        <x:v>Pipeline depth reduces CTA residency</x:v>
+      </x:c>
+      <x:c r="G30" s="156"/>
+      <x:c r="H30" s="156"/>
+      <x:c r="I30" s="156"/>
+      <x:c r="J30" s="156"/>
+      <x:c r="K30" s="156"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="156" t="str">
+        <x:v>Achieved occupancy (%)</x:v>
+      </x:c>
+      <x:c r="B31" s="157" t="n">
+        <x:v>30.93</x:v>
+      </x:c>
+      <x:c r="C31" s="157" t="n">
+        <x:v>31.31</x:v>
+      </x:c>
+      <x:c r="D31" s="157" t="n">
+        <x:v>24.16</x:v>
+      </x:c>
+      <x:c r="E31" s="157" t="n">
+        <x:v>24.41</x:v>
+      </x:c>
+      <x:c r="F31" s="156" t="str">
+        <x:v>Stage 3 preserves measured occupancy</x:v>
+      </x:c>
+      <x:c r="G31" s="156"/>
+      <x:c r="H31" s="156"/>
+      <x:c r="I31" s="156"/>
+      <x:c r="J31" s="156"/>
+      <x:c r="K31" s="156"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="160" t="str">
+        <x:v>CTA barrier stall (%)</x:v>
+      </x:c>
+      <x:c r="B32" s="161" t="n">
+        <x:v>67.1</x:v>
+      </x:c>
+      <x:c r="C32" s="161" t="n">
+        <x:v>67.7</x:v>
+      </x:c>
+      <x:c r="D32" s="161" t="n">
+        <x:v>66.1</x:v>
+      </x:c>
+      <x:c r="E32" s="161" t="n">
+        <x:v>67.5</x:v>
+      </x:c>
+      <x:c r="F32" s="160" t="str">
+        <x:v>More stages do not remove the main stall</x:v>
+      </x:c>
+      <x:c r="G32" s="160"/>
+      <x:c r="H32" s="160"/>
+      <x:c r="I32" s="160"/>
+      <x:c r="J32" s="160"/>
+      <x:c r="K32" s="160"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="154"/>
+      <x:c r="B33" s="154"/>
+      <x:c r="C33" s="154"/>
+      <x:c r="D33" s="154"/>
+      <x:c r="E33" s="154"/>
+      <x:c r="F33" s="154"/>
+      <x:c r="G33" s="154"/>
+      <x:c r="H33" s="154"/>
+      <x:c r="I33" s="154"/>
+      <x:c r="J33" s="154"/>
+      <x:c r="K33" s="154"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="154"/>
+      <x:c r="B34" s="154"/>
+      <x:c r="C34" s="154"/>
+      <x:c r="D34" s="154"/>
+      <x:c r="E34" s="154"/>
+      <x:c r="F34" s="154"/>
+      <x:c r="G34" s="154"/>
+      <x:c r="H34" s="154"/>
+      <x:c r="I34" s="154"/>
+      <x:c r="J34" s="154"/>
+      <x:c r="K34" s="154"/>
+    </x:row>
+    <x:row r="35" ht="42" customHeight="1">
+      <x:c r="A35" s="204" t="str">
+        <x:v>Decision: select Stage 3 for the 64 x 64 weight-block kernel. It gives the best fixed-shape NCU latency while retaining 3 CTA/SM; Stage 4 and Stage 5 reduce theoretical occupancy to 25% and regress medium-to-large M latency.</x:v>
+      </x:c>
+      <x:c r="B35" s="204"/>
+      <x:c r="C35" s="204"/>
+      <x:c r="D35" s="204"/>
+      <x:c r="E35" s="204"/>
+      <x:c r="F35" s="204"/>
+      <x:c r="G35" s="204"/>
+      <x:c r="H35" s="204"/>
+      <x:c r="I35" s="204"/>
+      <x:c r="J35" s="204"/>
+      <x:c r="K35" s="204"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:K1"/>
+    <x:mergeCell ref="A2:K2"/>
+    <x:mergeCell ref="A19:K19"/>
+    <x:mergeCell ref="F20:K20"/>
+    <x:mergeCell ref="F21:K21"/>
+    <x:mergeCell ref="F22:K22"/>
+    <x:mergeCell ref="F23:K23"/>
+    <x:mergeCell ref="F24:K24"/>
+    <x:mergeCell ref="F25:K25"/>
+    <x:mergeCell ref="F26:K26"/>
+    <x:mergeCell ref="F27:K27"/>
+    <x:mergeCell ref="F28:K28"/>
+    <x:mergeCell ref="F29:K29"/>
+    <x:mergeCell ref="F30:K30"/>
+    <x:mergeCell ref="F31:K31"/>
+    <x:mergeCell ref="F32:K32"/>
+    <x:mergeCell ref="A35:K35"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="J5:K16">
+    <x:cfRule type="colorScale" priority="1">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF8B4B4"/>
+        <x:color rgb="FFFEF3C7"/>
+        <x:color rgb="FFB7EFC5"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record warpgroup register experiment
Record paired NCU results showing no stable benefit from the 40/128 producer/math register budget. Also make the benchmark robust when NCU filters one timed kernel.
</commit_message>
<xml_diff>
--- a/docs/hybrid_sparse_performance.xlsx
+++ b/docs/hybrid_sparse_performance.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="Re9730e67123e4611"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R5fbaa80d48ed430a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="Rb1608c13041242d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="R79160dfc86dc4aad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="R257808f6a9f44a41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="R0aecc7acd3c74a17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="Rf48d9f1c90634b3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R193aa380385248e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R00b71e88d1c140b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R6c28e023c8034566"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="Rd91ccc9a312944f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="Rfc5d74d2a786404b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="Rc3f76944c8ed4641"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="Rfa970d1d0fdc4f16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register Realloc" sheetId="8" r:id="R378ef51881e940c8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -30,7 +31,7 @@
     <x:numFmt numFmtId="207" formatCode="0.0%"/>
     <x:numFmt numFmtId="208" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="22">
+  <x:fonts count="23">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -154,8 +155,13 @@
       <x:color rgb="FF166534"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF9A3412"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="29">
+  <x:fills count="34">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -295,6 +301,31 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF1F5F9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1D3265"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD8ECF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF294F7A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF1F5F9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7ED"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -462,7 +493,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="205">
+  <x:cellXfs count="230">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -882,6 +913,57 @@
     <x:xf numFmtId="0" fontId="17" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="20" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="20" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="31" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="17" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -4981,4 +5063,421 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="36" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="208" t="str">
+        <x:v>Warpgroup Register Reallocation</x:v>
+      </x:c>
+      <x:c r="B1" s="208"/>
+      <x:c r="C1" s="208"/>
+      <x:c r="D1" s="208"/>
+      <x:c r="E1" s="208"/>
+      <x:c r="F1" s="208"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="211" t="str">
+        <x:v>NVIDIA H20 | M=1024, N=1408, K=2048 | 64 x 64 weight block | Stage 3 TMA | producer=40 registers | math=128 registers</x:v>
+      </x:c>
+      <x:c r="B2" s="211"/>
+      <x:c r="C2" s="211"/>
+      <x:c r="D2" s="211"/>
+      <x:c r="E2" s="211"/>
+      <x:c r="F2" s="211"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="154"/>
+      <x:c r="B3" s="154"/>
+      <x:c r="C3" s="154"/>
+      <x:c r="D3" s="154"/>
+      <x:c r="E3" s="154"/>
+      <x:c r="F3" s="154"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="218" t="str">
+        <x:v>Summary</x:v>
+      </x:c>
+      <x:c r="B4" s="218" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="C4" s="154"/>
+      <x:c r="D4" s="154"/>
+      <x:c r="E4" s="154"/>
+      <x:c r="F4" s="154"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="156" t="str">
+        <x:v>Stage 3 mean NCU duration (us)</x:v>
+      </x:c>
+      <x:c r="B5" s="157" t="n">
+        <x:f>AVERAGE(B13,D13)</x:f>
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="C5" s="154"/>
+      <x:c r="D5" s="154"/>
+      <x:c r="E5" s="154"/>
+      <x:c r="F5" s="154"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="156" t="str">
+        <x:v>Register-reallocation mean (us)</x:v>
+      </x:c>
+      <x:c r="B6" s="157" t="n">
+        <x:f>AVERAGE(C13,E13)</x:f>
+        <x:v>61.985</x:v>
+      </x:c>
+      <x:c r="C6" s="154"/>
+      <x:c r="D6" s="154"/>
+      <x:c r="E6" s="154"/>
+      <x:c r="F6" s="154"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="156" t="str">
+        <x:v>Latency change</x:v>
+      </x:c>
+      <x:c r="B7" s="223" t="n">
+        <x:f>B6/B5-1</x:f>
+        <x:v>-0.00024193548387096975</x:v>
+      </x:c>
+      <x:c r="C7" s="154"/>
+      <x:c r="D7" s="154"/>
+      <x:c r="E7" s="154"/>
+      <x:c r="F7" s="154"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="160" t="str">
+        <x:v>Decision</x:v>
+      </x:c>
+      <x:c r="B8" s="160" t="str">
+        <x:v>Preserve implementation; do not select</x:v>
+      </x:c>
+      <x:c r="C8" s="154"/>
+      <x:c r="D8" s="154"/>
+      <x:c r="E8" s="154"/>
+      <x:c r="F8" s="154"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="154"/>
+      <x:c r="B9" s="154"/>
+      <x:c r="C9" s="154"/>
+      <x:c r="D9" s="154"/>
+      <x:c r="E9" s="154"/>
+      <x:c r="F9" s="154"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="154"/>
+      <x:c r="B10" s="154"/>
+      <x:c r="C10" s="154"/>
+      <x:c r="D10" s="154"/>
+      <x:c r="E10" s="154"/>
+      <x:c r="F10" s="154"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="217" t="str">
+        <x:v>Two Paired NCU Runs</x:v>
+      </x:c>
+      <x:c r="B11" s="217"/>
+      <x:c r="C11" s="217"/>
+      <x:c r="D11" s="217"/>
+      <x:c r="E11" s="217"/>
+      <x:c r="F11" s="217"/>
+    </x:row>
+    <x:row r="12" ht="36" customHeight="1">
+      <x:c r="A12" s="218" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B12" s="218" t="str">
+        <x:v>Stage 3 R1</x:v>
+      </x:c>
+      <x:c r="C12" s="218" t="str">
+        <x:v>Reg realloc R1</x:v>
+      </x:c>
+      <x:c r="D12" s="218" t="str">
+        <x:v>Stage 3 R2</x:v>
+      </x:c>
+      <x:c r="E12" s="218" t="str">
+        <x:v>Reg realloc R2</x:v>
+      </x:c>
+      <x:c r="F12" s="218" t="str">
+        <x:v>Observation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="156" t="str">
+        <x:v>Duration (us)</x:v>
+      </x:c>
+      <x:c r="B13" s="157" t="n">
+        <x:v>62.27</x:v>
+      </x:c>
+      <x:c r="C13" s="157" t="n">
+        <x:v>61.6</x:v>
+      </x:c>
+      <x:c r="D13" s="157" t="n">
+        <x:v>61.73</x:v>
+      </x:c>
+      <x:c r="E13" s="157" t="n">
+        <x:v>62.37</x:v>
+      </x:c>
+      <x:c r="F13" s="221" t="str">
+        <x:v>The direction reverses between runs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="156" t="str">
+        <x:v>SM busy (%)</x:v>
+      </x:c>
+      <x:c r="B14" s="157" t="n">
+        <x:v>70.19</x:v>
+      </x:c>
+      <x:c r="C14" s="157" t="n">
+        <x:v>68.62</x:v>
+      </x:c>
+      <x:c r="D14" s="157" t="n">
+        <x:v>70.71</x:v>
+      </x:c>
+      <x:c r="E14" s="157" t="n">
+        <x:v>69.17</x:v>
+      </x:c>
+      <x:c r="F14" s="221" t="str">
+        <x:v>Reallocation is consistently lower</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="156" t="str">
+        <x:v>Eligible warps / scheduler</x:v>
+      </x:c>
+      <x:c r="B15" s="157" t="n">
+        <x:v>0.29</x:v>
+      </x:c>
+      <x:c r="C15" s="157" t="n">
+        <x:v>0.29</x:v>
+      </x:c>
+      <x:c r="D15" s="157" t="n">
+        <x:v>0.29</x:v>
+      </x:c>
+      <x:c r="E15" s="157" t="n">
+        <x:v>0.29</x:v>
+      </x:c>
+      <x:c r="F15" s="221" t="str">
+        <x:v>No scheduler-level change</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="156" t="str">
+        <x:v>Warp cycles / issued instruction</x:v>
+      </x:c>
+      <x:c r="B16" s="157" t="n">
+        <x:v>23.76</x:v>
+      </x:c>
+      <x:c r="C16" s="157" t="n">
+        <x:v>24.43</x:v>
+      </x:c>
+      <x:c r="D16" s="157" t="n">
+        <x:v>23.89</x:v>
+      </x:c>
+      <x:c r="E16" s="157" t="n">
+        <x:v>24.37</x:v>
+      </x:c>
+      <x:c r="F16" s="221" t="str">
+        <x:v>Reallocation is slightly higher</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="156" t="str">
+        <x:v>Registers / thread</x:v>
+      </x:c>
+      <x:c r="B17" s="157" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C17" s="157" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="D17" s="157" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="E17" s="157" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F17" s="221" t="str">
+        <x:v>Math warpgroup does not use the larger budget</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="156" t="str">
+        <x:v>Dynamic shared memory (KB/CTA)</x:v>
+      </x:c>
+      <x:c r="B18" s="157" t="n">
+        <x:v>66.56</x:v>
+      </x:c>
+      <x:c r="C18" s="157" t="n">
+        <x:v>66.56</x:v>
+      </x:c>
+      <x:c r="D18" s="157" t="n">
+        <x:v>66.56</x:v>
+      </x:c>
+      <x:c r="E18" s="157" t="n">
+        <x:v>66.56</x:v>
+      </x:c>
+      <x:c r="F18" s="221" t="str">
+        <x:v>Unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="156" t="str">
+        <x:v>Theoretical occupancy (%)</x:v>
+      </x:c>
+      <x:c r="B19" s="157" t="n">
+        <x:v>37.5</x:v>
+      </x:c>
+      <x:c r="C19" s="157" t="n">
+        <x:v>37.5</x:v>
+      </x:c>
+      <x:c r="D19" s="157" t="n">
+        <x:v>37.5</x:v>
+      </x:c>
+      <x:c r="E19" s="157" t="n">
+        <x:v>37.5</x:v>
+      </x:c>
+      <x:c r="F19" s="221" t="str">
+        <x:v>Still limited to 3 CTA/SM by shared memory</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="156" t="str">
+        <x:v>Achieved occupancy (%)</x:v>
+      </x:c>
+      <x:c r="B20" s="157" t="n">
+        <x:v>31.23</x:v>
+      </x:c>
+      <x:c r="C20" s="157" t="n">
+        <x:v>31.34</x:v>
+      </x:c>
+      <x:c r="D20" s="157" t="n">
+        <x:v>31.37</x:v>
+      </x:c>
+      <x:c r="E20" s="157" t="n">
+        <x:v>31.34</x:v>
+      </x:c>
+      <x:c r="F20" s="221" t="str">
+        <x:v>Effectively unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="156" t="str">
+        <x:v>CTA barrier stall (%)</x:v>
+      </x:c>
+      <x:c r="B21" s="157" t="n">
+        <x:v>68.4</x:v>
+      </x:c>
+      <x:c r="C21" s="157" t="n">
+        <x:v>68.1</x:v>
+      </x:c>
+      <x:c r="D21" s="157" t="n">
+        <x:v>67.9</x:v>
+      </x:c>
+      <x:c r="E21" s="157" t="n">
+        <x:v>67.3</x:v>
+      </x:c>
+      <x:c r="F21" s="221" t="str">
+        <x:v>Main bottleneck remains</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="160" t="str">
+        <x:v>Local-memory spilling requests</x:v>
+      </x:c>
+      <x:c r="B22" s="161" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C22" s="161" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D22" s="161" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E22" s="161" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F22" s="222" t="str">
+        <x:v>No producer spill</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="154"/>
+      <x:c r="B23" s="154"/>
+      <x:c r="C23" s="154"/>
+      <x:c r="D23" s="154"/>
+      <x:c r="E23" s="154"/>
+      <x:c r="F23" s="154"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="154"/>
+      <x:c r="B24" s="154"/>
+      <x:c r="C24" s="154"/>
+      <x:c r="D24" s="154"/>
+      <x:c r="E24" s="154"/>
+      <x:c r="F24" s="154"/>
+    </x:row>
+    <x:row r="25" ht="52" customHeight="1">
+      <x:c r="A25" s="226" t="str">
+        <x:v>Decision: the setmaxnreg instructions are correct and do not introduce spills, but the kernel still compiles to 60 registers/thread. The two-run mean changes by less than 0.1%, so the implementation is retained for future larger-accumulator tiles and is not selected for the current 64 x 64 kernel.</x:v>
+      </x:c>
+      <x:c r="B25" s="226"/>
+      <x:c r="C25" s="226"/>
+      <x:c r="D25" s="226"/>
+      <x:c r="E25" s="226"/>
+      <x:c r="F25" s="226"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="154"/>
+      <x:c r="B26" s="154"/>
+      <x:c r="C26" s="154"/>
+      <x:c r="D26" s="154"/>
+      <x:c r="E26" s="154"/>
+      <x:c r="F26" s="154"/>
+    </x:row>
+    <x:row r="27" ht="42" customHeight="1">
+      <x:c r="A27" s="229" t="str">
+        <x:v>Environment note: a separate process occupied about 4.5 GiB of GPU memory during the Kineto sweep and produced bimodal timings; those sweep numbers are archived as raw logs but excluded from the decision.</x:v>
+      </x:c>
+      <x:c r="B27" s="229"/>
+      <x:c r="C27" s="229"/>
+      <x:c r="D27" s="229"/>
+      <x:c r="E27" s="229"/>
+      <x:c r="F27" s="229"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
+    <x:mergeCell ref="A11:F11"/>
+    <x:mergeCell ref="A25:F25"/>
+    <x:mergeCell ref="A27:F27"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="B7:B7">
+    <x:cfRule type="colorScale" priority="1">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFB7EFC5"/>
+        <x:color rgb="FFFEF3C7"/>
+        <x:color rgb="FFF8B4B4"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record metadata optimization results
Add the NCU and paired benchmark comparison for direct, TMA-staged, and producer-copied metadata paths. Mark completed experiments and the current best candidate in the checklist.
</commit_message>
<xml_diff>
--- a/docs/hybrid_sparse_performance.xlsx
+++ b/docs/hybrid_sparse_performance.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R193aa380385248e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R00b71e88d1c140b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R6c28e023c8034566"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="Rd91ccc9a312944f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="Rfc5d74d2a786404b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="Rc3f76944c8ed4641"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="Rfa970d1d0fdc4f16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register Realloc" sheetId="8" r:id="R378ef51881e940c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R9b0e80d92f4e4d0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R1d42ea3110df42ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="Ra905d591c1cd48fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="R17e5c44162e14fbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="R5fc14d8f10294afb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="R9bd090c8ca774a28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="Re135756942a3493a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register Realloc" sheetId="8" r:id="R2d0d094837204869"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Iterations" sheetId="9" r:id="R2f405c9c674c42d3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="9">
+  <x:numFmts count="10">
     <x:numFmt numFmtId="200" formatCode="0.00"/>
     <x:numFmt numFmtId="201" formatCode="0.000x"/>
     <x:numFmt numFmtId="202" formatCode="0%"/>
@@ -30,8 +31,9 @@
     <x:numFmt numFmtId="206" formatCode="0.000"/>
     <x:numFmt numFmtId="207" formatCode="0.0%"/>
     <x:numFmt numFmtId="208" formatCode="#,##0"/>
+    <x:numFmt numFmtId="209" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="23">
+  <x:fonts count="34">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -160,8 +162,72 @@
       <x:color rgb="FF9A3412"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF155B7A"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="13"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="9"/>
+      <x:color rgb="FF52657A"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF24456E"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF176B35"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="18"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF155B7A"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF24456E"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF176B35"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="13"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="9"/>
+      <x:color rgb="FF52657A"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="34">
+  <x:fills count="38">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -328,8 +394,28 @@
         <x:fgColor rgb="FFFFF7ED"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1B2B5B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEEF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF24456E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F8FC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="20">
+  <x:borders count="29">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -489,11 +575,101 @@
         <x:color rgb="FFA8B7C7"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="230">
+  <x:cellXfs count="337">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -966,11 +1142,284 @@
     <x:xf numFmtId="0" fontId="22" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="24" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="25" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="25" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="26" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="26" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="26" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="26" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="26" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="27" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="27" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="27" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="27" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="27" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="30" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="30" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="30" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="30" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="30" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="30" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="30" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="17" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="17" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="17" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="17" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="17" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="31" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="31" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="31" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="31" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="31" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="17" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="17" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="17" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="17" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="17" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="33" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="1">
+  <x:dxfs count="3">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -979,6 +1428,27 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF176B35"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFD8F3DF"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A2323"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFAD4D4"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -5480,4 +5950,803 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="17" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="300" t="str">
+        <x:v>Hybrid Sparse Metadata Optimization</x:v>
+      </x:c>
+      <x:c r="B1" s="300"/>
+      <x:c r="C1" s="300"/>
+      <x:c r="D1" s="300"/>
+      <x:c r="E1" s="300"/>
+      <x:c r="F1" s="300"/>
+      <x:c r="G1" s="300"/>
+      <x:c r="H1" s="300"/>
+      <x:c r="I1" s="300"/>
+      <x:c r="J1" s="300"/>
+      <x:c r="K1" s="300"/>
+      <x:c r="L1" s="300"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="301" t="str">
+        <x:v>NVIDIA H20 | M x N x K = 1024 x 1408 x 2048 | NCU --set full | BF16 input/output | FP32 accumulation</x:v>
+      </x:c>
+      <x:c r="B2" s="301"/>
+      <x:c r="C2" s="301"/>
+      <x:c r="D2" s="301"/>
+      <x:c r="E2" s="301"/>
+      <x:c r="F2" s="301"/>
+      <x:c r="G2" s="301"/>
+      <x:c r="H2" s="301"/>
+      <x:c r="I2" s="301"/>
+      <x:c r="J2" s="301"/>
+      <x:c r="K2" s="301"/>
+      <x:c r="L2" s="301"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="154"/>
+      <x:c r="B3" s="154"/>
+      <x:c r="C3" s="154"/>
+      <x:c r="D3" s="154"/>
+      <x:c r="E3" s="154"/>
+      <x:c r="F3" s="154"/>
+      <x:c r="G3" s="154"/>
+      <x:c r="H3" s="154"/>
+      <x:c r="I3" s="154"/>
+      <x:c r="J3" s="154"/>
+      <x:c r="K3" s="154"/>
+      <x:c r="L3" s="154"/>
+    </x:row>
+    <x:row r="4" ht="32" customHeight="1">
+      <x:c r="A4" s="302" t="str">
+        <x:v>Version</x:v>
+      </x:c>
+      <x:c r="B4" s="302" t="str">
+        <x:v>Metadata path</x:v>
+      </x:c>
+      <x:c r="C4" s="302" t="str">
+        <x:v>Epilogue overlap</x:v>
+      </x:c>
+      <x:c r="D4" s="302" t="str">
+        <x:v>NCU latency (us)</x:v>
+      </x:c>
+      <x:c r="E4" s="302" t="str">
+        <x:v>Speedup vs Stage 3</x:v>
+      </x:c>
+      <x:c r="F4" s="302" t="str">
+        <x:v>Barrier stall</x:v>
+      </x:c>
+      <x:c r="G4" s="302" t="str">
+        <x:v>Long scoreboard</x:v>
+      </x:c>
+      <x:c r="H4" s="302" t="str">
+        <x:v>Eligible warps</x:v>
+      </x:c>
+      <x:c r="I4" s="302" t="str">
+        <x:v>Executed instructions</x:v>
+      </x:c>
+      <x:c r="J4" s="302" t="str">
+        <x:v>Registers / thread</x:v>
+      </x:c>
+      <x:c r="K4" s="302" t="str">
+        <x:v>Dynamic smem (KB)</x:v>
+      </x:c>
+      <x:c r="L4" s="302" t="str">
+        <x:v>Tensor pipe active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="303" t="str">
+        <x:v>Stage 3</x:v>
+      </x:c>
+      <x:c r="B5" s="304" t="str">
+        <x:v>Block-row shared staging</x:v>
+      </x:c>
+      <x:c r="C5" s="304" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D5" s="305" t="n">
+        <x:v>61.6</x:v>
+      </x:c>
+      <x:c r="E5" s="306" t="n">
+        <x:f>$D$5/D5</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F5" s="305" t="n">
+        <x:v>16.094</x:v>
+      </x:c>
+      <x:c r="G5" s="305" t="n">
+        <x:v>1.693</x:v>
+      </x:c>
+      <x:c r="H5" s="305" t="n">
+        <x:v>0.29</x:v>
+      </x:c>
+      <x:c r="I5" s="307" t="n">
+        <x:v>5099990</x:v>
+      </x:c>
+      <x:c r="J5" s="308" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="K5" s="305" t="n">
+        <x:v>66.56</x:v>
+      </x:c>
+      <x:c r="L5" s="309" t="n">
+        <x:v>0.15278</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="310" t="str">
+        <x:v>Direct metadata</x:v>
+      </x:c>
+      <x:c r="B6" s="311" t="str">
+        <x:v>Math warp global load</x:v>
+      </x:c>
+      <x:c r="C6" s="311" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D6" s="312" t="n">
+        <x:v>61.44</x:v>
+      </x:c>
+      <x:c r="E6" s="313" t="n">
+        <x:f>$D$5/D6</x:f>
+        <x:v>1.0026041666666667</x:v>
+      </x:c>
+      <x:c r="F6" s="312" t="n">
+        <x:v>16.053</x:v>
+      </x:c>
+      <x:c r="G6" s="312" t="n">
+        <x:v>2.879</x:v>
+      </x:c>
+      <x:c r="H6" s="312" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="I6" s="314" t="n">
+        <x:v>4981946</x:v>
+      </x:c>
+      <x:c r="J6" s="315" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="K6" s="312" t="n">
+        <x:v>58.368</x:v>
+      </x:c>
+      <x:c r="L6" s="316" t="n">
+        <x:v>0.14541</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="310" t="str">
+        <x:v>Epilogue overlap</x:v>
+      </x:c>
+      <x:c r="B7" s="311" t="str">
+        <x:v>Math warp global load</x:v>
+      </x:c>
+      <x:c r="C7" s="311" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D7" s="312" t="n">
+        <x:v>61.28</x:v>
+      </x:c>
+      <x:c r="E7" s="313" t="n">
+        <x:f>$D$5/D7</x:f>
+        <x:v>1.0052219321148825</x:v>
+      </x:c>
+      <x:c r="F7" s="312" t="n">
+        <x:v>7.033</x:v>
+      </x:c>
+      <x:c r="G7" s="312" t="n">
+        <x:v>3.768</x:v>
+      </x:c>
+      <x:c r="H7" s="312" t="n">
+        <x:v>0.247</x:v>
+      </x:c>
+      <x:c r="I7" s="314" t="n">
+        <x:v>4917475</x:v>
+      </x:c>
+      <x:c r="J7" s="315" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="K7" s="312" t="n">
+        <x:v>58.368</x:v>
+      </x:c>
+      <x:c r="L7" s="316" t="n">
+        <x:v>0.1461</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="310" t="str">
+        <x:v>Register prefetch</x:v>
+      </x:c>
+      <x:c r="B8" s="311" t="str">
+        <x:v>Math warp register prefetch</x:v>
+      </x:c>
+      <x:c r="C8" s="311" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D8" s="312" t="n">
+        <x:v>61.632</x:v>
+      </x:c>
+      <x:c r="E8" s="313" t="n">
+        <x:f>$D$5/D8</x:f>
+        <x:v>0.9994807892004154</x:v>
+      </x:c>
+      <x:c r="F8" s="312" t="n">
+        <x:v>6.743</x:v>
+      </x:c>
+      <x:c r="G8" s="312" t="n">
+        <x:v>3.598</x:v>
+      </x:c>
+      <x:c r="H8" s="312" t="n">
+        <x:v>0.259</x:v>
+      </x:c>
+      <x:c r="I8" s="314" t="n">
+        <x:v>5189006</x:v>
+      </x:c>
+      <x:c r="J8" s="315" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="K8" s="312" t="n">
+        <x:v>58.368</x:v>
+      </x:c>
+      <x:c r="L8" s="316" t="n">
+        <x:v>0.14645</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="310" t="str">
+        <x:v>Stage-local TMA</x:v>
+      </x:c>
+      <x:c r="B9" s="311" t="str">
+        <x:v>Extra 512 B TMA per sparse block</x:v>
+      </x:c>
+      <x:c r="C9" s="311" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D9" s="312" t="n">
+        <x:v>62.048</x:v>
+      </x:c>
+      <x:c r="E9" s="313" t="n">
+        <x:f>$D$5/D9</x:f>
+        <x:v>0.9927797833935018</x:v>
+      </x:c>
+      <x:c r="F9" s="312" t="n">
+        <x:v>8.171</x:v>
+      </x:c>
+      <x:c r="G9" s="312" t="n">
+        <x:v>2.362</x:v>
+      </x:c>
+      <x:c r="H9" s="312" t="n">
+        <x:v>0.271</x:v>
+      </x:c>
+      <x:c r="I9" s="314" t="n">
+        <x:v>4762508</x:v>
+      </x:c>
+      <x:c r="J9" s="315" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="K9" s="312" t="n">
+        <x:v>59.392</x:v>
+      </x:c>
+      <x:c r="L9" s="316" t="n">
+        <x:v>0.15506</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="317" t="str">
+        <x:v>Producer warp copy</x:v>
+      </x:c>
+      <x:c r="B10" s="318" t="str">
+        <x:v>Coalesced 512 B vector copy</x:v>
+      </x:c>
+      <x:c r="C10" s="318" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D10" s="319" t="n">
+        <x:v>59.872</x:v>
+      </x:c>
+      <x:c r="E10" s="320" t="n">
+        <x:f>$D$5/D10</x:f>
+        <x:v>1.028861571352218</x:v>
+      </x:c>
+      <x:c r="F10" s="319" t="n">
+        <x:v>7.332</x:v>
+      </x:c>
+      <x:c r="G10" s="319" t="n">
+        <x:v>1.517</x:v>
+      </x:c>
+      <x:c r="H10" s="319" t="n">
+        <x:v>0.275</x:v>
+      </x:c>
+      <x:c r="I10" s="321" t="n">
+        <x:v>5204709</x:v>
+      </x:c>
+      <x:c r="J10" s="322" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="K10" s="319" t="n">
+        <x:v>59.392</x:v>
+      </x:c>
+      <x:c r="L10" s="323" t="n">
+        <x:v>0.15525</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="154"/>
+      <x:c r="B11" s="154"/>
+      <x:c r="C11" s="154"/>
+      <x:c r="D11" s="154"/>
+      <x:c r="E11" s="154"/>
+      <x:c r="F11" s="154"/>
+      <x:c r="G11" s="154"/>
+      <x:c r="H11" s="154"/>
+      <x:c r="I11" s="154"/>
+      <x:c r="J11" s="154"/>
+      <x:c r="K11" s="154"/>
+      <x:c r="L11" s="154"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="154"/>
+      <x:c r="B12" s="154"/>
+      <x:c r="C12" s="154"/>
+      <x:c r="D12" s="154"/>
+      <x:c r="E12" s="154"/>
+      <x:c r="F12" s="154"/>
+      <x:c r="G12" s="154"/>
+      <x:c r="H12" s="154"/>
+      <x:c r="I12" s="154"/>
+      <x:c r="J12" s="154"/>
+      <x:c r="K12" s="154"/>
+      <x:c r="L12" s="154"/>
+    </x:row>
+    <x:row r="13" ht="26" customHeight="1">
+      <x:c r="A13" s="324" t="str">
+        <x:v>Current Best: Producer-Warp Metadata Copy</x:v>
+      </x:c>
+      <x:c r="B13" s="324"/>
+      <x:c r="C13" s="324"/>
+      <x:c r="D13" s="324"/>
+      <x:c r="E13" s="324"/>
+      <x:c r="F13" s="154"/>
+      <x:c r="G13" s="154"/>
+      <x:c r="H13" s="154"/>
+      <x:c r="I13" s="154"/>
+      <x:c r="J13" s="154"/>
+      <x:c r="K13" s="154"/>
+      <x:c r="L13" s="154"/>
+    </x:row>
+    <x:row r="14" ht="32" customHeight="1">
+      <x:c r="A14" s="302" t="str">
+        <x:v>Shape (M x N x K)</x:v>
+      </x:c>
+      <x:c r="B14" s="302" t="str">
+        <x:v>Kernel latency (us)</x:v>
+      </x:c>
+      <x:c r="C14" s="302" t="str">
+        <x:v>DeepGEMM latency (us)</x:v>
+      </x:c>
+      <x:c r="D14" s="302" t="str">
+        <x:v>Speedup over DeepGEMM</x:v>
+      </x:c>
+      <x:c r="E14" s="302" t="str">
+        <x:v>Result</x:v>
+      </x:c>
+      <x:c r="F14" s="154"/>
+      <x:c r="G14" s="154"/>
+      <x:c r="H14" s="154"/>
+      <x:c r="I14" s="154"/>
+      <x:c r="J14" s="154"/>
+      <x:c r="K14" s="154"/>
+      <x:c r="L14" s="154"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="325" t="str">
+        <x:v>128 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B15" s="326" t="n">
+        <x:v>16.32</x:v>
+      </x:c>
+      <x:c r="C15" s="326" t="n">
+        <x:v>10.64</x:v>
+      </x:c>
+      <x:c r="D15" s="327" t="n">
+        <x:f>C15/B15</x:f>
+        <x:v>0.6519607843137255</x:v>
+      </x:c>
+      <x:c r="E15" s="328" t="str">
+        <x:f>IF(D15&gt;=1.25,"Target met",IF(D15&gt;=1,"Faster","Slower"))</x:f>
+        <x:v>Slower</x:v>
+      </x:c>
+      <x:c r="F15" s="154"/>
+      <x:c r="G15" s="154"/>
+      <x:c r="H15" s="154"/>
+      <x:c r="I15" s="154"/>
+      <x:c r="J15" s="154"/>
+      <x:c r="K15" s="154"/>
+      <x:c r="L15" s="154"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="329" t="str">
+        <x:v>128 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B16" s="330" t="n">
+        <x:v>11.61</x:v>
+      </x:c>
+      <x:c r="C16" s="330" t="n">
+        <x:v>9.18</x:v>
+      </x:c>
+      <x:c r="D16" s="313" t="n">
+        <x:f>C16/B16</x:f>
+        <x:v>0.7906976744186046</x:v>
+      </x:c>
+      <x:c r="E16" s="331" t="str">
+        <x:f>IF(D16&gt;=1.25,"Target met",IF(D16&gt;=1,"Faster","Slower"))</x:f>
+        <x:v>Slower</x:v>
+      </x:c>
+      <x:c r="F16" s="154"/>
+      <x:c r="G16" s="154"/>
+      <x:c r="H16" s="154"/>
+      <x:c r="I16" s="154"/>
+      <x:c r="J16" s="154"/>
+      <x:c r="K16" s="154"/>
+      <x:c r="L16" s="154"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="329" t="str">
+        <x:v>256 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B17" s="330" t="n">
+        <x:v>47.04</x:v>
+      </x:c>
+      <x:c r="C17" s="330" t="n">
+        <x:v>14.68</x:v>
+      </x:c>
+      <x:c r="D17" s="313" t="n">
+        <x:f>C17/B17</x:f>
+        <x:v>0.3120748299319728</x:v>
+      </x:c>
+      <x:c r="E17" s="331" t="str">
+        <x:f>IF(D17&gt;=1.25,"Target met",IF(D17&gt;=1,"Faster","Slower"))</x:f>
+        <x:v>Slower</x:v>
+      </x:c>
+      <x:c r="F17" s="154"/>
+      <x:c r="G17" s="154"/>
+      <x:c r="H17" s="154"/>
+      <x:c r="I17" s="154"/>
+      <x:c r="J17" s="154"/>
+      <x:c r="K17" s="154"/>
+      <x:c r="L17" s="154"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="329" t="str">
+        <x:v>256 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B18" s="330" t="n">
+        <x:v>16.45</x:v>
+      </x:c>
+      <x:c r="C18" s="330" t="n">
+        <x:v>13.97</x:v>
+      </x:c>
+      <x:c r="D18" s="313" t="n">
+        <x:f>C18/B18</x:f>
+        <x:v>0.8492401215805472</x:v>
+      </x:c>
+      <x:c r="E18" s="331" t="str">
+        <x:f>IF(D18&gt;=1.25,"Target met",IF(D18&gt;=1,"Faster","Slower"))</x:f>
+        <x:v>Slower</x:v>
+      </x:c>
+      <x:c r="F18" s="154"/>
+      <x:c r="G18" s="154"/>
+      <x:c r="H18" s="154"/>
+      <x:c r="I18" s="154"/>
+      <x:c r="J18" s="154"/>
+      <x:c r="K18" s="154"/>
+      <x:c r="L18" s="154"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="329" t="str">
+        <x:v>512 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B19" s="330" t="n">
+        <x:v>53.85</x:v>
+      </x:c>
+      <x:c r="C19" s="330" t="n">
+        <x:v>50.34</x:v>
+      </x:c>
+      <x:c r="D19" s="313" t="n">
+        <x:f>C19/B19</x:f>
+        <x:v>0.9348189415041783</x:v>
+      </x:c>
+      <x:c r="E19" s="331" t="str">
+        <x:f>IF(D19&gt;=1.25,"Target met",IF(D19&gt;=1,"Faster","Slower"))</x:f>
+        <x:v>Slower</x:v>
+      </x:c>
+      <x:c r="F19" s="154"/>
+      <x:c r="G19" s="154"/>
+      <x:c r="H19" s="154"/>
+      <x:c r="I19" s="154"/>
+      <x:c r="J19" s="154"/>
+      <x:c r="K19" s="154"/>
+      <x:c r="L19" s="154"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="329" t="str">
+        <x:v>512 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B20" s="330" t="n">
+        <x:v>55.67</x:v>
+      </x:c>
+      <x:c r="C20" s="330" t="n">
+        <x:v>27.27</x:v>
+      </x:c>
+      <x:c r="D20" s="313" t="n">
+        <x:f>C20/B20</x:f>
+        <x:v>0.48985090713130947</x:v>
+      </x:c>
+      <x:c r="E20" s="331" t="str">
+        <x:f>IF(D20&gt;=1.25,"Target met",IF(D20&gt;=1,"Faster","Slower"))</x:f>
+        <x:v>Slower</x:v>
+      </x:c>
+      <x:c r="F20" s="154"/>
+      <x:c r="G20" s="154"/>
+      <x:c r="H20" s="154"/>
+      <x:c r="I20" s="154"/>
+      <x:c r="J20" s="154"/>
+      <x:c r="K20" s="154"/>
+      <x:c r="L20" s="154"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="329" t="str">
+        <x:v>1024 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B21" s="330" t="n">
+        <x:v>97.34</x:v>
+      </x:c>
+      <x:c r="C21" s="330" t="n">
+        <x:v>98.38</x:v>
+      </x:c>
+      <x:c r="D21" s="313" t="n">
+        <x:f>C21/B21</x:f>
+        <x:v>1.0106841997123484</x:v>
+      </x:c>
+      <x:c r="E21" s="331" t="str">
+        <x:f>IF(D21&gt;=1.25,"Target met",IF(D21&gt;=1,"Faster","Slower"))</x:f>
+        <x:v>Faster</x:v>
+      </x:c>
+      <x:c r="F21" s="154"/>
+      <x:c r="G21" s="154"/>
+      <x:c r="H21" s="154"/>
+      <x:c r="I21" s="154"/>
+      <x:c r="J21" s="154"/>
+      <x:c r="K21" s="154"/>
+      <x:c r="L21" s="154"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="329" t="str">
+        <x:v>1024 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B22" s="330" t="n">
+        <x:v>97.09</x:v>
+      </x:c>
+      <x:c r="C22" s="330" t="n">
+        <x:v>97.88</x:v>
+      </x:c>
+      <x:c r="D22" s="313" t="n">
+        <x:f>C22/B22</x:f>
+        <x:v>1.0081367803069317</x:v>
+      </x:c>
+      <x:c r="E22" s="331" t="str">
+        <x:f>IF(D22&gt;=1.25,"Target met",IF(D22&gt;=1,"Faster","Slower"))</x:f>
+        <x:v>Faster</x:v>
+      </x:c>
+      <x:c r="F22" s="154"/>
+      <x:c r="G22" s="154"/>
+      <x:c r="H22" s="154"/>
+      <x:c r="I22" s="154"/>
+      <x:c r="J22" s="154"/>
+      <x:c r="K22" s="154"/>
+      <x:c r="L22" s="154"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="329" t="str">
+        <x:v>2048 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B23" s="330" t="n">
+        <x:v>164.67</x:v>
+      </x:c>
+      <x:c r="C23" s="330" t="n">
+        <x:v>194.35</x:v>
+      </x:c>
+      <x:c r="D23" s="313" t="n">
+        <x:f>C23/B23</x:f>
+        <x:v>1.1802392664116113</x:v>
+      </x:c>
+      <x:c r="E23" s="331" t="str">
+        <x:f>IF(D23&gt;=1.25,"Target met",IF(D23&gt;=1,"Faster","Slower"))</x:f>
+        <x:v>Faster</x:v>
+      </x:c>
+      <x:c r="F23" s="154"/>
+      <x:c r="G23" s="154"/>
+      <x:c r="H23" s="154"/>
+      <x:c r="I23" s="154"/>
+      <x:c r="J23" s="154"/>
+      <x:c r="K23" s="154"/>
+      <x:c r="L23" s="154"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="329" t="str">
+        <x:v>2048 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B24" s="330" t="n">
+        <x:v>148.14</x:v>
+      </x:c>
+      <x:c r="C24" s="330" t="n">
+        <x:v>93.4</x:v>
+      </x:c>
+      <x:c r="D24" s="313" t="n">
+        <x:f>C24/B24</x:f>
+        <x:v>0.6304846766572162</x:v>
+      </x:c>
+      <x:c r="E24" s="331" t="str">
+        <x:f>IF(D24&gt;=1.25,"Target met",IF(D24&gt;=1,"Faster","Slower"))</x:f>
+        <x:v>Slower</x:v>
+      </x:c>
+      <x:c r="F24" s="154"/>
+      <x:c r="G24" s="154"/>
+      <x:c r="H24" s="154"/>
+      <x:c r="I24" s="154"/>
+      <x:c r="J24" s="154"/>
+      <x:c r="K24" s="154"/>
+      <x:c r="L24" s="154"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="329" t="str">
+        <x:v>4096 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B25" s="330" t="n">
+        <x:v>169.82</x:v>
+      </x:c>
+      <x:c r="C25" s="330" t="n">
+        <x:v>184.31</x:v>
+      </x:c>
+      <x:c r="D25" s="313" t="n">
+        <x:f>C25/B25</x:f>
+        <x:v>1.085325638911789</x:v>
+      </x:c>
+      <x:c r="E25" s="331" t="str">
+        <x:f>IF(D25&gt;=1.25,"Target met",IF(D25&gt;=1,"Faster","Slower"))</x:f>
+        <x:v>Faster</x:v>
+      </x:c>
+      <x:c r="F25" s="154"/>
+      <x:c r="G25" s="154"/>
+      <x:c r="H25" s="154"/>
+      <x:c r="I25" s="154"/>
+      <x:c r="J25" s="154"/>
+      <x:c r="K25" s="154"/>
+      <x:c r="L25" s="154"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="332" t="str">
+        <x:v>4096 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B26" s="333" t="n">
+        <x:v>159.7</x:v>
+      </x:c>
+      <x:c r="C26" s="333" t="n">
+        <x:v>182.25</x:v>
+      </x:c>
+      <x:c r="D26" s="334" t="n">
+        <x:f>C26/B26</x:f>
+        <x:v>1.141202254226675</x:v>
+      </x:c>
+      <x:c r="E26" s="335" t="str">
+        <x:f>IF(D26&gt;=1.25,"Target met",IF(D26&gt;=1,"Faster","Slower"))</x:f>
+        <x:v>Faster</x:v>
+      </x:c>
+      <x:c r="F26" s="154"/>
+      <x:c r="G26" s="154"/>
+      <x:c r="H26" s="154"/>
+      <x:c r="I26" s="154"/>
+      <x:c r="J26" s="154"/>
+      <x:c r="K26" s="154"/>
+      <x:c r="L26" s="154"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="154"/>
+      <x:c r="B27" s="154"/>
+      <x:c r="C27" s="154"/>
+      <x:c r="D27" s="154"/>
+      <x:c r="E27" s="154"/>
+      <x:c r="F27" s="154"/>
+      <x:c r="G27" s="154"/>
+      <x:c r="H27" s="154"/>
+      <x:c r="I27" s="154"/>
+      <x:c r="J27" s="154"/>
+      <x:c r="K27" s="154"/>
+      <x:c r="L27" s="154"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="154"/>
+      <x:c r="B28" s="154"/>
+      <x:c r="C28" s="154"/>
+      <x:c r="D28" s="154"/>
+      <x:c r="E28" s="154"/>
+      <x:c r="F28" s="154"/>
+      <x:c r="G28" s="154"/>
+      <x:c r="H28" s="154"/>
+      <x:c r="I28" s="154"/>
+      <x:c r="J28" s="154"/>
+      <x:c r="K28" s="154"/>
+      <x:c r="L28" s="154"/>
+    </x:row>
+    <x:row r="29" ht="34" customHeight="1">
+      <x:c r="A29" s="336" t="str">
+        <x:v>Benchmark note: all eight GPUs had substantial external load. Use paired rows and NCU deltas for iteration decisions; the 1.25x DeepGEMM target is not yet verified.</x:v>
+      </x:c>
+      <x:c r="B29" s="336"/>
+      <x:c r="C29" s="336"/>
+      <x:c r="D29" s="336"/>
+      <x:c r="E29" s="336"/>
+      <x:c r="F29" s="336"/>
+      <x:c r="G29" s="336"/>
+      <x:c r="H29" s="336"/>
+      <x:c r="I29" s="336"/>
+      <x:c r="J29" s="336"/>
+      <x:c r="K29" s="336"/>
+      <x:c r="L29" s="336"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:L1"/>
+    <x:mergeCell ref="A2:L2"/>
+    <x:mergeCell ref="A13:E13"/>
+    <x:mergeCell ref="A29:L29"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="E5:E10">
+    <x:cfRule type="colorScale" priority="1">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF8C4C4"/>
+        <x:color rgb="FFFFF0BF"/>
+        <x:color rgb="FFB9EFCB"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="D15:D26">
+    <x:cfRule type="colorScale" priority="2">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF8C4C4"/>
+        <x:color rgb="FFFFF0BF"/>
+        <x:color rgb="FFB9EFCB"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="E15:E26">
+    <x:cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="Faster"/>
+    <x:cfRule type="containsText" dxfId="2" priority="4" operator="containsText" text="Slower"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record output-tile optimization
Document the 128x64 output-tile and staged block-kind iterations, including stable 1.25x-plus paired results and NCU deltas. The workbook was rendered and checked for formula errors.
</commit_message>
<xml_diff>
--- a/docs/hybrid_sparse_performance.xlsx
+++ b/docs/hybrid_sparse_performance.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R9b0e80d92f4e4d0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R1d42ea3110df42ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="Ra905d591c1cd48fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="R17e5c44162e14fbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="R5fc14d8f10294afb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="R9bd090c8ca774a28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="Re135756942a3493a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register Realloc" sheetId="8" r:id="R2d0d094837204869"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Iterations" sheetId="9" r:id="R2f405c9c674c42d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R2c2671842a2f4acb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="Rdf2687aedcad44b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R7eebe30c090b42b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="R73289d838cff4067"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="R63c59aef73b94102"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="Rdffd2fc2c695447d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="R802bad8d5dd24658"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register Realloc" sheetId="8" r:id="R007fce9f93794f65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Iterations" sheetId="9" r:id="Reb208ff8bc9b4b82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output Tile Reuse" sheetId="10" r:id="Rbb95db97bd31481c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -33,7 +34,7 @@
     <x:numFmt numFmtId="208" formatCode="#,##0"/>
     <x:numFmt numFmtId="209" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="34">
+  <x:fonts count="52">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -226,8 +227,107 @@
       <x:color rgb="FF52657A"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF236B86"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1D6B3C"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF4E5D6C"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="18"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF236B86"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1D6B3C"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF4E5D6C"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1D6B3C"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF4E5D6C"/>
+      <x:name val="Aptos"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="38">
+  <x:fills count="44">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -414,8 +514,38 @@
         <x:fgColor rgb="FFF5F8FC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F3265"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EEF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF294E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9F2E3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F6FA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="29">
+  <x:borders count="41">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -665,11 +795,119 @@
         <x:color rgb="FFD8E0EA"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:left>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD7DEE8"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="337">
+  <x:cellXfs count="532">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1413,6 +1651,453 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="33" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="34" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="34" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="40" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="40" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="40" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="40" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="40" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="40" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="40" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="40" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="40" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="40" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="40" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="40" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="35" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="41" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="41" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="41" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="36" fillId="41" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="36" fillId="41" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="36" fillId="41" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="42" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="42" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="42" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="43" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="43" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="43" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="43" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="43" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="37" fillId="43" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="37" fillId="43" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="37" fillId="43" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="36" fillId="41" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="42" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="43" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="36" fillId="41" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="42" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="43" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="208" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="36" fillId="41" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="36" fillId="41" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="42" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="42" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="43" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="43" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="40" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="40" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="40" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="41" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="42" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="43" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="37" fillId="43" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="37" fillId="43" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="37" fillId="43" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="40" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="42" fillId="40" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="42" fillId="40" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="42" fillId="40" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="41" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="41" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="41" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="41" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="43" fillId="41" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="43" fillId="41" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="43" fillId="41" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="43" fillId="41" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="41" fillId="42" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="41" fillId="42" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="41" fillId="42" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="42" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="41" fillId="43" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="41" fillId="43" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="41" fillId="43" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="43" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="42" fillId="40" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="42" fillId="40" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="41" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="41" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="41" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="41" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="41" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="41" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="41" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="45" fillId="43" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="45" fillId="43" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="45" fillId="43" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="46" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="46" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="47" fillId="40" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="40" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="40" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="48" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="48" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="48" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="48" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="49" fillId="41" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="49" fillId="41" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="49" fillId="41" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="49" fillId="41" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="42" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="48" fillId="42" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="48" fillId="42" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="42" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="43" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="48" fillId="43" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="48" fillId="43" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="43" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="40" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="40" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="48" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="48" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="48" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="48" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="48" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="48" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="48" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="50" fillId="43" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="50" fillId="43" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="50" fillId="43" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="51" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="51" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1437,7 +2122,7 @@
         <x:color rgb="FF176B35"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD8F3DF"/>
         </x:patternFill>
       </x:fill>
@@ -1447,7 +2132,7 @@
         <x:color rgb="FF8A2323"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFAD4D4"/>
         </x:patternFill>
       </x:fill>
@@ -1900,6 +2585,544 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="31" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="440" t="str">
+        <x:v>Hybrid Sparse Output-Tile Reuse</x:v>
+      </x:c>
+      <x:c r="B1" s="440"/>
+      <x:c r="C1" s="440"/>
+      <x:c r="D1" s="440"/>
+      <x:c r="E1" s="440"/>
+      <x:c r="F1" s="440"/>
+      <x:c r="G1" s="440"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="441" t="str">
+        <x:v>NVIDIA H20 | BF16 input/output | FP32 accumulation | M x N x K = 4096 x 2048 x 1408 | L2 flush disabled</x:v>
+      </x:c>
+      <x:c r="B2" s="441"/>
+      <x:c r="C2" s="441"/>
+      <x:c r="D2" s="441"/>
+      <x:c r="E2" s="441"/>
+      <x:c r="F2" s="441"/>
+      <x:c r="G2" s="441"/>
+    </x:row>
+    <x:row r="3" ht="20" customHeight="1">
+      <x:c r="A3" s="488"/>
+      <x:c r="B3" s="488"/>
+      <x:c r="C3" s="488"/>
+      <x:c r="D3" s="488"/>
+      <x:c r="E3" s="488"/>
+      <x:c r="F3" s="488"/>
+      <x:c r="G3" s="488"/>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="489" t="str">
+        <x:v>Version</x:v>
+      </x:c>
+      <x:c r="B4" s="490" t="str">
+        <x:v>Run 1 (us)</x:v>
+      </x:c>
+      <x:c r="C4" s="490" t="str">
+        <x:v>Run 2 (us)</x:v>
+      </x:c>
+      <x:c r="D4" s="490" t="str">
+        <x:v>Run 3 (us)</x:v>
+      </x:c>
+      <x:c r="E4" s="490" t="str">
+        <x:v>Average (us)</x:v>
+      </x:c>
+      <x:c r="F4" s="490" t="str">
+        <x:v>Paired speedup</x:v>
+      </x:c>
+      <x:c r="G4" s="491" t="str">
+        <x:v>Decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="20" customHeight="1">
+      <x:c r="A5" s="492" t="str">
+        <x:v>Producer copy 64x64</x:v>
+      </x:c>
+      <x:c r="B5" s="493" t="n">
+        <x:v>155.83</x:v>
+      </x:c>
+      <x:c r="C5" s="493" t="n">
+        <x:v>155.6</x:v>
+      </x:c>
+      <x:c r="D5" s="493" t="n">
+        <x:v>156.41</x:v>
+      </x:c>
+      <x:c r="E5" s="493" t="n">
+        <x:f>AVERAGE(B5:D5)</x:f>
+        <x:v>155.9466666666667</x:v>
+      </x:c>
+      <x:c r="F5" s="494" t="n">
+        <x:f>AVERAGE($B$9/B5,$C$9/C5,$D$9/D5)</x:f>
+        <x:v>1.1659354427141075</x:v>
+      </x:c>
+      <x:c r="G5" s="495" t="str">
+        <x:v>Baseline</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="20" customHeight="1">
+      <x:c r="A6" s="496" t="str">
+        <x:v>Output tile 128x64</x:v>
+      </x:c>
+      <x:c r="B6" s="497" t="n">
+        <x:v>145.63</x:v>
+      </x:c>
+      <x:c r="C6" s="497" t="n">
+        <x:v>153.28</x:v>
+      </x:c>
+      <x:c r="D6" s="497" t="n">
+        <x:v>145.94</x:v>
+      </x:c>
+      <x:c r="E6" s="497" t="n">
+        <x:f>AVERAGE(B6:D6)</x:f>
+        <x:v>148.28333333333333</x:v>
+      </x:c>
+      <x:c r="F6" s="498" t="n">
+        <x:f>AVERAGE($B$9/B6,$C$9/C6,$D$9/D6)</x:f>
+        <x:v>1.226884757589631</x:v>
+      </x:c>
+      <x:c r="G6" s="499" t="str">
+        <x:v>Retained</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="20" customHeight="1">
+      <x:c r="A7" s="500" t="str">
+        <x:v>Stage kind</x:v>
+      </x:c>
+      <x:c r="B7" s="501" t="n">
+        <x:v>144.07</x:v>
+      </x:c>
+      <x:c r="C7" s="501" t="n">
+        <x:v>144.4</x:v>
+      </x:c>
+      <x:c r="D7" s="501" t="n">
+        <x:v>144.33</x:v>
+      </x:c>
+      <x:c r="E7" s="501" t="n">
+        <x:f>AVERAGE(B7:D7)</x:f>
+        <x:v>144.26666666666668</x:v>
+      </x:c>
+      <x:c r="F7" s="502" t="n">
+        <x:f>AVERAGE($B$9/B7,$C$9/C7,$D$9/D7)</x:f>
+        <x:v>1.2603285021897923</x:v>
+      </x:c>
+      <x:c r="G7" s="503" t="str">
+        <x:v>Current best</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="20" customHeight="1">
+      <x:c r="A8" s="504" t="str">
+        <x:v>Stage selector</x:v>
+      </x:c>
+      <x:c r="B8" s="505" t="n">
+        <x:v>144.24</x:v>
+      </x:c>
+      <x:c r="C8" s="505" t="n">
+        <x:v>145.22</x:v>
+      </x:c>
+      <x:c r="D8" s="505" t="n">
+        <x:v>144.61</x:v>
+      </x:c>
+      <x:c r="E8" s="505" t="n">
+        <x:f>AVERAGE(B8:D8)</x:f>
+        <x:v>144.69000000000003</x:v>
+      </x:c>
+      <x:c r="F8" s="506" t="n">
+        <x:f>AVERAGE($B$9/B8,$C$9/C8,$D$9/D8)</x:f>
+        <x:v>1.256650106303988</x:v>
+      </x:c>
+      <x:c r="G8" s="507" t="str">
+        <x:v>Not adopted</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="20" customHeight="1">
+      <x:c r="A9" s="508" t="str">
+        <x:v>DeepGEMM</x:v>
+      </x:c>
+      <x:c r="B9" s="509" t="n">
+        <x:v>181.6</x:v>
+      </x:c>
+      <x:c r="C9" s="509" t="n">
+        <x:v>181.72</x:v>
+      </x:c>
+      <x:c r="D9" s="509" t="n">
+        <x:v>182.15</x:v>
+      </x:c>
+      <x:c r="E9" s="509" t="n">
+        <x:f>AVERAGE(B9:D9)</x:f>
+        <x:v>181.82333333333335</x:v>
+      </x:c>
+      <x:c r="F9" s="510" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G9" s="511" t="str">
+        <x:v>Dense baseline</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="20" customHeight="1">
+      <x:c r="A10" s="512"/>
+      <x:c r="B10" s="513"/>
+      <x:c r="C10" s="513"/>
+      <x:c r="D10" s="513"/>
+      <x:c r="E10" s="513"/>
+      <x:c r="F10" s="513"/>
+      <x:c r="G10" s="488"/>
+    </x:row>
+    <x:row r="11" ht="20" customHeight="1">
+      <x:c r="A11" s="512"/>
+      <x:c r="B11" s="513"/>
+      <x:c r="C11" s="513"/>
+      <x:c r="D11" s="513"/>
+      <x:c r="E11" s="513"/>
+      <x:c r="F11" s="513"/>
+      <x:c r="G11" s="488"/>
+    </x:row>
+    <x:row r="12" ht="20" customHeight="1">
+      <x:c r="A12" s="468" t="str">
+        <x:v>Paired NCU Comparison at 4096 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B12" s="469"/>
+      <x:c r="C12" s="469"/>
+      <x:c r="D12" s="469"/>
+      <x:c r="E12" s="469"/>
+      <x:c r="F12" s="513"/>
+      <x:c r="G12" s="488"/>
+    </x:row>
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="489" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B13" s="516" t="str">
+        <x:v>Output 128x64</x:v>
+      </x:c>
+      <x:c r="C13" s="516" t="str">
+        <x:v>Stage kind</x:v>
+      </x:c>
+      <x:c r="D13" s="516" t="str">
+        <x:v>DeepGEMM</x:v>
+      </x:c>
+      <x:c r="E13" s="517" t="str">
+        <x:v>Stage vs Output</x:v>
+      </x:c>
+      <x:c r="F13" s="513"/>
+      <x:c r="G13" s="488"/>
+    </x:row>
+    <x:row r="14" ht="20" customHeight="1">
+      <x:c r="A14" s="492" t="str">
+        <x:v>NCU duration (us)</x:v>
+      </x:c>
+      <x:c r="B14" s="518" t="n">
+        <x:v>171.168</x:v>
+      </x:c>
+      <x:c r="C14" s="518" t="n">
+        <x:v>160.832</x:v>
+      </x:c>
+      <x:c r="D14" s="518" t="n">
+        <x:v>201.504</x:v>
+      </x:c>
+      <x:c r="E14" s="519" t="n">
+        <x:f>C14/B14-1</x:f>
+        <x:v>-0.060385118713778385</x:v>
+      </x:c>
+      <x:c r="F14" s="513"/>
+      <x:c r="G14" s="488"/>
+    </x:row>
+    <x:row r="15" ht="20" customHeight="1">
+      <x:c r="A15" s="496" t="str">
+        <x:v>SM throughput (% peak)</x:v>
+      </x:c>
+      <x:c r="B15" s="520" t="n">
+        <x:v>79.016669</x:v>
+      </x:c>
+      <x:c r="C15" s="520" t="n">
+        <x:v>83.466808</x:v>
+      </x:c>
+      <x:c r="D15" s="520" t="n">
+        <x:v>92.852352</x:v>
+      </x:c>
+      <x:c r="E15" s="521" t="n">
+        <x:f>C15/B15-1</x:f>
+        <x:v>0.05631899011080832</x:v>
+      </x:c>
+      <x:c r="F15" s="513"/>
+      <x:c r="G15" s="488"/>
+    </x:row>
+    <x:row r="16" ht="20" customHeight="1">
+      <x:c r="A16" s="496" t="str">
+        <x:v>Tensor pipe active (% elapsed)</x:v>
+      </x:c>
+      <x:c r="B16" s="520" t="n">
+        <x:v>19.754167</x:v>
+      </x:c>
+      <x:c r="C16" s="520" t="n">
+        <x:v>20.866702</x:v>
+      </x:c>
+      <x:c r="D16" s="520" t="n">
+        <x:v>23.213088</x:v>
+      </x:c>
+      <x:c r="E16" s="521" t="n">
+        <x:f>C16/B16-1</x:f>
+        <x:v>0.056319003479114116</x:v>
+      </x:c>
+      <x:c r="F16" s="513"/>
+      <x:c r="G16" s="488"/>
+    </x:row>
+    <x:row r="17" ht="20" customHeight="1">
+      <x:c r="A17" s="496" t="str">
+        <x:v>Global-load instructions</x:v>
+      </x:c>
+      <x:c r="B17" s="522" t="n">
+        <x:v>112640</x:v>
+      </x:c>
+      <x:c r="C17" s="522" t="n">
+        <x:v>22528</x:v>
+      </x:c>
+      <x:c r="D17" s="522" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="521" t="n">
+        <x:f>C17/B17-1</x:f>
+        <x:v>-0.8</x:v>
+      </x:c>
+      <x:c r="F17" s="513"/>
+      <x:c r="G17" s="488"/>
+    </x:row>
+    <x:row r="18" ht="20" customHeight="1">
+      <x:c r="A18" s="496" t="str">
+        <x:v>Shared-load instructions</x:v>
+      </x:c>
+      <x:c r="B18" s="522" t="n">
+        <x:v>180224</x:v>
+      </x:c>
+      <x:c r="C18" s="522" t="n">
+        <x:v>360448</x:v>
+      </x:c>
+      <x:c r="D18" s="522" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="521" t="n">
+        <x:f>C18/B18-1</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F18" s="513"/>
+      <x:c r="G18" s="488"/>
+    </x:row>
+    <x:row r="19" ht="20" customHeight="1">
+      <x:c r="A19" s="496" t="str">
+        <x:v>Executed instructions</x:v>
+      </x:c>
+      <x:c r="B19" s="522" t="n">
+        <x:v>19758052</x:v>
+      </x:c>
+      <x:c r="C19" s="522" t="n">
+        <x:v>18422500</x:v>
+      </x:c>
+      <x:c r="D19" s="522" t="n">
+        <x:v>3460690</x:v>
+      </x:c>
+      <x:c r="E19" s="521" t="n">
+        <x:f>C19/B19-1</x:f>
+        <x:v>-0.06759532771753007</x:v>
+      </x:c>
+      <x:c r="F19" s="513"/>
+      <x:c r="G19" s="488"/>
+    </x:row>
+    <x:row r="20" ht="20" customHeight="1">
+      <x:c r="A20" s="496" t="str">
+        <x:v>Barrier stall (cycles / inst)</x:v>
+      </x:c>
+      <x:c r="B20" s="520" t="n">
+        <x:v>11.560631</x:v>
+      </x:c>
+      <x:c r="C20" s="520" t="n">
+        <x:v>7.831359</x:v>
+      </x:c>
+      <x:c r="D20" s="520" t="n">
+        <x:v>44.203692</x:v>
+      </x:c>
+      <x:c r="E20" s="521" t="n">
+        <x:f>C20/B20-1</x:f>
+        <x:v>-0.32258377592018983</x:v>
+      </x:c>
+      <x:c r="F20" s="513"/>
+      <x:c r="G20" s="488"/>
+    </x:row>
+    <x:row r="21" ht="20" customHeight="1">
+      <x:c r="A21" s="523" t="str">
+        <x:v>Long scoreboard (cycles / inst)</x:v>
+      </x:c>
+      <x:c r="B21" s="524" t="n">
+        <x:v>0.922514</x:v>
+      </x:c>
+      <x:c r="C21" s="524" t="n">
+        <x:v>1.159809</x:v>
+      </x:c>
+      <x:c r="D21" s="524" t="n">
+        <x:v>7.893343</x:v>
+      </x:c>
+      <x:c r="E21" s="525" t="n">
+        <x:f>C21/B21-1</x:f>
+        <x:v>0.25722644859590216</x:v>
+      </x:c>
+      <x:c r="F21" s="513"/>
+      <x:c r="G21" s="488"/>
+    </x:row>
+    <x:row r="22" ht="20" customHeight="1">
+      <x:c r="A22" s="512"/>
+      <x:c r="B22" s="488"/>
+      <x:c r="C22" s="488"/>
+      <x:c r="D22" s="488"/>
+      <x:c r="E22" s="488"/>
+      <x:c r="F22" s="488"/>
+      <x:c r="G22" s="488"/>
+    </x:row>
+    <x:row r="23" ht="20" customHeight="1">
+      <x:c r="A23" s="512"/>
+      <x:c r="B23" s="488"/>
+      <x:c r="C23" s="488"/>
+      <x:c r="D23" s="488"/>
+      <x:c r="E23" s="488"/>
+      <x:c r="F23" s="488"/>
+      <x:c r="G23" s="488"/>
+    </x:row>
+    <x:row r="24" ht="20" customHeight="1">
+      <x:c r="A24" s="468" t="str">
+        <x:v>Current-Best Kernel Configuration</x:v>
+      </x:c>
+      <x:c r="B24" s="480"/>
+      <x:c r="C24" s="480"/>
+      <x:c r="D24" s="480"/>
+      <x:c r="E24" s="480"/>
+      <x:c r="F24" s="488"/>
+      <x:c r="G24" s="488"/>
+    </x:row>
+    <x:row r="25" ht="20" customHeight="1">
+      <x:c r="A25" s="526" t="str">
+        <x:v>Weight block / weight tile</x:v>
+      </x:c>
+      <x:c r="B25" s="495" t="str">
+        <x:v>64 x 64</x:v>
+      </x:c>
+      <x:c r="C25" s="488"/>
+      <x:c r="D25" s="488"/>
+      <x:c r="E25" s="488"/>
+      <x:c r="F25" s="488"/>
+      <x:c r="G25" s="488"/>
+    </x:row>
+    <x:row r="26" ht="20" customHeight="1">
+      <x:c r="A26" s="527" t="str">
+        <x:v>Output tile</x:v>
+      </x:c>
+      <x:c r="B26" s="499" t="str">
+        <x:v>128 x 64</x:v>
+      </x:c>
+      <x:c r="C26" s="488"/>
+      <x:c r="D26" s="488"/>
+      <x:c r="E26" s="488"/>
+      <x:c r="F26" s="488"/>
+      <x:c r="G26" s="488"/>
+    </x:row>
+    <x:row r="27" ht="20" customHeight="1">
+      <x:c r="A27" s="527" t="str">
+        <x:v>Math warpgroup</x:v>
+      </x:c>
+      <x:c r="B27" s="499" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C27" s="488"/>
+      <x:c r="D27" s="488"/>
+      <x:c r="E27" s="488"/>
+      <x:c r="F27" s="488"/>
+      <x:c r="G27" s="488"/>
+    </x:row>
+    <x:row r="28" ht="20" customHeight="1">
+      <x:c r="A28" s="527" t="str">
+        <x:v>Threads / CTA</x:v>
+      </x:c>
+      <x:c r="B28" s="499" t="str">
+        <x:v>384</x:v>
+      </x:c>
+      <x:c r="C28" s="488"/>
+      <x:c r="D28" s="488"/>
+      <x:c r="E28" s="488"/>
+      <x:c r="F28" s="488"/>
+      <x:c r="G28" s="488"/>
+    </x:row>
+    <x:row r="29" ht="20" customHeight="1">
+      <x:c r="A29" s="527" t="str">
+        <x:v>TMA pipeline stages</x:v>
+      </x:c>
+      <x:c r="B29" s="499" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C29" s="488"/>
+      <x:c r="D29" s="488"/>
+      <x:c r="E29" s="488"/>
+      <x:c r="F29" s="488"/>
+      <x:c r="G29" s="488"/>
+    </x:row>
+    <x:row r="30" ht="20" customHeight="1">
+      <x:c r="A30" s="528" t="str">
+        <x:v>Persistent occupancy target</x:v>
+      </x:c>
+      <x:c r="B30" s="529" t="str">
+        <x:v>2 CTA / SM</x:v>
+      </x:c>
+      <x:c r="C30" s="488"/>
+      <x:c r="D30" s="488"/>
+      <x:c r="E30" s="488"/>
+      <x:c r="F30" s="488"/>
+      <x:c r="G30" s="488"/>
+    </x:row>
+    <x:row r="31" ht="20" customHeight="1">
+      <x:c r="A31" s="512"/>
+      <x:c r="B31" s="488"/>
+      <x:c r="C31" s="488"/>
+      <x:c r="D31" s="488"/>
+      <x:c r="E31" s="488"/>
+      <x:c r="F31" s="488"/>
+      <x:c r="G31" s="488"/>
+    </x:row>
+    <x:row r="32" ht="42" customHeight="1">
+      <x:c r="A32" s="530" t="str">
+        <x:v>Result: stage-kind reached 1.261x, 1.259x, and 1.262x over DeepGEMM in three paired 100-iteration runs. The broader shape sweep showed scheduling noise, so only the repeated target result is treated as verified.</x:v>
+      </x:c>
+      <x:c r="B32" s="531"/>
+      <x:c r="C32" s="531"/>
+      <x:c r="D32" s="531"/>
+      <x:c r="E32" s="531"/>
+      <x:c r="F32" s="531"/>
+      <x:c r="G32" s="531"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A2:G2"/>
+    <x:mergeCell ref="A12:E12"/>
+    <x:mergeCell ref="A24:E24"/>
+    <x:mergeCell ref="A32:G32"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>

</xml_diff>

<commit_message>
docs: record all-shape benchmark
Add repeated paired results for all 12 standard shapes and document the shape-dependent crossover. Workbook rendering and formula validation passed.
</commit_message>
<xml_diff>
--- a/docs/hybrid_sparse_performance.xlsx
+++ b/docs/hybrid_sparse_performance.xlsx
@@ -2,16 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R2c2671842a2f4acb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="Rdf2687aedcad44b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R7eebe30c090b42b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="R73289d838cff4067"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="R63c59aef73b94102"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="Rdffd2fc2c695447d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="R802bad8d5dd24658"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register Realloc" sheetId="8" r:id="R007fce9f93794f65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Iterations" sheetId="9" r:id="Reb208ff8bc9b4b82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output Tile Reuse" sheetId="10" r:id="Rbb95db97bd31481c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R43262663f511418b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R652fb022ea5248c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R1c3730a503a2482a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="R00f6c05150de41dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="Re7dc6092db964ce1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="R7803c82e761a47ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="Raf953dcd44bb4c81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register Realloc" sheetId="8" r:id="R2e871898bbed4bfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Iterations" sheetId="9" r:id="Rcdf3df8e3b7844b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output Tile Reuse" sheetId="10" r:id="Rb6f3134ce876477e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Specified Shapes" sheetId="11" r:id="R0a129b80b3364ea4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -327,7 +328,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="44">
+  <x:fills count="50">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -512,6 +513,36 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF5F8FC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F3265"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EEF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF294E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9F2E3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F6FA"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -907,7 +938,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="532">
+  <x:cellXfs count="626">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2100,11 +2131,215 @@
     <x:xf numFmtId="0" fontId="51" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="40" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="46" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="46" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="46" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="46" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="46" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="46" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="49" fillId="41" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="42" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="43" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="48" fillId="43" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="48" fillId="43" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="43" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="48" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="48" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="49" fillId="47" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="49" fillId="47" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="49" fillId="47" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="49" fillId="47" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="48" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="48" fillId="48" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="48" fillId="48" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="48" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="49" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="48" fillId="49" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="48" fillId="49" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="49" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="50" fillId="49" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="50" fillId="49" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="51" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="51" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="34" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="34" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="35" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="49" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="49" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="49" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="37" fillId="49" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="37" fillId="49" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="37" fillId="49" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="42" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="41" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="45" fillId="49" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="45" fillId="49" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="45" fillId="49" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="41" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="46" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="48" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="50" fillId="49" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="50" fillId="49" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="50" fillId="49" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="48" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="3">
+  <x:dxfs count="7">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -2134,6 +2369,48 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFFAD4D4"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1D6B3C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFD9F2E3"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C2E2E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE0E0"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1D6B3C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFD9F2E3"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C2E2E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE0E0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -2599,26 +2876,26 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="440" t="str">
+      <x:c r="A1" s="532" t="str">
         <x:v>Hybrid Sparse Output-Tile Reuse</x:v>
       </x:c>
-      <x:c r="B1" s="440"/>
-      <x:c r="C1" s="440"/>
-      <x:c r="D1" s="440"/>
-      <x:c r="E1" s="440"/>
-      <x:c r="F1" s="440"/>
-      <x:c r="G1" s="440"/>
+      <x:c r="B1" s="532"/>
+      <x:c r="C1" s="532"/>
+      <x:c r="D1" s="532"/>
+      <x:c r="E1" s="532"/>
+      <x:c r="F1" s="532"/>
+      <x:c r="G1" s="532"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
-      <x:c r="A2" s="441" t="str">
+      <x:c r="A2" s="533" t="str">
         <x:v>NVIDIA H20 | BF16 input/output | FP32 accumulation | M x N x K = 4096 x 2048 x 1408 | L2 flush disabled</x:v>
       </x:c>
-      <x:c r="B2" s="441"/>
-      <x:c r="C2" s="441"/>
-      <x:c r="D2" s="441"/>
-      <x:c r="E2" s="441"/>
-      <x:c r="F2" s="441"/>
-      <x:c r="G2" s="441"/>
+      <x:c r="B2" s="533"/>
+      <x:c r="C2" s="533"/>
+      <x:c r="D2" s="533"/>
+      <x:c r="E2" s="533"/>
+      <x:c r="F2" s="533"/>
+      <x:c r="G2" s="533"/>
     </x:row>
     <x:row r="3" ht="20" customHeight="1">
       <x:c r="A3" s="488"/>
@@ -2630,25 +2907,25 @@
       <x:c r="G3" s="488"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="489" t="str">
+      <x:c r="A4" s="534" t="str">
         <x:v>Version</x:v>
       </x:c>
-      <x:c r="B4" s="490" t="str">
+      <x:c r="B4" s="535" t="str">
         <x:v>Run 1 (us)</x:v>
       </x:c>
-      <x:c r="C4" s="490" t="str">
+      <x:c r="C4" s="535" t="str">
         <x:v>Run 2 (us)</x:v>
       </x:c>
-      <x:c r="D4" s="490" t="str">
+      <x:c r="D4" s="535" t="str">
         <x:v>Run 3 (us)</x:v>
       </x:c>
-      <x:c r="E4" s="490" t="str">
+      <x:c r="E4" s="535" t="str">
         <x:v>Average (us)</x:v>
       </x:c>
-      <x:c r="F4" s="490" t="str">
+      <x:c r="F4" s="535" t="str">
         <x:v>Paired speedup</x:v>
       </x:c>
-      <x:c r="G4" s="491" t="str">
+      <x:c r="G4" s="535" t="str">
         <x:v>Decision</x:v>
       </x:c>
     </x:row>
@@ -2673,7 +2950,7 @@
         <x:f>AVERAGE($B$9/B5,$C$9/C5,$D$9/D5)</x:f>
         <x:v>1.1659354427141075</x:v>
       </x:c>
-      <x:c r="G5" s="495" t="str">
+      <x:c r="G5" s="543" t="str">
         <x:v>Baseline</x:v>
       </x:c>
     </x:row>
@@ -2698,81 +2975,81 @@
         <x:f>AVERAGE($B$9/B6,$C$9/C6,$D$9/D6)</x:f>
         <x:v>1.226884757589631</x:v>
       </x:c>
-      <x:c r="G6" s="499" t="str">
+      <x:c r="G6" s="544" t="str">
         <x:v>Retained</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
-      <x:c r="A7" s="500" t="str">
+      <x:c r="A7" s="553" t="str">
         <x:v>Stage kind</x:v>
       </x:c>
-      <x:c r="B7" s="501" t="n">
+      <x:c r="B7" s="554" t="n">
         <x:v>144.07</x:v>
       </x:c>
-      <x:c r="C7" s="501" t="n">
+      <x:c r="C7" s="554" t="n">
         <x:v>144.4</x:v>
       </x:c>
-      <x:c r="D7" s="501" t="n">
+      <x:c r="D7" s="554" t="n">
         <x:v>144.33</x:v>
       </x:c>
-      <x:c r="E7" s="501" t="n">
+      <x:c r="E7" s="554" t="n">
         <x:f>AVERAGE(B7:D7)</x:f>
         <x:v>144.26666666666668</x:v>
       </x:c>
-      <x:c r="F7" s="502" t="n">
+      <x:c r="F7" s="555" t="n">
         <x:f>AVERAGE($B$9/B7,$C$9/C7,$D$9/D7)</x:f>
         <x:v>1.2603285021897923</x:v>
       </x:c>
-      <x:c r="G7" s="503" t="str">
+      <x:c r="G7" s="556" t="str">
         <x:v>Current best</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
-      <x:c r="A8" s="504" t="str">
+      <x:c r="A8" s="557" t="str">
         <x:v>Stage selector</x:v>
       </x:c>
-      <x:c r="B8" s="505" t="n">
+      <x:c r="B8" s="558" t="n">
         <x:v>144.24</x:v>
       </x:c>
-      <x:c r="C8" s="505" t="n">
+      <x:c r="C8" s="558" t="n">
         <x:v>145.22</x:v>
       </x:c>
-      <x:c r="D8" s="505" t="n">
+      <x:c r="D8" s="558" t="n">
         <x:v>144.61</x:v>
       </x:c>
-      <x:c r="E8" s="505" t="n">
+      <x:c r="E8" s="558" t="n">
         <x:f>AVERAGE(B8:D8)</x:f>
         <x:v>144.69000000000003</x:v>
       </x:c>
-      <x:c r="F8" s="506" t="n">
+      <x:c r="F8" s="559" t="n">
         <x:f>AVERAGE($B$9/B8,$C$9/C8,$D$9/D8)</x:f>
         <x:v>1.256650106303988</x:v>
       </x:c>
-      <x:c r="G8" s="507" t="str">
+      <x:c r="G8" s="560" t="str">
         <x:v>Not adopted</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
-      <x:c r="A9" s="508" t="str">
+      <x:c r="A9" s="561" t="str">
         <x:v>DeepGEMM</x:v>
       </x:c>
-      <x:c r="B9" s="509" t="n">
+      <x:c r="B9" s="562" t="n">
         <x:v>181.6</x:v>
       </x:c>
-      <x:c r="C9" s="509" t="n">
+      <x:c r="C9" s="562" t="n">
         <x:v>181.72</x:v>
       </x:c>
-      <x:c r="D9" s="509" t="n">
+      <x:c r="D9" s="562" t="n">
         <x:v>182.15</x:v>
       </x:c>
-      <x:c r="E9" s="509" t="n">
+      <x:c r="E9" s="562" t="n">
         <x:f>AVERAGE(B9:D9)</x:f>
         <x:v>181.82333333333335</x:v>
       </x:c>
-      <x:c r="F9" s="510" t="n">
+      <x:c r="F9" s="563" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G9" s="511" t="str">
+      <x:c r="G9" s="564" t="str">
         <x:v>Dense baseline</x:v>
       </x:c>
     </x:row>
@@ -2795,30 +3072,30 @@
       <x:c r="G11" s="488"/>
     </x:row>
     <x:row r="12" ht="20" customHeight="1">
-      <x:c r="A12" s="468" t="str">
+      <x:c r="A12" s="540" t="str">
         <x:v>Paired NCU Comparison at 4096 x 2048 x 1408</x:v>
       </x:c>
-      <x:c r="B12" s="469"/>
-      <x:c r="C12" s="469"/>
-      <x:c r="D12" s="469"/>
-      <x:c r="E12" s="469"/>
+      <x:c r="B12" s="541"/>
+      <x:c r="C12" s="541"/>
+      <x:c r="D12" s="541"/>
+      <x:c r="E12" s="541"/>
       <x:c r="F12" s="513"/>
       <x:c r="G12" s="488"/>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
-      <x:c r="A13" s="489" t="str">
+      <x:c r="A13" s="534" t="str">
         <x:v>Metric</x:v>
       </x:c>
-      <x:c r="B13" s="516" t="str">
+      <x:c r="B13" s="538" t="str">
         <x:v>Output 128x64</x:v>
       </x:c>
-      <x:c r="C13" s="516" t="str">
+      <x:c r="C13" s="538" t="str">
         <x:v>Stage kind</x:v>
       </x:c>
-      <x:c r="D13" s="516" t="str">
+      <x:c r="D13" s="538" t="str">
         <x:v>DeepGEMM</x:v>
       </x:c>
-      <x:c r="E13" s="517" t="str">
+      <x:c r="E13" s="538" t="str">
         <x:v>Stage vs Output</x:v>
       </x:c>
       <x:c r="F13" s="513"/>
@@ -2837,7 +3114,7 @@
       <x:c r="D14" s="518" t="n">
         <x:v>201.504</x:v>
       </x:c>
-      <x:c r="E14" s="519" t="n">
+      <x:c r="E14" s="551" t="n">
         <x:f>C14/B14-1</x:f>
         <x:v>-0.060385118713778385</x:v>
       </x:c>
@@ -2857,7 +3134,7 @@
       <x:c r="D15" s="520" t="n">
         <x:v>92.852352</x:v>
       </x:c>
-      <x:c r="E15" s="521" t="n">
+      <x:c r="E15" s="552" t="n">
         <x:f>C15/B15-1</x:f>
         <x:v>0.05631899011080832</x:v>
       </x:c>
@@ -2877,7 +3154,7 @@
       <x:c r="D16" s="520" t="n">
         <x:v>23.213088</x:v>
       </x:c>
-      <x:c r="E16" s="521" t="n">
+      <x:c r="E16" s="552" t="n">
         <x:f>C16/B16-1</x:f>
         <x:v>0.056319003479114116</x:v>
       </x:c>
@@ -2897,7 +3174,7 @@
       <x:c r="D17" s="522" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E17" s="521" t="n">
+      <x:c r="E17" s="552" t="n">
         <x:f>C17/B17-1</x:f>
         <x:v>-0.8</x:v>
       </x:c>
@@ -2917,7 +3194,7 @@
       <x:c r="D18" s="522" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E18" s="521" t="n">
+      <x:c r="E18" s="552" t="n">
         <x:f>C18/B18-1</x:f>
         <x:v>1</x:v>
       </x:c>
@@ -2937,7 +3214,7 @@
       <x:c r="D19" s="522" t="n">
         <x:v>3460690</x:v>
       </x:c>
-      <x:c r="E19" s="521" t="n">
+      <x:c r="E19" s="552" t="n">
         <x:f>C19/B19-1</x:f>
         <x:v>-0.06759532771753007</x:v>
       </x:c>
@@ -2957,7 +3234,7 @@
       <x:c r="D20" s="520" t="n">
         <x:v>44.203692</x:v>
       </x:c>
-      <x:c r="E20" s="521" t="n">
+      <x:c r="E20" s="552" t="n">
         <x:f>C20/B20-1</x:f>
         <x:v>-0.32258377592018983</x:v>
       </x:c>
@@ -2965,19 +3242,19 @@
       <x:c r="G20" s="488"/>
     </x:row>
     <x:row r="21" ht="20" customHeight="1">
-      <x:c r="A21" s="523" t="str">
+      <x:c r="A21" s="496" t="str">
         <x:v>Long scoreboard (cycles / inst)</x:v>
       </x:c>
-      <x:c r="B21" s="524" t="n">
+      <x:c r="B21" s="520" t="n">
         <x:v>0.922514</x:v>
       </x:c>
-      <x:c r="C21" s="524" t="n">
+      <x:c r="C21" s="520" t="n">
         <x:v>1.159809</x:v>
       </x:c>
-      <x:c r="D21" s="524" t="n">
+      <x:c r="D21" s="520" t="n">
         <x:v>7.893343</x:v>
       </x:c>
-      <x:c r="E21" s="525" t="n">
+      <x:c r="E21" s="552" t="n">
         <x:f>C21/B21-1</x:f>
         <x:v>0.25722644859590216</x:v>
       </x:c>
@@ -3003,21 +3280,21 @@
       <x:c r="G23" s="488"/>
     </x:row>
     <x:row r="24" ht="20" customHeight="1">
-      <x:c r="A24" s="468" t="str">
+      <x:c r="A24" s="540" t="str">
         <x:v>Current-Best Kernel Configuration</x:v>
       </x:c>
-      <x:c r="B24" s="480"/>
-      <x:c r="C24" s="480"/>
-      <x:c r="D24" s="480"/>
-      <x:c r="E24" s="480"/>
+      <x:c r="B24" s="542"/>
+      <x:c r="C24" s="542"/>
+      <x:c r="D24" s="542"/>
+      <x:c r="E24" s="542"/>
       <x:c r="F24" s="488"/>
       <x:c r="G24" s="488"/>
     </x:row>
     <x:row r="25" ht="20" customHeight="1">
-      <x:c r="A25" s="526" t="str">
+      <x:c r="A25" s="565" t="str">
         <x:v>Weight block / weight tile</x:v>
       </x:c>
-      <x:c r="B25" s="495" t="str">
+      <x:c r="B25" s="543" t="str">
         <x:v>64 x 64</x:v>
       </x:c>
       <x:c r="C25" s="488"/>
@@ -3027,10 +3304,10 @@
       <x:c r="G25" s="488"/>
     </x:row>
     <x:row r="26" ht="20" customHeight="1">
-      <x:c r="A26" s="527" t="str">
+      <x:c r="A26" s="566" t="str">
         <x:v>Output tile</x:v>
       </x:c>
-      <x:c r="B26" s="499" t="str">
+      <x:c r="B26" s="544" t="str">
         <x:v>128 x 64</x:v>
       </x:c>
       <x:c r="C26" s="488"/>
@@ -3040,10 +3317,10 @@
       <x:c r="G26" s="488"/>
     </x:row>
     <x:row r="27" ht="20" customHeight="1">
-      <x:c r="A27" s="527" t="str">
+      <x:c r="A27" s="566" t="str">
         <x:v>Math warpgroup</x:v>
       </x:c>
-      <x:c r="B27" s="499" t="str">
+      <x:c r="B27" s="544" t="str">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C27" s="488"/>
@@ -3053,10 +3330,10 @@
       <x:c r="G27" s="488"/>
     </x:row>
     <x:row r="28" ht="20" customHeight="1">
-      <x:c r="A28" s="527" t="str">
+      <x:c r="A28" s="566" t="str">
         <x:v>Threads / CTA</x:v>
       </x:c>
-      <x:c r="B28" s="499" t="str">
+      <x:c r="B28" s="544" t="str">
         <x:v>384</x:v>
       </x:c>
       <x:c r="C28" s="488"/>
@@ -3066,10 +3343,10 @@
       <x:c r="G28" s="488"/>
     </x:row>
     <x:row r="29" ht="20" customHeight="1">
-      <x:c r="A29" s="527" t="str">
+      <x:c r="A29" s="566" t="str">
         <x:v>TMA pipeline stages</x:v>
       </x:c>
-      <x:c r="B29" s="499" t="str">
+      <x:c r="B29" s="544" t="str">
         <x:v>3</x:v>
       </x:c>
       <x:c r="C29" s="488"/>
@@ -3079,10 +3356,10 @@
       <x:c r="G29" s="488"/>
     </x:row>
     <x:row r="30" ht="20" customHeight="1">
-      <x:c r="A30" s="528" t="str">
+      <x:c r="A30" s="566" t="str">
         <x:v>Persistent occupancy target</x:v>
       </x:c>
-      <x:c r="B30" s="529" t="str">
+      <x:c r="B30" s="544" t="str">
         <x:v>2 CTA / SM</x:v>
       </x:c>
       <x:c r="C30" s="488"/>
@@ -3101,15 +3378,15 @@
       <x:c r="G31" s="488"/>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
-      <x:c r="A32" s="530" t="str">
+      <x:c r="A32" s="567" t="str">
         <x:v>Result: stage-kind reached 1.261x, 1.259x, and 1.262x over DeepGEMM in three paired 100-iteration runs. The broader shape sweep showed scheduling noise, so only the repeated target result is treated as verified.</x:v>
       </x:c>
-      <x:c r="B32" s="531"/>
-      <x:c r="C32" s="531"/>
-      <x:c r="D32" s="531"/>
-      <x:c r="E32" s="531"/>
-      <x:c r="F32" s="531"/>
-      <x:c r="G32" s="531"/>
+      <x:c r="B32" s="568"/>
+      <x:c r="C32" s="568"/>
+      <x:c r="D32" s="568"/>
+      <x:c r="E32" s="568"/>
+      <x:c r="F32" s="568"/>
+      <x:c r="G32" s="568"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3119,6 +3396,435 @@
     <x:mergeCell ref="A24:E24"/>
     <x:mergeCell ref="A32:G32"/>
   </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="532" t="str">
+        <x:v>Current-Best Kernel: All Specified Shapes</x:v>
+      </x:c>
+      <x:c r="B1" s="532"/>
+      <x:c r="C1" s="532"/>
+      <x:c r="D1" s="532"/>
+      <x:c r="E1" s="532"/>
+      <x:c r="F1" s="532"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="533" t="str">
+        <x:v>NVIDIA H20 | BF16 input/output | FP32 accumulation | no L2 flush | stage-kind kernel vs DeepGEMM</x:v>
+      </x:c>
+      <x:c r="B2" s="533"/>
+      <x:c r="C2" s="533"/>
+      <x:c r="D2" s="533"/>
+      <x:c r="E2" s="533"/>
+      <x:c r="F2" s="533"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="488"/>
+      <x:c r="B3" s="488"/>
+      <x:c r="C3" s="488"/>
+      <x:c r="D3" s="488"/>
+      <x:c r="E3" s="488"/>
+      <x:c r="F3" s="488"/>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="614" t="str">
+        <x:v>Shape (M x N x K)</x:v>
+      </x:c>
+      <x:c r="B4" s="614" t="str">
+        <x:v>Hybrid median (us)</x:v>
+      </x:c>
+      <x:c r="C4" s="614" t="str">
+        <x:v>DeepGEMM median (us)</x:v>
+      </x:c>
+      <x:c r="D4" s="614" t="str">
+        <x:v>Paired speedup median</x:v>
+      </x:c>
+      <x:c r="E4" s="614" t="str">
+        <x:v>Repeats</x:v>
+      </x:c>
+      <x:c r="F4" s="614" t="str">
+        <x:v>Result</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="615" t="str">
+        <x:v>128 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B5" s="518" t="n">
+        <x:v>18.288</x:v>
+      </x:c>
+      <x:c r="C5" s="518" t="n">
+        <x:v>10.374</x:v>
+      </x:c>
+      <x:c r="D5" s="494" t="n">
+        <x:v>0.54395</x:v>
+      </x:c>
+      <x:c r="E5" s="616" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F5" s="495" t="str">
+        <x:f>IF(D5&gt;=1,"Faster","Slower")</x:f>
+        <x:v>Slower</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="617" t="str">
+        <x:v>128 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B6" s="520" t="n">
+        <x:v>13.804</x:v>
+      </x:c>
+      <x:c r="C6" s="520" t="n">
+        <x:v>8.588</x:v>
+      </x:c>
+      <x:c r="D6" s="498" t="n">
+        <x:v>0.65502</x:v>
+      </x:c>
+      <x:c r="E6" s="618" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F6" s="499" t="str">
+        <x:f>IF(D6&gt;=1,"Faster","Slower")</x:f>
+        <x:v>Slower</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="617" t="str">
+        <x:v>256 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B7" s="520" t="n">
+        <x:v>18.318</x:v>
+      </x:c>
+      <x:c r="C7" s="520" t="n">
+        <x:v>14.534</x:v>
+      </x:c>
+      <x:c r="D7" s="498" t="n">
+        <x:v>0.781972</x:v>
+      </x:c>
+      <x:c r="E7" s="618" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F7" s="499" t="str">
+        <x:f>IF(D7&gt;=1,"Faster","Slower")</x:f>
+        <x:v>Slower</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="617" t="str">
+        <x:v>256 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B8" s="520" t="n">
+        <x:v>13.613</x:v>
+      </x:c>
+      <x:c r="C8" s="520" t="n">
+        <x:v>13.489</x:v>
+      </x:c>
+      <x:c r="D8" s="498" t="n">
+        <x:v>1.005102</x:v>
+      </x:c>
+      <x:c r="E8" s="618" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F8" s="499" t="str">
+        <x:f>IF(D8&gt;=1,"Faster","Slower")</x:f>
+        <x:v>Faster</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="617" t="str">
+        <x:v>512 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B9" s="520" t="n">
+        <x:v>57.813</x:v>
+      </x:c>
+      <x:c r="C9" s="520" t="n">
+        <x:v>50.62</x:v>
+      </x:c>
+      <x:c r="D9" s="498" t="n">
+        <x:v>0.869215</x:v>
+      </x:c>
+      <x:c r="E9" s="618" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F9" s="499" t="str">
+        <x:f>IF(D9&gt;=1,"Faster","Slower")</x:f>
+        <x:v>Slower</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="617" t="str">
+        <x:v>512 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B10" s="520" t="n">
+        <x:v>47.783</x:v>
+      </x:c>
+      <x:c r="C10" s="520" t="n">
+        <x:v>49.467</x:v>
+      </x:c>
+      <x:c r="D10" s="498" t="n">
+        <x:v>1.037029</x:v>
+      </x:c>
+      <x:c r="E10" s="618" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F10" s="499" t="str">
+        <x:f>IF(D10&gt;=1,"Faster","Slower")</x:f>
+        <x:v>Faster</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="617" t="str">
+        <x:v>1024 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B11" s="520" t="n">
+        <x:v>96.664</x:v>
+      </x:c>
+      <x:c r="C11" s="520" t="n">
+        <x:v>99.172</x:v>
+      </x:c>
+      <x:c r="D11" s="498" t="n">
+        <x:v>1.018104</x:v>
+      </x:c>
+      <x:c r="E11" s="618" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F11" s="499" t="str">
+        <x:f>IF(D11&gt;=1,"Faster","Slower")</x:f>
+        <x:v>Faster</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="617" t="str">
+        <x:v>1024 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B12" s="520" t="n">
+        <x:v>92.811</x:v>
+      </x:c>
+      <x:c r="C12" s="520" t="n">
+        <x:v>97.045</x:v>
+      </x:c>
+      <x:c r="D12" s="498" t="n">
+        <x:v>1.046104</x:v>
+      </x:c>
+      <x:c r="E12" s="618" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F12" s="499" t="str">
+        <x:f>IF(D12&gt;=1,"Faster","Slower")</x:f>
+        <x:v>Faster</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="617" t="str">
+        <x:v>2048 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B13" s="520" t="n">
+        <x:v>151.47</x:v>
+      </x:c>
+      <x:c r="C13" s="520" t="n">
+        <x:v>194.308</x:v>
+      </x:c>
+      <x:c r="D13" s="498" t="n">
+        <x:v>1.281488</x:v>
+      </x:c>
+      <x:c r="E13" s="618" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F13" s="499" t="str">
+        <x:f>IF(D13&gt;=1,"Faster","Slower")</x:f>
+        <x:v>Faster</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="617" t="str">
+        <x:v>2048 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B14" s="520" t="n">
+        <x:v>74.663</x:v>
+      </x:c>
+      <x:c r="C14" s="520" t="n">
+        <x:v>93.136</x:v>
+      </x:c>
+      <x:c r="D14" s="498" t="n">
+        <x:v>1.245302</x:v>
+      </x:c>
+      <x:c r="E14" s="618" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F14" s="499" t="str">
+        <x:f>IF(D14&gt;=1,"Faster","Slower")</x:f>
+        <x:v>Faster</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="617" t="str">
+        <x:v>4096 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B15" s="520" t="n">
+        <x:v>149.449</x:v>
+      </x:c>
+      <x:c r="C15" s="520" t="n">
+        <x:v>184.406</x:v>
+      </x:c>
+      <x:c r="D15" s="498" t="n">
+        <x:v>1.224565</x:v>
+      </x:c>
+      <x:c r="E15" s="618" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F15" s="499" t="str">
+        <x:f>IF(D15&gt;=1,"Faster","Slower")</x:f>
+        <x:v>Faster</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="619" t="str">
+        <x:v>4096 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B16" s="524" t="n">
+        <x:v>144.589</x:v>
+      </x:c>
+      <x:c r="C16" s="524" t="n">
+        <x:v>181.909</x:v>
+      </x:c>
+      <x:c r="D16" s="620" t="n">
+        <x:v>1.25736</x:v>
+      </x:c>
+      <x:c r="E16" s="621" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F16" s="529" t="str">
+        <x:f>IF(D16&gt;=1,"Faster","Slower")</x:f>
+        <x:v>Faster</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="488"/>
+      <x:c r="B17" s="488"/>
+      <x:c r="C17" s="488"/>
+      <x:c r="D17" s="488"/>
+      <x:c r="E17" s="488"/>
+      <x:c r="F17" s="488"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="488"/>
+      <x:c r="B18" s="488"/>
+      <x:c r="C18" s="488"/>
+      <x:c r="D18" s="488"/>
+      <x:c r="E18" s="488"/>
+      <x:c r="F18" s="488"/>
+    </x:row>
+    <x:row r="19" ht="23" customHeight="1">
+      <x:c r="A19" s="542" t="str">
+        <x:v>Summary</x:v>
+      </x:c>
+      <x:c r="B19" s="542"/>
+      <x:c r="C19" s="542"/>
+      <x:c r="D19" s="542"/>
+      <x:c r="E19" s="488"/>
+      <x:c r="F19" s="488"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="622" t="str">
+        <x:v>Shapes faster than DeepGEMM</x:v>
+      </x:c>
+      <x:c r="B20" s="495" t="n">
+        <x:f>COUNTIF(D5:D16,"&gt;=1")</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C20" s="488"/>
+      <x:c r="D20" s="488"/>
+      <x:c r="E20" s="488"/>
+      <x:c r="F20" s="488"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="623" t="str">
+        <x:v>Shapes reaching at least 1.25x</x:v>
+      </x:c>
+      <x:c r="B21" s="499" t="n">
+        <x:f>COUNTIF(D5:D16,"&gt;=1.25")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C21" s="488"/>
+      <x:c r="D21" s="488"/>
+      <x:c r="E21" s="488"/>
+      <x:c r="F21" s="488"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="623" t="str">
+        <x:v>Best shape</x:v>
+      </x:c>
+      <x:c r="B22" s="499" t="str">
+        <x:v>2048 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C22" s="488"/>
+      <x:c r="D22" s="488"/>
+      <x:c r="E22" s="488"/>
+      <x:c r="F22" s="488"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="624" t="str">
+        <x:v>Best median speedup</x:v>
+      </x:c>
+      <x:c r="B23" s="625" t="n">
+        <x:v>1.281488</x:v>
+      </x:c>
+      <x:c r="C23" s="488"/>
+      <x:c r="D23" s="488"/>
+      <x:c r="E23" s="488"/>
+      <x:c r="F23" s="488"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="488"/>
+      <x:c r="B24" s="488"/>
+      <x:c r="C24" s="488"/>
+      <x:c r="D24" s="488"/>
+      <x:c r="E24" s="488"/>
+      <x:c r="F24" s="488"/>
+    </x:row>
+    <x:row r="25" ht="48" customHeight="1">
+      <x:c r="A25" s="568" t="str">
+        <x:v>Interpretation: the 128 x 64 output tile is not suitable for every shape. It loses at small M, reaches parity around M=256-1024 depending on N/K, and provides the strongest gains at M&gt;=2048. M=512 and M=1024 use seven repeats because the initial sweep contained scheduling outliers.</x:v>
+      </x:c>
+      <x:c r="B25" s="568"/>
+      <x:c r="C25" s="568"/>
+      <x:c r="D25" s="568"/>
+      <x:c r="E25" s="568"/>
+      <x:c r="F25" s="568"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
+    <x:mergeCell ref="A19:D19"/>
+    <x:mergeCell ref="A25:F25"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="D5:D16">
+    <x:cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThanOrEqual">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="F5:F16">
+    <x:cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="Faster"/>
+    <x:cfRule type="containsText" dxfId="6" priority="4" operator="containsText" text="Slower"/>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs: record tuned hybrid sparse results
Add the final eight-shape paired benchmark results and summarize the dispatch experiments. The workbook was re-imported, rendered, and scanned for formula errors.
</commit_message>
<xml_diff>
--- a/docs/hybrid_sparse_performance.xlsx
+++ b/docs/hybrid_sparse_performance.xlsx
@@ -2,17 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R43262663f511418b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R652fb022ea5248c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R1c3730a503a2482a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="R00f6c05150de41dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="Re7dc6092db964ce1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="R7803c82e761a47ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="Raf953dcd44bb4c81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register Realloc" sheetId="8" r:id="R2e871898bbed4bfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Iterations" sheetId="9" r:id="Rcdf3df8e3b7844b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output Tile Reuse" sheetId="10" r:id="Rb6f3134ce876477e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Specified Shapes" sheetId="11" r:id="R0a129b80b3364ea4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R5eb3555ca3b942d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R4fbe53c6960741e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R8961f97deac04e8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="R619cc00686654058"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="Rffe933a0d411493a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="Rf64f8cf01e624509"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="R1aaaaf7266044af4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register Realloc" sheetId="8" r:id="R97db8ba5eea34c30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Iterations" sheetId="9" r:id="Rb921ee5a6080407b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output Tile Reuse" sheetId="10" r:id="R9ccbbe2c36804bbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Specified Shapes" sheetId="11" r:id="R21cc14967f8e46ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuned Dispatch" sheetId="12" r:id="Rcaddb03379554db6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -35,7 +36,7 @@
     <x:numFmt numFmtId="208" formatCode="#,##0"/>
     <x:numFmt numFmtId="209" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="52">
+  <x:fonts count="56">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -327,8 +328,30 @@
       <x:color rgb="FF4E5D6C"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF17637D"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF526174"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="50">
+  <x:fills count="55">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -575,8 +598,33 @@
         <x:fgColor rgb="FFF3F6FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF203764"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF274A78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDF2F7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F7FA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="41">
+  <x:borders count="44">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -934,11 +982,29 @@
         <x:color rgb="FFD7DEE8"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8E1EC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD8E1EC"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8E1EC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD8E1EC"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="626">
+  <x:cellXfs count="667">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2335,11 +2401,102 @@
     <x:xf numFmtId="0" fontId="50" fillId="49" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="50" fillId="49" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="48" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="52" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="52" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="53" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="53" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="53" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="53" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="53" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="53" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="53" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="53" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="53" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="53" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="53" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="53" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="53" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="53" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="53" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="53" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="53" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="53" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="53" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="54" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="54" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="54" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="54" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="55" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="55" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="7">
+  <x:dxfs count="9">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -2378,7 +2535,7 @@
         <x:color rgb="FF1D6B3C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9F2E3"/>
         </x:patternFill>
       </x:fill>
@@ -2388,7 +2545,7 @@
         <x:color rgb="FF9C2E2E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE0E0"/>
         </x:patternFill>
       </x:fill>
@@ -2399,7 +2556,7 @@
         <x:color rgb="FF1D6B3C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9F2E3"/>
         </x:patternFill>
       </x:fill>
@@ -2409,8 +2566,28 @@
         <x:color rgb="FF9C2E2E"/>
       </x:font>
       <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE0E0"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF176B3A"/>
+      </x:font>
+      <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE0E0"/>
+          <x:bgColor rgb="FFD7F0DF"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FFA93333"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFADADA"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -3829,6 +4006,288 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="21" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="21" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="628" t="str">
+        <x:v>Tuned Hybrid Sparse Dispatch</x:v>
+      </x:c>
+      <x:c r="B1" s="628"/>
+      <x:c r="C1" s="628"/>
+      <x:c r="D1" s="628"/>
+      <x:c r="E1" s="628"/>
+      <x:c r="F1" s="628"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="631" t="str">
+        <x:v>NVIDIA H20 | BF16 input/output | FP32 accumulation | 25% hybrid sparsity | 7 paired repeats x 300 | commit 76e5d8b</x:v>
+      </x:c>
+      <x:c r="B2" s="631"/>
+      <x:c r="C2" s="631"/>
+      <x:c r="D2" s="631"/>
+      <x:c r="E2" s="631"/>
+      <x:c r="F2" s="631"/>
+    </x:row>
+    <x:row r="4" ht="34" customHeight="1">
+      <x:c r="A4" s="636" t="str">
+        <x:v>Shape (M x N x K)</x:v>
+      </x:c>
+      <x:c r="B4" s="636" t="str">
+        <x:v>Tuned median (us)</x:v>
+      </x:c>
+      <x:c r="C4" s="636" t="str">
+        <x:v>DeepGEMM median (us)</x:v>
+      </x:c>
+      <x:c r="D4" s="636" t="str">
+        <x:v>Speedup</x:v>
+      </x:c>
+      <x:c r="E4" s="636" t="str">
+        <x:v>Repeats</x:v>
+      </x:c>
+      <x:c r="F4" s="636" t="str">
+        <x:v>Selected kernel</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="641" t="str">
+        <x:v>128 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B5" s="647" t="n">
+        <x:v>8.87</x:v>
+      </x:c>
+      <x:c r="C5" s="647" t="n">
+        <x:v>9.54</x:v>
+      </x:c>
+      <x:c r="D5" s="650" t="n">
+        <x:f>C5/B5</x:f>
+        <x:v>1.0755355129650508</x:v>
+      </x:c>
+      <x:c r="E5" s="653" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F5" s="641" t="str">
+        <x:v>output48 descriptor reuse</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="642" t="str">
+        <x:v>128 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B6" s="648" t="n">
+        <x:v>8.04</x:v>
+      </x:c>
+      <x:c r="C6" s="648" t="n">
+        <x:v>8.59</x:v>
+      </x:c>
+      <x:c r="D6" s="651" t="n">
+        <x:f>C6/B6</x:f>
+        <x:v>1.068407960199005</x:v>
+      </x:c>
+      <x:c r="E6" s="654" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F6" s="642" t="str">
+        <x:v>output64 fixed-shape stage7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="642" t="str">
+        <x:v>256 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B7" s="648" t="n">
+        <x:v>12.55</x:v>
+      </x:c>
+      <x:c r="C7" s="648" t="n">
+        <x:v>13.75</x:v>
+      </x:c>
+      <x:c r="D7" s="651" t="n">
+        <x:f>C7/B7</x:f>
+        <x:v>1.095617529880478</x:v>
+      </x:c>
+      <x:c r="E7" s="654" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F7" s="642" t="str">
+        <x:v>output88 group-stage descriptor reuse</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="642" t="str">
+        <x:v>256 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B8" s="648" t="n">
+        <x:v>12.26</x:v>
+      </x:c>
+      <x:c r="C8" s="648" t="n">
+        <x:v>13.21</x:v>
+      </x:c>
+      <x:c r="D8" s="651" t="n">
+        <x:f>C8/B8</x:f>
+        <x:v>1.0774877650897228</x:v>
+      </x:c>
+      <x:c r="E8" s="654" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F8" s="642" t="str">
+        <x:v>output128 group-stage descriptor reuse</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="642" t="str">
+        <x:v>512 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B9" s="648" t="n">
+        <x:v>21.89</x:v>
+      </x:c>
+      <x:c r="C9" s="648" t="n">
+        <x:v>25.2</x:v>
+      </x:c>
+      <x:c r="D9" s="651" t="n">
+        <x:f>C9/B9</x:f>
+        <x:v>1.1512105984467793</x:v>
+      </x:c>
+      <x:c r="E9" s="654" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F9" s="642" t="str">
+        <x:v>output80 group-stage descriptor reuse</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="642" t="str">
+        <x:v>512 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B10" s="648" t="n">
+        <x:v>22.86</x:v>
+      </x:c>
+      <x:c r="C10" s="648" t="n">
+        <x:v>24.54</x:v>
+      </x:c>
+      <x:c r="D10" s="651" t="n">
+        <x:f>C10/B10</x:f>
+        <x:v>1.073490813648294</x:v>
+      </x:c>
+      <x:c r="E10" s="654" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F10" s="642" t="str">
+        <x:v>output128 group-stage descriptor reuse</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="642" t="str">
+        <x:v>1024 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B11" s="648" t="n">
+        <x:v>41.98</x:v>
+      </x:c>
+      <x:c r="C11" s="648" t="n">
+        <x:v>48.45</x:v>
+      </x:c>
+      <x:c r="D11" s="651" t="n">
+        <x:f>C11/B11</x:f>
+        <x:v>1.1541210100047643</x:v>
+      </x:c>
+      <x:c r="E11" s="654" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F11" s="642" t="str">
+        <x:v>output80 group-stage descriptor reuse</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="643" t="str">
+        <x:v>1024 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B12" s="649" t="n">
+        <x:v>43.42</x:v>
+      </x:c>
+      <x:c r="C12" s="649" t="n">
+        <x:v>47.33</x:v>
+      </x:c>
+      <x:c r="D12" s="652" t="n">
+        <x:f>C12/B12</x:f>
+        <x:v>1.0900506678949793</x:v>
+      </x:c>
+      <x:c r="E12" s="655" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F12" s="643" t="str">
+        <x:v>output96 baseline group-stage</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="656" t="str">
+        <x:v>Summary</x:v>
+      </x:c>
+      <x:c r="B15" s="656"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="658" t="str">
+        <x:v>Shapes faster than DeepGEMM</x:v>
+      </x:c>
+      <x:c r="B16" s="661" t="n">
+        <x:f>COUNTIF(D5:D12,"&gt;1")</x:f>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="658" t="str">
+        <x:v>Best speedup</x:v>
+      </x:c>
+      <x:c r="B17" s="662" t="n">
+        <x:f>MAX(D5:D12)</x:f>
+        <x:v>1.1541210100047643</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="658" t="str">
+        <x:v>Slowest tuned latency</x:v>
+      </x:c>
+      <x:c r="B18" s="663" t="n">
+        <x:f>MAX(B5:B12)</x:f>
+        <x:v>43.42</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="34" customHeight="1">
+      <x:c r="A21" s="666" t="str">
+        <x:v>Speedup is DeepGEMM latency divided by tuned total latency. Values above 1.0x mean the hybrid sparse kernel is faster.</x:v>
+      </x:c>
+      <x:c r="B21" s="666"/>
+      <x:c r="C21" s="666"/>
+      <x:c r="D21" s="666"/>
+      <x:c r="E21" s="666"/>
+      <x:c r="F21" s="666"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
+    <x:mergeCell ref="A15:B15"/>
+    <x:mergeCell ref="A21:F21"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="D5:D12">
+    <x:cfRule type="cellIs" dxfId="7" priority="1" operator="greaterThanOrEqual">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="8" priority="2" operator="lessThan">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>

</xml_diff>

<commit_message>
docs: update hybrid sparse performance workbook
Refresh the tuned-dispatch sheet with the final eight-shape H20 measurements and selected kernels. The workbook passed formula-error inspection and visual render verification before replacement.
</commit_message>
<xml_diff>
--- a/docs/hybrid_sparse_performance.xlsx
+++ b/docs/hybrid_sparse_performance.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R5eb3555ca3b942d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R4fbe53c6960741e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R8961f97deac04e8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="R619cc00686654058"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="Rffe933a0d411493a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="Rf64f8cf01e624509"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="R1aaaaf7266044af4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register Realloc" sheetId="8" r:id="R97db8ba5eea34c30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Iterations" sheetId="9" r:id="Rb921ee5a6080407b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output Tile Reuse" sheetId="10" r:id="R9ccbbe2c36804bbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Specified Shapes" sheetId="11" r:id="R21cc14967f8e46ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuned Dispatch" sheetId="12" r:id="Rcaddb03379554db6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="Radf88247ea634bb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R3e8d66059f7a40c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R27ba814d69b3493b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="R449e4596194542b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="R47f2af311a5c46b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="Rf660b3c357524fd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="R03d73db18b7c48e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register Realloc" sheetId="8" r:id="Rca5900293eb04b18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Iterations" sheetId="9" r:id="Rfe336d99dd0144f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output Tile Reuse" sheetId="10" r:id="R459819cea6494ebd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Specified Shapes" sheetId="11" r:id="Re593b7346bca40a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuned Dispatch" sheetId="12" r:id="Re1d4deb8fab44e13"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2576,7 +2576,7 @@
         <x:color rgb="FF176B3A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD7F0DF"/>
         </x:patternFill>
       </x:fill>
@@ -2586,7 +2586,7 @@
         <x:color rgb="FFA93333"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFADADA"/>
         </x:patternFill>
       </x:fill>
@@ -4030,7 +4030,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="631" t="str">
-        <x:v>NVIDIA H20 | BF16 input/output | FP32 accumulation | 25% hybrid sparsity | 7 paired repeats x 300 | commit 76e5d8b</x:v>
+        <x:v>NVIDIA H20 | BF16 input/output | FP32 accumulation | 25% hybrid sparsity | 7 paired repeats x 300 | commit 0cccd83</x:v>
       </x:c>
       <x:c r="B2" s="631"/>
       <x:c r="C2" s="631"/>
@@ -4063,14 +4063,14 @@
         <x:v>128 x 1408 x 2048</x:v>
       </x:c>
       <x:c r="B5" s="647" t="n">
-        <x:v>8.87</x:v>
+        <x:v>8.871</x:v>
       </x:c>
       <x:c r="C5" s="647" t="n">
-        <x:v>9.54</x:v>
+        <x:v>9.512</x:v>
       </x:c>
       <x:c r="D5" s="650" t="n">
         <x:f>C5/B5</x:f>
-        <x:v>1.0755355129650508</x:v>
+        <x:v>1.0722579190621124</x:v>
       </x:c>
       <x:c r="E5" s="653" t="n">
         <x:v>7</x:v>
@@ -4084,20 +4084,20 @@
         <x:v>128 x 2048 x 1408</x:v>
       </x:c>
       <x:c r="B6" s="648" t="n">
-        <x:v>8.04</x:v>
+        <x:v>7.272</x:v>
       </x:c>
       <x:c r="C6" s="648" t="n">
-        <x:v>8.59</x:v>
+        <x:v>8.535</x:v>
       </x:c>
       <x:c r="D6" s="651" t="n">
         <x:f>C6/B6</x:f>
-        <x:v>1.068407960199005</x:v>
+        <x:v>1.1736798679867986</x:v>
       </x:c>
       <x:c r="E6" s="654" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F6" s="642" t="str">
-        <x:v>output64 fixed-shape stage7</x:v>
+        <x:v>output64 constexpr branch group</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
@@ -4105,14 +4105,14 @@
         <x:v>256 x 1408 x 2048</x:v>
       </x:c>
       <x:c r="B7" s="648" t="n">
-        <x:v>12.55</x:v>
+        <x:v>12.549</x:v>
       </x:c>
       <x:c r="C7" s="648" t="n">
-        <x:v>13.75</x:v>
+        <x:v>13.763000000000002</x:v>
       </x:c>
       <x:c r="D7" s="651" t="n">
         <x:f>C7/B7</x:f>
-        <x:v>1.095617529880478</x:v>
+        <x:v>1.096740776157463</x:v>
       </x:c>
       <x:c r="E7" s="654" t="n">
         <x:v>7</x:v>
@@ -4126,20 +4126,20 @@
         <x:v>256 x 2048 x 1408</x:v>
       </x:c>
       <x:c r="B8" s="648" t="n">
-        <x:v>12.26</x:v>
+        <x:v>11.776</x:v>
       </x:c>
       <x:c r="C8" s="648" t="n">
-        <x:v>13.21</x:v>
+        <x:v>13.205999999999998</x:v>
       </x:c>
       <x:c r="D8" s="651" t="n">
         <x:f>C8/B8</x:f>
-        <x:v>1.0774877650897228</x:v>
+        <x:v>1.1214334239130432</x:v>
       </x:c>
       <x:c r="E8" s="654" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F8" s="642" t="str">
-        <x:v>output128 group-stage descriptor reuse</x:v>
+        <x:v>output128 fixed-shape stage4 async group2</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
@@ -4147,14 +4147,14 @@
         <x:v>512 x 1408 x 2048</x:v>
       </x:c>
       <x:c r="B9" s="648" t="n">
-        <x:v>21.89</x:v>
+        <x:v>21.892</x:v>
       </x:c>
       <x:c r="C9" s="648" t="n">
-        <x:v>25.2</x:v>
+        <x:v>25.207</x:v>
       </x:c>
       <x:c r="D9" s="651" t="n">
         <x:f>C9/B9</x:f>
-        <x:v>1.1512105984467793</x:v>
+        <x:v>1.1514251781472684</x:v>
       </x:c>
       <x:c r="E9" s="654" t="n">
         <x:v>7</x:v>
@@ -4168,14 +4168,14 @@
         <x:v>512 x 2048 x 1408</x:v>
       </x:c>
       <x:c r="B10" s="648" t="n">
-        <x:v>22.86</x:v>
+        <x:v>22.87</x:v>
       </x:c>
       <x:c r="C10" s="648" t="n">
-        <x:v>24.54</x:v>
+        <x:v>24.546</x:v>
       </x:c>
       <x:c r="D10" s="651" t="n">
         <x:f>C10/B10</x:f>
-        <x:v>1.073490813648294</x:v>
+        <x:v>1.0732837778749453</x:v>
       </x:c>
       <x:c r="E10" s="654" t="n">
         <x:v>7</x:v>
@@ -4189,14 +4189,14 @@
         <x:v>1024 x 1408 x 2048</x:v>
       </x:c>
       <x:c r="B11" s="648" t="n">
-        <x:v>41.98</x:v>
+        <x:v>41.945</x:v>
       </x:c>
       <x:c r="C11" s="648" t="n">
-        <x:v>48.45</x:v>
+        <x:v>48.463</x:v>
       </x:c>
       <x:c r="D11" s="651" t="n">
         <x:f>C11/B11</x:f>
-        <x:v>1.1541210100047643</x:v>
+        <x:v>1.1553939682918106</x:v>
       </x:c>
       <x:c r="E11" s="654" t="n">
         <x:v>7</x:v>
@@ -4210,14 +4210,14 @@
         <x:v>1024 x 2048 x 1408</x:v>
       </x:c>
       <x:c r="B12" s="649" t="n">
-        <x:v>43.42</x:v>
+        <x:v>43.411</x:v>
       </x:c>
       <x:c r="C12" s="649" t="n">
-        <x:v>47.33</x:v>
+        <x:v>47.295</x:v>
       </x:c>
       <x:c r="D12" s="652" t="n">
         <x:f>C12/B12</x:f>
-        <x:v>1.0900506678949793</x:v>
+        <x:v>1.089470410725392</x:v>
       </x:c>
       <x:c r="E12" s="655" t="n">
         <x:v>7</x:v>
@@ -4247,7 +4247,7 @@
       </x:c>
       <x:c r="B17" s="662" t="n">
         <x:f>MAX(D5:D12)</x:f>
-        <x:v>1.1541210100047643</x:v>
+        <x:v>1.1736798679867986</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -4256,7 +4256,7 @@
       </x:c>
       <x:c r="B18" s="663" t="n">
         <x:f>MAX(B5:B12)</x:f>
-        <x:v>43.42</x:v>
+        <x:v>43.411</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="34" customHeight="1">

</xml_diff>

<commit_message>
docs: record all dispatched shape benchmarks
Update the tuned-dispatch sheet with all twelve H20 shapes, including shape-specific kernels and generic fallbacks. The workbook passed formula-error inspection and visual render verification.
</commit_message>
<xml_diff>
--- a/docs/hybrid_sparse_performance.xlsx
+++ b/docs/hybrid_sparse_performance.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="Radf88247ea634bb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R3e8d66059f7a40c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R27ba814d69b3493b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="R449e4596194542b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="R47f2af311a5c46b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="Rf660b3c357524fd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="R03d73db18b7c48e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register Realloc" sheetId="8" r:id="Rca5900293eb04b18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Iterations" sheetId="9" r:id="Rfe336d99dd0144f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output Tile Reuse" sheetId="10" r:id="R459819cea6494ebd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Specified Shapes" sheetId="11" r:id="Re593b7346bca40a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuned Dispatch" sheetId="12" r:id="Re1d4deb8fab44e13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="Re17f188a91b34f0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R7ee36ebe7d1c4bb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R84547bdb35b24afb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="Rc9b60360a9994e25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="Re61b2817b13d46c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="R5f12d60a6d474897"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="R21206ba5944b4dcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register Realloc" sheetId="8" r:id="Rdf4cec4540394fb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Iterations" sheetId="9" r:id="Rcb0fb2b176a8434c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output Tile Reuse" sheetId="10" r:id="R3fdc61cd198b4ee8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Specified Shapes" sheetId="11" r:id="R6745efc7f3a84061"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuned Dispatch" sheetId="12" r:id="R42b42b5d9e9c49d3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -36,7 +36,7 @@
     <x:numFmt numFmtId="208" formatCode="#,##0"/>
     <x:numFmt numFmtId="209" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="56">
+  <x:fonts count="62">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -350,8 +350,41 @@
       <x:color rgb="FF526174"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="12"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF5D6B7E"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="55">
+  <x:fills count="59">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -621,6 +654,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF4F7FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF203764"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEFF3F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F7FA"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -1004,7 +1057,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="667">
+  <x:cellXfs count="706">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2492,11 +2545,84 @@
     <x:xf numFmtId="0" fontId="55" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="35" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="54" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="54" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="56" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="57" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="56" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="56" fillId="55" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="56" fillId="55" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="57" fillId="55" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="56" fillId="55" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="56" fillId="55" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="56" fillId="55" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="57" fillId="55" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="56" fillId="55" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="56" fillId="55" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="57" fillId="55" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="56" fillId="55" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="56" fillId="55" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="56" fillId="55" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="56" fillId="55" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="56" fillId="55" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="56" fillId="55" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="56" fillId="55" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="55" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="56" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="58" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="59" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="60" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="56" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="58" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="56" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="58" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="56" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="61" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="9">
+  <x:dxfs count="11">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -2588,6 +2714,26 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFFADADA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF176B3A"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFD7F0DF"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FFA33A32"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF8D7DA"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -4030,7 +4176,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="631" t="str">
-        <x:v>NVIDIA H20 | BF16 input/output | FP32 accumulation | 25% hybrid sparsity | 7 paired repeats x 300 | commit 0cccd83</x:v>
+        <x:v>NVIDIA H20 | BF16 input/output | FP32 accumulation | 25% hybrid sparsity | 7 paired repeats x 300 | commit f50ec26</x:v>
       </x:c>
       <x:c r="B2" s="631"/>
       <x:c r="C2" s="631"/>
@@ -4063,14 +4209,14 @@
         <x:v>128 x 1408 x 2048</x:v>
       </x:c>
       <x:c r="B5" s="647" t="n">
-        <x:v>8.871</x:v>
+        <x:v>8.872</x:v>
       </x:c>
       <x:c r="C5" s="647" t="n">
-        <x:v>9.512</x:v>
+        <x:v>9.513</x:v>
       </x:c>
       <x:c r="D5" s="650" t="n">
         <x:f>C5/B5</x:f>
-        <x:v>1.0722579190621124</x:v>
+        <x:v>1.0722497745716861</x:v>
       </x:c>
       <x:c r="E5" s="653" t="n">
         <x:v>7</x:v>
@@ -4084,14 +4230,14 @@
         <x:v>128 x 2048 x 1408</x:v>
       </x:c>
       <x:c r="B6" s="648" t="n">
-        <x:v>7.272</x:v>
+        <x:v>7.275000000000001</x:v>
       </x:c>
       <x:c r="C6" s="648" t="n">
-        <x:v>8.535</x:v>
+        <x:v>8.556</x:v>
       </x:c>
       <x:c r="D6" s="651" t="n">
         <x:f>C6/B6</x:f>
-        <x:v>1.1736798679867986</x:v>
+        <x:v>1.176082474226804</x:v>
       </x:c>
       <x:c r="E6" s="654" t="n">
         <x:v>7</x:v>
@@ -4105,14 +4251,14 @@
         <x:v>256 x 1408 x 2048</x:v>
       </x:c>
       <x:c r="B7" s="648" t="n">
-        <x:v>12.549</x:v>
+        <x:v>12.558</x:v>
       </x:c>
       <x:c r="C7" s="648" t="n">
-        <x:v>13.763000000000002</x:v>
+        <x:v>13.712999999999997</x:v>
       </x:c>
       <x:c r="D7" s="651" t="n">
         <x:f>C7/B7</x:f>
-        <x:v>1.096740776157463</x:v>
+        <x:v>1.091973244147157</x:v>
       </x:c>
       <x:c r="E7" s="654" t="n">
         <x:v>7</x:v>
@@ -4126,14 +4272,14 @@
         <x:v>256 x 2048 x 1408</x:v>
       </x:c>
       <x:c r="B8" s="648" t="n">
-        <x:v>11.776</x:v>
+        <x:v>11.764</x:v>
       </x:c>
       <x:c r="C8" s="648" t="n">
-        <x:v>13.205999999999998</x:v>
+        <x:v>13.227999999999998</x:v>
       </x:c>
       <x:c r="D8" s="651" t="n">
         <x:f>C8/B8</x:f>
-        <x:v>1.1214334239130432</x:v>
+        <x:v>1.1244474668480107</x:v>
       </x:c>
       <x:c r="E8" s="654" t="n">
         <x:v>7</x:v>
@@ -4147,14 +4293,14 @@
         <x:v>512 x 1408 x 2048</x:v>
       </x:c>
       <x:c r="B9" s="648" t="n">
-        <x:v>21.892</x:v>
+        <x:v>21.901</x:v>
       </x:c>
       <x:c r="C9" s="648" t="n">
-        <x:v>25.207</x:v>
+        <x:v>25.205</x:v>
       </x:c>
       <x:c r="D9" s="651" t="n">
         <x:f>C9/B9</x:f>
-        <x:v>1.1514251781472684</x:v>
+        <x:v>1.150860691292635</x:v>
       </x:c>
       <x:c r="E9" s="654" t="n">
         <x:v>7</x:v>
@@ -4168,14 +4314,14 @@
         <x:v>512 x 2048 x 1408</x:v>
       </x:c>
       <x:c r="B10" s="648" t="n">
-        <x:v>22.87</x:v>
+        <x:v>22.88</x:v>
       </x:c>
       <x:c r="C10" s="648" t="n">
-        <x:v>24.546</x:v>
+        <x:v>24.553</x:v>
       </x:c>
       <x:c r="D10" s="651" t="n">
         <x:f>C10/B10</x:f>
-        <x:v>1.0732837778749453</x:v>
+        <x:v>1.0731206293706295</x:v>
       </x:c>
       <x:c r="E10" s="654" t="n">
         <x:v>7</x:v>
@@ -4189,14 +4335,14 @@
         <x:v>1024 x 1408 x 2048</x:v>
       </x:c>
       <x:c r="B11" s="648" t="n">
-        <x:v>41.945</x:v>
+        <x:v>42.005</x:v>
       </x:c>
       <x:c r="C11" s="648" t="n">
-        <x:v>48.463</x:v>
+        <x:v>48.521</x:v>
       </x:c>
       <x:c r="D11" s="651" t="n">
         <x:f>C11/B11</x:f>
-        <x:v>1.1553939682918106</x:v>
+        <x:v>1.1551243899535768</x:v>
       </x:c>
       <x:c r="E11" s="654" t="n">
         <x:v>7</x:v>
@@ -4210,14 +4356,14 @@
         <x:v>1024 x 2048 x 1408</x:v>
       </x:c>
       <x:c r="B12" s="649" t="n">
-        <x:v>43.411</x:v>
+        <x:v>43.402</x:v>
       </x:c>
       <x:c r="C12" s="649" t="n">
-        <x:v>47.295</x:v>
+        <x:v>47.239</x:v>
       </x:c>
       <x:c r="D12" s="652" t="n">
         <x:f>C12/B12</x:f>
-        <x:v>1.089470410725392</x:v>
+        <x:v>1.088406064236671</x:v>
       </x:c>
       <x:c r="E12" s="655" t="n">
         <x:v>7</x:v>
@@ -4226,61 +4372,177 @@
         <x:v>output96 baseline group-stage</x:v>
       </x:c>
     </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="674" t="str">
+        <x:v>2048 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B13" s="682" t="n">
+        <x:v>95.629</x:v>
+      </x:c>
+      <x:c r="C13" s="682" t="n">
+        <x:v>94.612</x:v>
+      </x:c>
+      <x:c r="D13" s="686" t="n">
+        <x:f>C13/B13</x:f>
+        <x:v>0.9893651507387925</x:v>
+      </x:c>
+      <x:c r="E13" s="690" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F13" s="674" t="str">
+        <x:v>generic output64 group-stage fallback</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="675" t="str">
+        <x:v>2048 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B14" s="681" t="n">
+        <x:v>94.211</x:v>
+      </x:c>
+      <x:c r="C14" s="681" t="n">
+        <x:v>92.253</x:v>
+      </x:c>
+      <x:c r="D14" s="687" t="n">
+        <x:f>C14/B14</x:f>
+        <x:v>0.9792168642727495</x:v>
+      </x:c>
+      <x:c r="E14" s="677" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F14" s="675" t="str">
+        <x:v>generic output64 group-stage fallback</x:v>
+      </x:c>
+    </x:row>
     <x:row r="15" ht="24" customHeight="1">
-      <x:c r="A15" s="656" t="str">
+      <x:c r="A15" s="676" t="str">
+        <x:v>4096 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="B15" s="683" t="n">
+        <x:v>180.242</x:v>
+      </x:c>
+      <x:c r="C15" s="681" t="n">
+        <x:v>182.627</x:v>
+      </x:c>
+      <x:c r="D15" s="687" t="n">
+        <x:f>C15/B15</x:f>
+        <x:v>1.0132322100287392</x:v>
+      </x:c>
+      <x:c r="E15" s="677" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F15" s="675" t="str">
+        <x:v>generic output64 group-stage fallback</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="675" t="str">
+        <x:v>4096 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="B16" s="681" t="n">
+        <x:v>180.255</x:v>
+      </x:c>
+      <x:c r="C16" s="681" t="n">
+        <x:v>181.732</x:v>
+      </x:c>
+      <x:c r="D16" s="687" t="n">
+        <x:f>C16/B16</x:f>
+        <x:v>1.008193947463316</x:v>
+      </x:c>
+      <x:c r="E16" s="677" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F16" s="675" t="str">
+        <x:v>generic output64 group-stage fallback</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="658"/>
+      <x:c r="B17" s="662"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="658"/>
+      <x:c r="B18" s="663"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="692" t="str">
         <x:v>Summary</x:v>
       </x:c>
-      <x:c r="B15" s="656"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="658" t="str">
+      <x:c r="B19" s="692"/>
+      <x:c r="C19"/>
+      <x:c r="D19"/>
+      <x:c r="E19"/>
+      <x:c r="F19"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="697" t="str">
         <x:v>Shapes faster than DeepGEMM</x:v>
       </x:c>
-      <x:c r="B16" s="661" t="n">
-        <x:f>COUNTIF(D5:D12,"&gt;1")</x:f>
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="658" t="str">
+      <x:c r="B20" s="701" t="n">
+        <x:f>COUNTIF(D5:D16,"&gt;1")</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C20"/>
+      <x:c r="D20"/>
+      <x:c r="E20"/>
+      <x:c r="F20"/>
+    </x:row>
+    <x:row r="21" ht="34" customHeight="1">
+      <x:c r="A21" s="698" t="str">
         <x:v>Best speedup</x:v>
       </x:c>
-      <x:c r="B17" s="662" t="n">
-        <x:f>MAX(D5:D12)</x:f>
-        <x:v>1.1736798679867986</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="658" t="str">
-        <x:v>Slowest tuned latency</x:v>
-      </x:c>
-      <x:c r="B18" s="663" t="n">
-        <x:f>MAX(B5:B12)</x:f>
-        <x:v>43.411</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="34" customHeight="1">
-      <x:c r="A21" s="666" t="str">
-        <x:v>Speedup is DeepGEMM latency divided by tuned total latency. Values above 1.0x mean the hybrid sparse kernel is faster.</x:v>
-      </x:c>
-      <x:c r="B21" s="666"/>
+      <x:c r="B21" s="702" t="n">
+        <x:f>MAX(D5:D16)</x:f>
+        <x:v>1.176082474226804</x:v>
+      </x:c>
       <x:c r="C21" s="666"/>
       <x:c r="D21" s="666"/>
       <x:c r="E21" s="666"/>
       <x:c r="F21" s="666"/>
     </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="697" t="str">
+        <x:v>Slowest tuned latency</x:v>
+      </x:c>
+      <x:c r="B22" s="703" t="n">
+        <x:f>MAX(B5:B16)</x:f>
+        <x:v>180.255</x:v>
+      </x:c>
+      <x:c r="C22"/>
+      <x:c r="D22"/>
+      <x:c r="E22"/>
+      <x:c r="F22"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="705" t="str">
+        <x:v>Speedup is DeepGEMM latency divided by tuned total latency. Values above 1.0x mean the hybrid sparse kernel is faster.</x:v>
+      </x:c>
+      <x:c r="B25" s="705"/>
+      <x:c r="C25" s="705"/>
+      <x:c r="D25" s="705"/>
+      <x:c r="E25" s="705"/>
+      <x:c r="F25" s="705"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
     <x:mergeCell ref="A2:F2"/>
-    <x:mergeCell ref="A15:B15"/>
-    <x:mergeCell ref="A21:F21"/>
+    <x:mergeCell ref="A19:B19"/>
+    <x:mergeCell ref="A25:F25"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="D5:D12">
     <x:cfRule type="cellIs" dxfId="7" priority="1" operator="greaterThanOrEqual">
       <x:formula>1</x:formula>
     </x:cfRule>
     <x:cfRule type="cellIs" dxfId="8" priority="2" operator="lessThan">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="D13:D16">
+    <x:cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThanOrEqual">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="10" priority="4" operator="lessThan">
       <x:formula>1</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>

</xml_diff>

<commit_message>
docs: record best kernel per hybrid shape
Update the tuned-dispatch sheet with the validated lowest-latency kernel selected independently for every benchmark shape. All twelve H20 shapes passed correctness checks and outperformed DeepGEMM.
</commit_message>
<xml_diff>
--- a/docs/hybrid_sparse_performance.xlsx
+++ b/docs/hybrid_sparse_performance.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="Re17f188a91b34f0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R7ee36ebe7d1c4bb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R84547bdb35b24afb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="Rc9b60360a9994e25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="Re61b2817b13d46c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="R5f12d60a6d474897"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="R21206ba5944b4dcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register Realloc" sheetId="8" r:id="Rdf4cec4540394fb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Iterations" sheetId="9" r:id="Rcb0fb2b176a8434c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output Tile Reuse" sheetId="10" r:id="R3fdc61cd198b4ee8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Specified Shapes" sheetId="11" r:id="R6745efc7f3a84061"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuned Dispatch" sheetId="12" r:id="R42b42b5d9e9c49d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R577934a1caa24654"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R08cdc903af464269"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R7fdaa16ea8194c4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="R25e28e470e2c47b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="R6f31603832c04a8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="R822059873e164e91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="R8c6e6238d7db4d78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register Realloc" sheetId="8" r:id="Re1e10b667594446a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Iterations" sheetId="9" r:id="R58b36bf393e9434b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output Tile Reuse" sheetId="10" r:id="R95d352f1da254afd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Specified Shapes" sheetId="11" r:id="R59dc77ecf39b4dca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuned Dispatch" sheetId="12" r:id="R7866dde075154200"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2722,7 +2722,7 @@
         <x:color rgb="FF176B3A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD7F0DF"/>
         </x:patternFill>
       </x:fill>
@@ -2732,7 +2732,7 @@
         <x:color rgb="FFA33A32"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF8D7DA"/>
         </x:patternFill>
       </x:fill>
@@ -4176,7 +4176,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="631" t="str">
-        <x:v>NVIDIA H20 | BF16 input/output | FP32 accumulation | 25% hybrid sparsity | 7 paired repeats x 300 | commit f50ec26</x:v>
+        <x:v>NVIDIA H20 | BF16 input/output | FP32 accumulation | 25% hybrid sparsity | per-shape best dispatch | 7 paired repeats x 300 | commit e2eb54f</x:v>
       </x:c>
       <x:c r="B2" s="631"/>
       <x:c r="C2" s="631"/>
@@ -4209,14 +4209,14 @@
         <x:v>128 x 1408 x 2048</x:v>
       </x:c>
       <x:c r="B5" s="647" t="n">
-        <x:v>8.872</x:v>
+        <x:v>8.879</x:v>
       </x:c>
       <x:c r="C5" s="647" t="n">
-        <x:v>9.513</x:v>
+        <x:v>9.524</x:v>
       </x:c>
       <x:c r="D5" s="650" t="n">
         <x:f>C5/B5</x:f>
-        <x:v>1.0722497745716861</x:v>
+        <x:v>1.0726433156887036</x:v>
       </x:c>
       <x:c r="E5" s="653" t="n">
         <x:v>7</x:v>
@@ -4230,14 +4230,14 @@
         <x:v>128 x 2048 x 1408</x:v>
       </x:c>
       <x:c r="B6" s="648" t="n">
-        <x:v>7.275000000000001</x:v>
+        <x:v>7.268</x:v>
       </x:c>
       <x:c r="C6" s="648" t="n">
-        <x:v>8.556</x:v>
+        <x:v>8.593</x:v>
       </x:c>
       <x:c r="D6" s="651" t="n">
         <x:f>C6/B6</x:f>
-        <x:v>1.176082474226804</x:v>
+        <x:v>1.1823059988992846</x:v>
       </x:c>
       <x:c r="E6" s="654" t="n">
         <x:v>7</x:v>
@@ -4251,14 +4251,14 @@
         <x:v>256 x 1408 x 2048</x:v>
       </x:c>
       <x:c r="B7" s="648" t="n">
-        <x:v>12.558</x:v>
+        <x:v>12.548</x:v>
       </x:c>
       <x:c r="C7" s="648" t="n">
-        <x:v>13.712999999999997</x:v>
+        <x:v>13.765</x:v>
       </x:c>
       <x:c r="D7" s="651" t="n">
         <x:f>C7/B7</x:f>
-        <x:v>1.091973244147157</x:v>
+        <x:v>1.0969875677398788</x:v>
       </x:c>
       <x:c r="E7" s="654" t="n">
         <x:v>7</x:v>
@@ -4272,14 +4272,14 @@
         <x:v>256 x 2048 x 1408</x:v>
       </x:c>
       <x:c r="B8" s="648" t="n">
-        <x:v>11.764</x:v>
+        <x:v>11.779</x:v>
       </x:c>
       <x:c r="C8" s="648" t="n">
-        <x:v>13.227999999999998</x:v>
+        <x:v>13.213</x:v>
       </x:c>
       <x:c r="D8" s="651" t="n">
         <x:f>C8/B8</x:f>
-        <x:v>1.1244474668480107</x:v>
+        <x:v>1.121742083368707</x:v>
       </x:c>
       <x:c r="E8" s="654" t="n">
         <x:v>7</x:v>
@@ -4293,14 +4293,14 @@
         <x:v>512 x 1408 x 2048</x:v>
       </x:c>
       <x:c r="B9" s="648" t="n">
-        <x:v>21.901</x:v>
+        <x:v>21.916</x:v>
       </x:c>
       <x:c r="C9" s="648" t="n">
-        <x:v>25.205</x:v>
+        <x:v>25.16</x:v>
       </x:c>
       <x:c r="D9" s="651" t="n">
         <x:f>C9/B9</x:f>
-        <x:v>1.150860691292635</x:v>
+        <x:v>1.1480197116262092</x:v>
       </x:c>
       <x:c r="E9" s="654" t="n">
         <x:v>7</x:v>
@@ -4314,14 +4314,14 @@
         <x:v>512 x 2048 x 1408</x:v>
       </x:c>
       <x:c r="B10" s="648" t="n">
-        <x:v>22.88</x:v>
+        <x:v>22.886</x:v>
       </x:c>
       <x:c r="C10" s="648" t="n">
-        <x:v>24.553</x:v>
+        <x:v>24.535</x:v>
       </x:c>
       <x:c r="D10" s="651" t="n">
         <x:f>C10/B10</x:f>
-        <x:v>1.0731206293706295</x:v>
+        <x:v>1.0720527833610067</x:v>
       </x:c>
       <x:c r="E10" s="654" t="n">
         <x:v>7</x:v>
@@ -4335,14 +4335,14 @@
         <x:v>1024 x 1408 x 2048</x:v>
       </x:c>
       <x:c r="B11" s="648" t="n">
-        <x:v>42.005</x:v>
+        <x:v>41.971</x:v>
       </x:c>
       <x:c r="C11" s="648" t="n">
-        <x:v>48.521</x:v>
+        <x:v>48.515</x:v>
       </x:c>
       <x:c r="D11" s="651" t="n">
         <x:f>C11/B11</x:f>
-        <x:v>1.1551243899535768</x:v>
+        <x:v>1.1559171809106288</x:v>
       </x:c>
       <x:c r="E11" s="654" t="n">
         <x:v>7</x:v>
@@ -4356,14 +4356,14 @@
         <x:v>1024 x 2048 x 1408</x:v>
       </x:c>
       <x:c r="B12" s="649" t="n">
-        <x:v>43.402</x:v>
+        <x:v>43.393</x:v>
       </x:c>
       <x:c r="C12" s="649" t="n">
-        <x:v>47.239</x:v>
+        <x:v>47.341</x:v>
       </x:c>
       <x:c r="D12" s="652" t="n">
         <x:f>C12/B12</x:f>
-        <x:v>1.088406064236671</x:v>
+        <x:v>1.0909824165187934</x:v>
       </x:c>
       <x:c r="E12" s="655" t="n">
         <x:v>7</x:v>
@@ -4377,20 +4377,20 @@
         <x:v>2048 x 1408 x 2048</x:v>
       </x:c>
       <x:c r="B13" s="682" t="n">
-        <x:v>95.629</x:v>
+        <x:v>76.966</x:v>
       </x:c>
       <x:c r="C13" s="682" t="n">
-        <x:v>94.612</x:v>
+        <x:v>94.674</x:v>
       </x:c>
       <x:c r="D13" s="686" t="n">
         <x:f>C13/B13</x:f>
-        <x:v>0.9893651507387925</x:v>
+        <x:v>1.2300756178052648</x:v>
       </x:c>
       <x:c r="E13" s="690" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F13" s="674" t="str">
-        <x:v>generic output64 group-stage fallback</x:v>
+        <x:v>output128 stage-kind</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -4398,20 +4398,20 @@
         <x:v>2048 x 2048 x 1408</x:v>
       </x:c>
       <x:c r="B14" s="681" t="n">
-        <x:v>94.211</x:v>
+        <x:v>74.42</x:v>
       </x:c>
       <x:c r="C14" s="681" t="n">
-        <x:v>92.253</x:v>
+        <x:v>92.351</x:v>
       </x:c>
       <x:c r="D14" s="687" t="n">
         <x:f>C14/B14</x:f>
-        <x:v>0.9792168642727495</x:v>
+        <x:v>1.2409432948132222</x:v>
       </x:c>
       <x:c r="E14" s="677" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F14" s="675" t="str">
-        <x:v>generic output64 group-stage fallback</x:v>
+        <x:v>output128 stage-kind</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
@@ -4419,20 +4419,20 @@
         <x:v>4096 x 1408 x 2048</x:v>
       </x:c>
       <x:c r="B15" s="683" t="n">
-        <x:v>180.242</x:v>
+        <x:v>149.138</x:v>
       </x:c>
       <x:c r="C15" s="681" t="n">
-        <x:v>182.627</x:v>
+        <x:v>182.777</x:v>
       </x:c>
       <x:c r="D15" s="687" t="n">
         <x:f>C15/B15</x:f>
-        <x:v>1.0132322100287392</x:v>
+        <x:v>1.2255561962745911</x:v>
       </x:c>
       <x:c r="E15" s="677" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F15" s="675" t="str">
-        <x:v>generic output64 group-stage fallback</x:v>
+        <x:v>output128 stage-kind</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -4440,20 +4440,20 @@
         <x:v>4096 x 2048 x 1408</x:v>
       </x:c>
       <x:c r="B16" s="681" t="n">
-        <x:v>180.255</x:v>
+        <x:v>144.6</x:v>
       </x:c>
       <x:c r="C16" s="681" t="n">
-        <x:v>181.732</x:v>
+        <x:v>181.872</x:v>
       </x:c>
       <x:c r="D16" s="687" t="n">
         <x:f>C16/B16</x:f>
-        <x:v>1.008193947463316</x:v>
+        <x:v>1.2577593360995851</x:v>
       </x:c>
       <x:c r="E16" s="677" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F16" s="675" t="str">
-        <x:v>generic output64 group-stage fallback</x:v>
+        <x:v>output128 stage-kind</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -4480,7 +4480,7 @@
       </x:c>
       <x:c r="B20" s="701" t="n">
         <x:f>COUNTIF(D5:D16,"&gt;1")</x:f>
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C20"/>
       <x:c r="D20"/>
@@ -4493,7 +4493,7 @@
       </x:c>
       <x:c r="B21" s="702" t="n">
         <x:f>MAX(D5:D16)</x:f>
-        <x:v>1.176082474226804</x:v>
+        <x:v>1.2577593360995851</x:v>
       </x:c>
       <x:c r="C21" s="666"/>
       <x:c r="D21" s="666"/>
@@ -4506,7 +4506,7 @@
       </x:c>
       <x:c r="B22" s="703" t="n">
         <x:f>MAX(B5:B16)</x:f>
-        <x:v>180.255</x:v>
+        <x:v>149.138</x:v>
       </x:c>
       <x:c r="C22"/>
       <x:c r="D22"/>
@@ -4515,7 +4515,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="705" t="str">
-        <x:v>Speedup is DeepGEMM latency divided by tuned total latency. Values above 1.0x mean the hybrid sparse kernel is faster.</x:v>
+        <x:v>Interpretation: each supported shape dispatches to its lowest-latency validated kernel; no large-M generic fallback is used.</x:v>
       </x:c>
       <x:c r="B25" s="705"/>
       <x:c r="C25" s="705"/>

</xml_diff>

<commit_message>
docs: add grouped expert scaling results
Add E32 and E64 contiguous and masked grouped GEMM measurements using the best dispatched kernel for each shape. The workbook formulas and rendered layout were validated locally.
</commit_message>
<xml_diff>
--- a/docs/hybrid_sparse_performance.xlsx
+++ b/docs/hybrid_sparse_performance.xlsx
@@ -2,18 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R577934a1caa24654"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R08cdc903af464269"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R7fdaa16ea8194c4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="R25e28e470e2c47b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="R6f31603832c04a8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="R822059873e164e91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="R8c6e6238d7db4d78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register Realloc" sheetId="8" r:id="Re1e10b667594446a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Iterations" sheetId="9" r:id="R58b36bf393e9434b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output Tile Reuse" sheetId="10" r:id="R95d352f1da254afd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Specified Shapes" sheetId="11" r:id="R59dc77ecf39b4dca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuned Dispatch" sheetId="12" r:id="R7866dde075154200"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="1" r:id="R2ac6e7c8dac0468b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy" sheetId="2" r:id="R24be52d7fa6c41f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistent LaneReady" sheetId="3" r:id="R3854ac69b6034ff3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cuBLAS Baseline" sheetId="4" r:id="R17b5426181de47a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="128x32 Stage3" sheetId="5" r:id="R5556738061c7489a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merge K2" sheetId="6" r:id="R83932728bde9483c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TMA Pipeline Stages" sheetId="7" r:id="R15188205ec784a69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register Realloc" sheetId="8" r:id="Rbbae617535cf43c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Iterations" sheetId="9" r:id="Rf979a54f89c547cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output Tile Reuse" sheetId="10" r:id="R14fc54e5fd7d40af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Specified Shapes" sheetId="11" r:id="R68ce33e8ec1d485b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuned Dispatch" sheetId="12" r:id="R9c1cf84d70274491"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grouped GEMM" sheetId="13" r:id="R2b6a08b12658444a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grouped E32-E64" sheetId="14" r:id="Rbbec5f9f4f6d480c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24,7 +26,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="10">
+  <x:numFmts count="11">
     <x:numFmt numFmtId="200" formatCode="0.00"/>
     <x:numFmt numFmtId="201" formatCode="0.000x"/>
     <x:numFmt numFmtId="202" formatCode="0%"/>
@@ -35,8 +37,9 @@
     <x:numFmt numFmtId="207" formatCode="0.0%"/>
     <x:numFmt numFmtId="208" formatCode="#,##0"/>
     <x:numFmt numFmtId="209" formatCode="0"/>
+    <x:numFmt numFmtId="210" formatCode="0.0"/>
   </x:numFmts>
-  <x:fonts count="62">
+  <x:fonts count="69">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -383,8 +386,48 @@
       <x:color rgb="FF5D6B7E"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF0F4C6E"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF46566E"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="22"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF0F4C6E"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF46566E"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="22"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos Display"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="59">
+  <x:fills count="76">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -676,8 +719,93 @@
         <x:fgColor rgb="FFF5F7FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1B2D5C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEEF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF24466F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F8FC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F7FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1B2D5C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEEF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF24466F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F7FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1B2D5C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEEF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF24466F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F7FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1B2D5C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEEF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF24466F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F7FA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="44">
+  <x:borders count="46">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -1053,11 +1181,21 @@
         <x:color rgb="FFD8E1EC"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:bottom style="medium">
+        <x:color rgb="FF18324F"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7E2EE"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="706">
+  <x:cellXfs count="844">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2618,11 +2756,337 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="61" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="60" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="62" fillId="60" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="62" fillId="60" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="61" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="61" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="61" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="61" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="62" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="62" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="63" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="63" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="63" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="62" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="62" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="62" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="64" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="65" fillId="60" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="42" fillId="61" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="62" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="62" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="41" fillId="62" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="41" fillId="62" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="66" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="41" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="41" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="41" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="41" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="41" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="41" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="41" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="41" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="67" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="68" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="62" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="62" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="66" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="66" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="66" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="66" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="67" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="63" fillId="67" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="63" fillId="67" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="63" fillId="67" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="64" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="65" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="66" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="42" fillId="66" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="67" fillId="67" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="68" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="41" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="41" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="62" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="62" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="70" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="70" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="70" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="70" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="63" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="63" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="63" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="64" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="65" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="66" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="42" fillId="70" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="67" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="68" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="62" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="62" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="74" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="74" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="74" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="74" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="63" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="63" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="63" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="64" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="65" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="66" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="42" fillId="74" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="67" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="68" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="11">
+  <x:dxfs count="31">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -2734,6 +3198,215 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFF8D7DA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8B2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8B2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8B2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8B2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8B2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8B2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE8B2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE8B2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE8B2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE8B2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -4550,6 +5223,2797 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="38" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="13" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="13" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="38" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="38" customHeight="1">
+      <x:c r="A1" s="817" t="str">
+        <x:v>Grouped GEMM Best-Dispatch Performance</x:v>
+      </x:c>
+      <x:c r="B1" s="817"/>
+      <x:c r="C1" s="817"/>
+      <x:c r="D1" s="817"/>
+      <x:c r="E1" s="817"/>
+      <x:c r="F1" s="817"/>
+      <x:c r="G1" s="817"/>
+      <x:c r="H1" s="817"/>
+      <x:c r="I1" s="817"/>
+      <x:c r="J1"/>
+      <x:c r="K1"/>
+    </x:row>
+    <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="813" t="str">
+        <x:v>NVIDIA H20 | BF16 input/output | FP32 accumulation | 64 x 64 weight blocks | 25% sparsity | Num Experts = 8 | 100 timing runs | L2 flush disabled</x:v>
+      </x:c>
+      <x:c r="B2" s="813"/>
+      <x:c r="C2" s="813"/>
+      <x:c r="D2" s="813"/>
+      <x:c r="E2" s="813"/>
+      <x:c r="F2" s="813"/>
+      <x:c r="G2" s="813"/>
+      <x:c r="H2" s="813"/>
+      <x:c r="I2" s="813"/>
+      <x:c r="J2"/>
+      <x:c r="K2"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="442"/>
+      <x:c r="B3" s="442"/>
+      <x:c r="C3" s="442"/>
+      <x:c r="D3" s="442"/>
+      <x:c r="E3" s="442"/>
+      <x:c r="F3" s="442"/>
+      <x:c r="G3" s="442"/>
+      <x:c r="H3" s="442"/>
+      <x:c r="I3" s="442"/>
+      <x:c r="J3"/>
+      <x:c r="K3"/>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="814" t="str">
+        <x:v>Contiguous Grouped GEMM - Best Kernel per Shape</x:v>
+      </x:c>
+      <x:c r="B4" s="814"/>
+      <x:c r="C4" s="814"/>
+      <x:c r="D4" s="814"/>
+      <x:c r="E4" s="814"/>
+      <x:c r="F4" s="814"/>
+      <x:c r="G4" s="814"/>
+      <x:c r="H4" s="814"/>
+      <x:c r="I4" s="814"/>
+      <x:c r="J4"/>
+      <x:c r="K4"/>
+    </x:row>
+    <x:row r="5" ht="36" customHeight="1">
+      <x:c r="A5" s="815" t="str">
+        <x:v>Num Experts</x:v>
+      </x:c>
+      <x:c r="B5" s="815" t="str">
+        <x:v>Shape (Total M x N x K)</x:v>
+      </x:c>
+      <x:c r="C5" s="815" t="str">
+        <x:v>Tokens / Expert</x:v>
+      </x:c>
+      <x:c r="D5" s="815" t="str">
+        <x:v>Max M</x:v>
+      </x:c>
+      <x:c r="E5" s="815" t="str">
+        <x:v>Hybrid latency (us)</x:v>
+      </x:c>
+      <x:c r="F5" s="815" t="str">
+        <x:v>DeepGEMM latency (us)</x:v>
+      </x:c>
+      <x:c r="G5" s="815" t="str">
+        <x:v>Speedup</x:v>
+      </x:c>
+      <x:c r="H5" s="815" t="str">
+        <x:v>Best kernel version</x:v>
+      </x:c>
+      <x:c r="I5" s="815" t="str">
+        <x:v>Validation</x:v>
+      </x:c>
+      <x:c r="J5"/>
+      <x:c r="K5"/>
+    </x:row>
+    <x:row r="6" ht="28" customHeight="1">
+      <x:c r="A6" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B6" s="754" t="str">
+        <x:v>128 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C6" s="755" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D6" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E6" s="792" t="n">
+        <x:v>32.5</x:v>
+      </x:c>
+      <x:c r="F6" s="792" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="G6" s="757" t="n">
+        <x:f>F6/E6</x:f>
+        <x:v>1.5692307692307692</x:v>
+      </x:c>
+      <x:c r="H6" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I6" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J6"/>
+      <x:c r="K6"/>
+    </x:row>
+    <x:row r="7" ht="28" customHeight="1">
+      <x:c r="A7" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B7" s="754" t="str">
+        <x:v>256 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C7" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="D7" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E7" s="792" t="n">
+        <x:v>32.4</x:v>
+      </x:c>
+      <x:c r="F7" s="792" t="n">
+        <x:v>51.3</x:v>
+      </x:c>
+      <x:c r="G7" s="757" t="n">
+        <x:f>F7/E7</x:f>
+        <x:v>1.5833333333333333</x:v>
+      </x:c>
+      <x:c r="H7" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I7" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J7"/>
+      <x:c r="K7"/>
+    </x:row>
+    <x:row r="8" ht="28" customHeight="1">
+      <x:c r="A8" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B8" s="754" t="str">
+        <x:v>512 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C8" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D8" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E8" s="792" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F8" s="792" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="G8" s="757" t="n">
+        <x:f>F8/E8</x:f>
+        <x:v>1.59375</x:v>
+      </x:c>
+      <x:c r="H8" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I8" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J8"/>
+      <x:c r="K8"/>
+    </x:row>
+    <x:row r="9" ht="28" customHeight="1">
+      <x:c r="A9" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B9" s="754" t="str">
+        <x:v>1024 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C9" s="755" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="D9" s="755" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E9" s="792" t="n">
+        <x:v>51.4</x:v>
+      </x:c>
+      <x:c r="F9" s="792" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="G9" s="757" t="n">
+        <x:f>F9/E9</x:f>
+        <x:v>0.9922178988326849</x:v>
+      </x:c>
+      <x:c r="H9" s="754" t="str">
+        <x:v>output64x128_stage2_single_wg</x:v>
+      </x:c>
+      <x:c r="I9" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J9"/>
+      <x:c r="K9"/>
+    </x:row>
+    <x:row r="10" ht="28" customHeight="1">
+      <x:c r="A10" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B10" s="754" t="str">
+        <x:v>2048 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C10" s="755" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="D10" s="755" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="E10" s="792" t="n">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="F10" s="792" t="n">
+        <x:v>97.1</x:v>
+      </x:c>
+      <x:c r="G10" s="757" t="n">
+        <x:f>F10/E10</x:f>
+        <x:v>1.261038961038961</x:v>
+      </x:c>
+      <x:c r="H10" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I10" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J10"/>
+      <x:c r="K10"/>
+    </x:row>
+    <x:row r="11" ht="28" customHeight="1">
+      <x:c r="A11" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="754" t="str">
+        <x:v>4096 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C11" s="755" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="D11" s="755" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="E11" s="792" t="n">
+        <x:v>150.5</x:v>
+      </x:c>
+      <x:c r="F11" s="792" t="n">
+        <x:v>185.4</x:v>
+      </x:c>
+      <x:c r="G11" s="757" t="n">
+        <x:f>F11/E11</x:f>
+        <x:v>1.2318936877076412</x:v>
+      </x:c>
+      <x:c r="H11" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I11" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J11"/>
+      <x:c r="K11"/>
+    </x:row>
+    <x:row r="12" ht="28" customHeight="1">
+      <x:c r="A12" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B12" s="754" t="str">
+        <x:v>128 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C12" s="755" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D12" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E12" s="792" t="n">
+        <x:v>25.4</x:v>
+      </x:c>
+      <x:c r="F12" s="792" t="n">
+        <x:v>53.2</x:v>
+      </x:c>
+      <x:c r="G12" s="757" t="n">
+        <x:f>F12/E12</x:f>
+        <x:v>2.0944881889763782</x:v>
+      </x:c>
+      <x:c r="H12" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I12" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J12"/>
+      <x:c r="K12"/>
+    </x:row>
+    <x:row r="13" ht="28" customHeight="1">
+      <x:c r="A13" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B13" s="754" t="str">
+        <x:v>256 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C13" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="D13" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E13" s="792" t="n">
+        <x:v>25.2</x:v>
+      </x:c>
+      <x:c r="F13" s="792" t="n">
+        <x:v>53.2</x:v>
+      </x:c>
+      <x:c r="G13" s="757" t="n">
+        <x:f>F13/E13</x:f>
+        <x:v>2.111111111111111</x:v>
+      </x:c>
+      <x:c r="H13" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I13" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J13"/>
+      <x:c r="K13"/>
+    </x:row>
+    <x:row r="14" ht="28" customHeight="1">
+      <x:c r="A14" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B14" s="754" t="str">
+        <x:v>512 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C14" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D14" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E14" s="792" t="n">
+        <x:v>24.8</x:v>
+      </x:c>
+      <x:c r="F14" s="792" t="n">
+        <x:v>53.1</x:v>
+      </x:c>
+      <x:c r="G14" s="757" t="n">
+        <x:f>F14/E14</x:f>
+        <x:v>2.1411290322580645</x:v>
+      </x:c>
+      <x:c r="H14" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I14" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J14"/>
+      <x:c r="K14"/>
+    </x:row>
+    <x:row r="15" ht="28" customHeight="1">
+      <x:c r="A15" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B15" s="754" t="str">
+        <x:v>1024 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C15" s="755" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="D15" s="755" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E15" s="792" t="n">
+        <x:v>44.9</x:v>
+      </x:c>
+      <x:c r="F15" s="792" t="n">
+        <x:v>53.2</x:v>
+      </x:c>
+      <x:c r="G15" s="757" t="n">
+        <x:f>F15/E15</x:f>
+        <x:v>1.1848552338530067</x:v>
+      </x:c>
+      <x:c r="H15" s="754" t="str">
+        <x:v>output64x128_stage2_single_wg</x:v>
+      </x:c>
+      <x:c r="I15" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J15"/>
+      <x:c r="K15"/>
+    </x:row>
+    <x:row r="16" ht="28" customHeight="1">
+      <x:c r="A16" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B16" s="754" t="str">
+        <x:v>2048 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C16" s="755" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="D16" s="755" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="E16" s="792" t="n">
+        <x:v>76.3</x:v>
+      </x:c>
+      <x:c r="F16" s="792" t="n">
+        <x:v>100.8</x:v>
+      </x:c>
+      <x:c r="G16" s="757" t="n">
+        <x:f>F16/E16</x:f>
+        <x:v>1.3211009174311927</x:v>
+      </x:c>
+      <x:c r="H16" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I16" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J16"/>
+      <x:c r="K16"/>
+    </x:row>
+    <x:row r="17" ht="28" customHeight="1">
+      <x:c r="A17" s="761" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B17" s="760" t="str">
+        <x:v>4096 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C17" s="761" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="D17" s="761" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="E17" s="793" t="n">
+        <x:v>149.5</x:v>
+      </x:c>
+      <x:c r="F17" s="793" t="n">
+        <x:v>196.6</x:v>
+      </x:c>
+      <x:c r="G17" s="763" t="n">
+        <x:f>F17/E17</x:f>
+        <x:v>1.3150501672240802</x:v>
+      </x:c>
+      <x:c r="H17" s="760" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I17" s="761" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J17"/>
+      <x:c r="K17"/>
+    </x:row>
+    <x:row r="18" ht="32" customHeight="1">
+      <x:c r="A18" s="442"/>
+      <x:c r="B18" s="442"/>
+      <x:c r="C18" s="442"/>
+      <x:c r="D18" s="442"/>
+      <x:c r="E18" s="442"/>
+      <x:c r="F18" s="442"/>
+      <x:c r="G18" s="442"/>
+      <x:c r="H18" s="442"/>
+      <x:c r="I18" s="442"/>
+      <x:c r="J18"/>
+      <x:c r="K18"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="442"/>
+      <x:c r="B19" s="442"/>
+      <x:c r="C19" s="442"/>
+      <x:c r="D19" s="442"/>
+      <x:c r="E19" s="442"/>
+      <x:c r="F19" s="442"/>
+      <x:c r="G19" s="442"/>
+      <x:c r="H19" s="442"/>
+      <x:c r="I19" s="442"/>
+    </x:row>
+    <x:row r="20" ht="28" customHeight="1">
+      <x:c r="A20" s="814" t="str">
+        <x:v>Masked Grouped GEMM - Best Kernel per Shape</x:v>
+      </x:c>
+      <x:c r="B20" s="814"/>
+      <x:c r="C20" s="814"/>
+      <x:c r="D20" s="814"/>
+      <x:c r="E20" s="814"/>
+      <x:c r="F20" s="814"/>
+      <x:c r="G20" s="814"/>
+      <x:c r="H20" s="814"/>
+      <x:c r="I20" s="814"/>
+    </x:row>
+    <x:row r="21" ht="36" customHeight="1">
+      <x:c r="A21" s="815" t="str">
+        <x:v>Num Experts</x:v>
+      </x:c>
+      <x:c r="B21" s="815" t="str">
+        <x:v>Shape (Total M x N x K)</x:v>
+      </x:c>
+      <x:c r="C21" s="815" t="str">
+        <x:v>Tokens / Expert</x:v>
+      </x:c>
+      <x:c r="D21" s="815" t="str">
+        <x:v>Max M</x:v>
+      </x:c>
+      <x:c r="E21" s="815" t="str">
+        <x:v>Hybrid latency (us)</x:v>
+      </x:c>
+      <x:c r="F21" s="815" t="str">
+        <x:v>DeepGEMM latency (us)</x:v>
+      </x:c>
+      <x:c r="G21" s="815" t="str">
+        <x:v>Speedup</x:v>
+      </x:c>
+      <x:c r="H21" s="815" t="str">
+        <x:v>Best kernel version</x:v>
+      </x:c>
+      <x:c r="I21" s="815" t="str">
+        <x:v>Validation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="28" customHeight="1">
+      <x:c r="A22" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B22" s="754" t="str">
+        <x:v>128 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C22" s="755" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D22" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E22" s="792" t="n">
+        <x:v>18.9</x:v>
+      </x:c>
+      <x:c r="F22" s="792" t="n">
+        <x:v>27.8</x:v>
+      </x:c>
+      <x:c r="G22" s="757" t="n">
+        <x:f>F22/E22</x:f>
+        <x:v>1.4708994708994712</x:v>
+      </x:c>
+      <x:c r="H22" s="754" t="str">
+        <x:v>output32x64_stage4_adaptive</x:v>
+      </x:c>
+      <x:c r="I22" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="28" customHeight="1">
+      <x:c r="A23" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B23" s="754" t="str">
+        <x:v>256 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C23" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="D23" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E23" s="792" t="n">
+        <x:v>18.5</x:v>
+      </x:c>
+      <x:c r="F23" s="792" t="n">
+        <x:v>27.6</x:v>
+      </x:c>
+      <x:c r="G23" s="757" t="n">
+        <x:f>F23/E23</x:f>
+        <x:v>1.491891891891892</x:v>
+      </x:c>
+      <x:c r="H23" s="754" t="str">
+        <x:v>output32x64_stage4_adaptive</x:v>
+      </x:c>
+      <x:c r="I23" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="28" customHeight="1">
+      <x:c r="A24" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B24" s="754" t="str">
+        <x:v>512 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C24" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D24" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E24" s="792" t="n">
+        <x:v>24.1</x:v>
+      </x:c>
+      <x:c r="F24" s="792" t="n">
+        <x:v>27.6</x:v>
+      </x:c>
+      <x:c r="G24" s="757" t="n">
+        <x:f>F24/E24</x:f>
+        <x:v>1.1452282157676348</x:v>
+      </x:c>
+      <x:c r="H24" s="754" t="str">
+        <x:v>fixed_stage2_masked_epilogue</x:v>
+      </x:c>
+      <x:c r="I24" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="28" customHeight="1">
+      <x:c r="A25" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B25" s="754" t="str">
+        <x:v>1024 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C25" s="755" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="D25" s="755" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E25" s="792" t="n">
+        <x:v>38.7</x:v>
+      </x:c>
+      <x:c r="F25" s="792" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="G25" s="757" t="n">
+        <x:f>F25/E25</x:f>
+        <x:v>1.317829457364341</x:v>
+      </x:c>
+      <x:c r="H25" s="754" t="str">
+        <x:v>output64x64_three_cta_runtime_k</x:v>
+      </x:c>
+      <x:c r="I25" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="28" customHeight="1">
+      <x:c r="A26" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B26" s="754" t="str">
+        <x:v>2048 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C26" s="755" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="D26" s="755" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="E26" s="792" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="F26" s="792" t="n">
+        <x:v>97.1</x:v>
+      </x:c>
+      <x:c r="G26" s="757" t="n">
+        <x:f>F26/E26</x:f>
+        <x:v>1.2776315789473685</x:v>
+      </x:c>
+      <x:c r="H26" s="754" t="str">
+        <x:v>output128x64_stage4_full_tile</x:v>
+      </x:c>
+      <x:c r="I26" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="28" customHeight="1">
+      <x:c r="A27" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B27" s="754" t="str">
+        <x:v>4096 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C27" s="755" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="D27" s="755" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="E27" s="792" t="n">
+        <x:v>148.5</x:v>
+      </x:c>
+      <x:c r="F27" s="792" t="n">
+        <x:v>185.6</x:v>
+      </x:c>
+      <x:c r="G27" s="757" t="n">
+        <x:f>F27/E27</x:f>
+        <x:v>1.2498316498316497</x:v>
+      </x:c>
+      <x:c r="H27" s="754" t="str">
+        <x:v>output128x64_output_reuse_handshake</x:v>
+      </x:c>
+      <x:c r="I27" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="28" customHeight="1">
+      <x:c r="A28" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B28" s="754" t="str">
+        <x:v>128 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C28" s="755" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D28" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E28" s="792" t="n">
+        <x:v>23.5</x:v>
+      </x:c>
+      <x:c r="F28" s="792" t="n">
+        <x:v>28.6</x:v>
+      </x:c>
+      <x:c r="G28" s="757" t="n">
+        <x:f>F28/E28</x:f>
+        <x:v>1.2170212765957447</x:v>
+      </x:c>
+      <x:c r="H28" s="754" t="str">
+        <x:v>output64x128_stage2_single_wg</x:v>
+      </x:c>
+      <x:c r="I28" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="28" customHeight="1">
+      <x:c r="A29" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B29" s="754" t="str">
+        <x:v>256 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C29" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="D29" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E29" s="792" t="n">
+        <x:v>23.4</x:v>
+      </x:c>
+      <x:c r="F29" s="792" t="n">
+        <x:v>28.9</x:v>
+      </x:c>
+      <x:c r="G29" s="757" t="n">
+        <x:f>F29/E29</x:f>
+        <x:v>1.235042735042735</x:v>
+      </x:c>
+      <x:c r="H29" s="754" t="str">
+        <x:v>output64x128_stage2_single_wg</x:v>
+      </x:c>
+      <x:c r="I29" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="28" customHeight="1">
+      <x:c r="A30" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B30" s="754" t="str">
+        <x:v>512 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C30" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D30" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E30" s="792" t="n">
+        <x:v>22.9</x:v>
+      </x:c>
+      <x:c r="F30" s="792" t="n">
+        <x:v>28.9</x:v>
+      </x:c>
+      <x:c r="G30" s="757" t="n">
+        <x:f>F30/E30</x:f>
+        <x:v>1.262008733624454</x:v>
+      </x:c>
+      <x:c r="H30" s="754" t="str">
+        <x:v>output64x128_stage2_single_wg</x:v>
+      </x:c>
+      <x:c r="I30" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="28" customHeight="1">
+      <x:c r="A31" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B31" s="754" t="str">
+        <x:v>1024 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C31" s="755" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="D31" s="755" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E31" s="792" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="F31" s="792" t="n">
+        <x:v>53.3</x:v>
+      </x:c>
+      <x:c r="G31" s="757" t="n">
+        <x:f>F31/E31</x:f>
+        <x:v>1.2395348837209301</x:v>
+      </x:c>
+      <x:c r="H31" s="754" t="str">
+        <x:v>output128x64_output_reuse_handshake</x:v>
+      </x:c>
+      <x:c r="I31" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="28" customHeight="1">
+      <x:c r="A32" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B32" s="754" t="str">
+        <x:v>2048 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C32" s="755" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="D32" s="755" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="E32" s="792" t="n">
+        <x:v>75.3</x:v>
+      </x:c>
+      <x:c r="F32" s="792" t="n">
+        <x:v>101.1</x:v>
+      </x:c>
+      <x:c r="G32" s="757" t="n">
+        <x:f>F32/E32</x:f>
+        <x:v>1.342629482071713</x:v>
+      </x:c>
+      <x:c r="H32" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I32" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="28" customHeight="1">
+      <x:c r="A33" s="761" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B33" s="760" t="str">
+        <x:v>4096 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C33" s="761" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="D33" s="761" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="E33" s="793" t="n">
+        <x:v>144.9</x:v>
+      </x:c>
+      <x:c r="F33" s="793" t="n">
+        <x:v>197.6</x:v>
+      </x:c>
+      <x:c r="G33" s="763" t="n">
+        <x:f>F33/E33</x:f>
+        <x:v>1.3636991028295375</x:v>
+      </x:c>
+      <x:c r="H33" s="760" t="str">
+        <x:v>output128x64_output_reuse_handshake</x:v>
+      </x:c>
+      <x:c r="I33" s="761" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="442"/>
+      <x:c r="B34" s="442"/>
+      <x:c r="C34" s="442"/>
+      <x:c r="D34" s="442"/>
+      <x:c r="E34" s="442"/>
+      <x:c r="F34" s="442"/>
+      <x:c r="G34" s="442"/>
+      <x:c r="H34" s="442"/>
+      <x:c r="I34" s="442"/>
+    </x:row>
+    <x:row r="35" ht="32" customHeight="1">
+      <x:c r="A35" s="816" t="str">
+        <x:v>Speedup = DeepGEMM latency / hybrid latency. Each row uses the best currently dispatched kernel for that shape; values above 1.0x mean Hybrid Sparse is faster.</x:v>
+      </x:c>
+      <x:c r="B35" s="816"/>
+      <x:c r="C35" s="816"/>
+      <x:c r="D35" s="816"/>
+      <x:c r="E35" s="816"/>
+      <x:c r="F35" s="816"/>
+      <x:c r="G35" s="816"/>
+      <x:c r="H35" s="816"/>
+      <x:c r="I35" s="816"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:I1"/>
+    <x:mergeCell ref="A2:I2"/>
+    <x:mergeCell ref="A4:I4"/>
+    <x:mergeCell ref="A20:I20"/>
+    <x:mergeCell ref="A35:I35"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="H5:H5">
+    <x:cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThanOrEqual">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="12" priority="2" operator="lessThan">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="E10:E15">
+    <x:cfRule type="cellIs" dxfId="13" priority="3" operator="greaterThanOrEqual">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="14" priority="4" operator="lessThan">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G6:G17">
+    <x:cfRule type="cellIs" dxfId="19" priority="9" operator="greaterThanOrEqual">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="20" priority="10" operator="lessThan">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G22:G33">
+    <x:cfRule type="cellIs" dxfId="21" priority="11" operator="greaterThanOrEqual">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="22" priority="12" operator="lessThan">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="38" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="13" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="38" customHeight="1">
+      <x:c r="A1" s="843" t="str">
+        <x:v>Grouped GEMM Expert-Scaling Performance</x:v>
+      </x:c>
+      <x:c r="B1" s="843"/>
+      <x:c r="C1" s="843"/>
+      <x:c r="D1" s="843"/>
+      <x:c r="E1" s="843"/>
+      <x:c r="F1" s="843"/>
+      <x:c r="G1" s="843"/>
+      <x:c r="H1" s="843"/>
+      <x:c r="I1" s="843"/>
+    </x:row>
+    <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="839" t="str">
+        <x:v>NVIDIA H20 | BF16 input/output | FP32 accumulation | 64 x 64 weight blocks | 25% sparsity | Num Experts = 32 / 64 | 100 timing runs | L2 flush disabled</x:v>
+      </x:c>
+      <x:c r="B2" s="839"/>
+      <x:c r="C2" s="839"/>
+      <x:c r="D2" s="839"/>
+      <x:c r="E2" s="839"/>
+      <x:c r="F2" s="839"/>
+      <x:c r="G2" s="839"/>
+      <x:c r="H2" s="839"/>
+      <x:c r="I2" s="839"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="442"/>
+      <x:c r="B3" s="442"/>
+      <x:c r="C3" s="442"/>
+      <x:c r="D3" s="442"/>
+      <x:c r="E3" s="442"/>
+      <x:c r="F3" s="442"/>
+      <x:c r="G3" s="442"/>
+      <x:c r="H3" s="442"/>
+      <x:c r="I3" s="442"/>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="840" t="str">
+        <x:v>E32 Contiguous Grouped GEMM - Best Kernel per Shape</x:v>
+      </x:c>
+      <x:c r="B4" s="840"/>
+      <x:c r="C4" s="840"/>
+      <x:c r="D4" s="840"/>
+      <x:c r="E4" s="840"/>
+      <x:c r="F4" s="840"/>
+      <x:c r="G4" s="840"/>
+      <x:c r="H4" s="840"/>
+      <x:c r="I4" s="840"/>
+    </x:row>
+    <x:row r="5" ht="36" customHeight="1">
+      <x:c r="A5" s="841" t="str">
+        <x:v>Num Experts</x:v>
+      </x:c>
+      <x:c r="B5" s="841" t="str">
+        <x:v>Shape (Total M x N x K)</x:v>
+      </x:c>
+      <x:c r="C5" s="841" t="str">
+        <x:v>Tokens / Expert</x:v>
+      </x:c>
+      <x:c r="D5" s="841" t="str">
+        <x:v>Max M</x:v>
+      </x:c>
+      <x:c r="E5" s="841" t="str">
+        <x:v>Hybrid latency (us)</x:v>
+      </x:c>
+      <x:c r="F5" s="841" t="str">
+        <x:v>DeepGEMM latency (us)</x:v>
+      </x:c>
+      <x:c r="G5" s="841" t="str">
+        <x:v>Speedup</x:v>
+      </x:c>
+      <x:c r="H5" s="841" t="str">
+        <x:v>Best kernel version</x:v>
+      </x:c>
+      <x:c r="I5" s="841" t="str">
+        <x:v>Validation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="28" customHeight="1">
+      <x:c r="A6" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B6" s="754" t="str">
+        <x:v>128 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C6" s="755" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D6" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E6" s="792" t="n">
+        <x:v>164.3</x:v>
+      </x:c>
+      <x:c r="F6" s="792" t="n">
+        <x:v>187.2</x:v>
+      </x:c>
+      <x:c r="G6" s="757" t="n">
+        <x:f>F6/E6</x:f>
+        <x:v>1.139379184418746</x:v>
+      </x:c>
+      <x:c r="H6" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I6" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="28" customHeight="1">
+      <x:c r="A7" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B7" s="754" t="str">
+        <x:v>256 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C7" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D7" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E7" s="792" t="n">
+        <x:v>164.3</x:v>
+      </x:c>
+      <x:c r="F7" s="792" t="n">
+        <x:v>187.2</x:v>
+      </x:c>
+      <x:c r="G7" s="757" t="n">
+        <x:f>F7/E7</x:f>
+        <x:v>1.139379184418746</x:v>
+      </x:c>
+      <x:c r="H7" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I7" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="28" customHeight="1">
+      <x:c r="A8" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B8" s="754" t="str">
+        <x:v>512 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C8" s="755" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D8" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E8" s="792" t="n">
+        <x:v>163.3</x:v>
+      </x:c>
+      <x:c r="F8" s="792" t="n">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="G8" s="757" t="n">
+        <x:f>F8/E8</x:f>
+        <x:v>1.1451316595223515</x:v>
+      </x:c>
+      <x:c r="H8" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I8" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="28" customHeight="1">
+      <x:c r="A9" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B9" s="754" t="str">
+        <x:v>1024 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C9" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="D9" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E9" s="792" t="n">
+        <x:v>161.9</x:v>
+      </x:c>
+      <x:c r="F9" s="792" t="n">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="G9" s="757" t="n">
+        <x:f>F9/E9</x:f>
+        <x:v>1.1550339715873996</x:v>
+      </x:c>
+      <x:c r="H9" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I9" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="28" customHeight="1">
+      <x:c r="A10" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B10" s="754" t="str">
+        <x:v>2048 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C10" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D10" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E10" s="792" t="n">
+        <x:v>159.5</x:v>
+      </x:c>
+      <x:c r="F10" s="792" t="n">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="G10" s="757" t="n">
+        <x:f>F10/E10</x:f>
+        <x:v>1.1724137931034482</x:v>
+      </x:c>
+      <x:c r="H10" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I10" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="28" customHeight="1">
+      <x:c r="A11" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B11" s="754" t="str">
+        <x:v>4096 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C11" s="755" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="D11" s="755" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E11" s="792" t="n">
+        <x:v>154.3</x:v>
+      </x:c>
+      <x:c r="F11" s="792" t="n">
+        <x:v>187.5</x:v>
+      </x:c>
+      <x:c r="G11" s="757" t="n">
+        <x:f>F11/E11</x:f>
+        <x:v>1.2151652624756966</x:v>
+      </x:c>
+      <x:c r="H11" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I11" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="28" customHeight="1">
+      <x:c r="A12" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B12" s="754" t="str">
+        <x:v>128 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C12" s="755" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D12" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E12" s="792" t="n">
+        <x:v>168.9</x:v>
+      </x:c>
+      <x:c r="F12" s="792" t="n">
+        <x:v>198.8</x:v>
+      </x:c>
+      <x:c r="G12" s="757" t="n">
+        <x:f>F12/E12</x:f>
+        <x:v>1.177027827116637</x:v>
+      </x:c>
+      <x:c r="H12" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I12" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="28" customHeight="1">
+      <x:c r="A13" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B13" s="754" t="str">
+        <x:v>256 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C13" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D13" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E13" s="792" t="n">
+        <x:v>168.3</x:v>
+      </x:c>
+      <x:c r="F13" s="792" t="n">
+        <x:v>199.3</x:v>
+      </x:c>
+      <x:c r="G13" s="757" t="n">
+        <x:f>F13/E13</x:f>
+        <x:v>1.184194890077243</x:v>
+      </x:c>
+      <x:c r="H13" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I13" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="28" customHeight="1">
+      <x:c r="A14" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B14" s="754" t="str">
+        <x:v>512 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C14" s="755" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D14" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E14" s="792" t="n">
+        <x:v>167.6</x:v>
+      </x:c>
+      <x:c r="F14" s="792" t="n">
+        <x:v>199.1</x:v>
+      </x:c>
+      <x:c r="G14" s="757" t="n">
+        <x:f>F14/E14</x:f>
+        <x:v>1.187947494033413</x:v>
+      </x:c>
+      <x:c r="H14" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I14" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="28" customHeight="1">
+      <x:c r="A15" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B15" s="754" t="str">
+        <x:v>1024 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C15" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="D15" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E15" s="792" t="n">
+        <x:v>165.9</x:v>
+      </x:c>
+      <x:c r="F15" s="792" t="n">
+        <x:v>198.9</x:v>
+      </x:c>
+      <x:c r="G15" s="757" t="n">
+        <x:f>F15/E15</x:f>
+        <x:v>1.1989150090415912</x:v>
+      </x:c>
+      <x:c r="H15" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I15" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="28" customHeight="1">
+      <x:c r="A16" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B16" s="754" t="str">
+        <x:v>2048 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C16" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D16" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E16" s="792" t="n">
+        <x:v>162.1</x:v>
+      </x:c>
+      <x:c r="F16" s="792" t="n">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="G16" s="757" t="n">
+        <x:f>F16/E16</x:f>
+        <x:v>1.2276372609500308</x:v>
+      </x:c>
+      <x:c r="H16" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I16" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="28" customHeight="1">
+      <x:c r="A17" s="761" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B17" s="760" t="str">
+        <x:v>4096 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C17" s="761" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="D17" s="761" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E17" s="793" t="n">
+        <x:v>154.5</x:v>
+      </x:c>
+      <x:c r="F17" s="793" t="n">
+        <x:v>198.9</x:v>
+      </x:c>
+      <x:c r="G17" s="763" t="n">
+        <x:f>F17/E17</x:f>
+        <x:v>1.2873786407766992</x:v>
+      </x:c>
+      <x:c r="H17" s="760" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I17" s="761" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="442"/>
+      <x:c r="B18" s="442"/>
+      <x:c r="C18" s="442"/>
+      <x:c r="D18" s="442"/>
+      <x:c r="E18" s="442"/>
+      <x:c r="F18" s="442"/>
+      <x:c r="G18" s="442"/>
+      <x:c r="H18" s="442"/>
+      <x:c r="I18" s="442"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="442"/>
+      <x:c r="B19" s="442"/>
+      <x:c r="C19" s="442"/>
+      <x:c r="D19" s="442"/>
+      <x:c r="E19" s="442"/>
+      <x:c r="F19" s="442"/>
+      <x:c r="G19" s="442"/>
+      <x:c r="H19" s="442"/>
+      <x:c r="I19" s="442"/>
+    </x:row>
+    <x:row r="20" ht="28" customHeight="1">
+      <x:c r="A20" s="840" t="str">
+        <x:v>E32 Masked Grouped GEMM - Best Kernel per Shape</x:v>
+      </x:c>
+      <x:c r="B20" s="840"/>
+      <x:c r="C20" s="840"/>
+      <x:c r="D20" s="840"/>
+      <x:c r="E20" s="840"/>
+      <x:c r="F20" s="840"/>
+      <x:c r="G20" s="840"/>
+      <x:c r="H20" s="840"/>
+      <x:c r="I20" s="840"/>
+    </x:row>
+    <x:row r="21" ht="36" customHeight="1">
+      <x:c r="A21" s="841" t="str">
+        <x:v>Num Experts</x:v>
+      </x:c>
+      <x:c r="B21" s="841" t="str">
+        <x:v>Shape (Total M x N x K)</x:v>
+      </x:c>
+      <x:c r="C21" s="841" t="str">
+        <x:v>Tokens / Expert</x:v>
+      </x:c>
+      <x:c r="D21" s="841" t="str">
+        <x:v>Max M</x:v>
+      </x:c>
+      <x:c r="E21" s="841" t="str">
+        <x:v>Hybrid latency (us)</x:v>
+      </x:c>
+      <x:c r="F21" s="841" t="str">
+        <x:v>DeepGEMM latency (us)</x:v>
+      </x:c>
+      <x:c r="G21" s="841" t="str">
+        <x:v>Speedup</x:v>
+      </x:c>
+      <x:c r="H21" s="841" t="str">
+        <x:v>Best kernel version</x:v>
+      </x:c>
+      <x:c r="I21" s="841" t="str">
+        <x:v>Validation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="28" customHeight="1">
+      <x:c r="A22" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B22" s="754" t="str">
+        <x:v>128 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C22" s="755" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D22" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E22" s="792" t="n">
+        <x:v>65.1</x:v>
+      </x:c>
+      <x:c r="F22" s="792" t="n">
+        <x:v>97.9</x:v>
+      </x:c>
+      <x:c r="G22" s="757" t="n">
+        <x:f>F22/E22</x:f>
+        <x:v>1.5038402457757298</x:v>
+      </x:c>
+      <x:c r="H22" s="754" t="str">
+        <x:v>output32x64_stage4_adaptive</x:v>
+      </x:c>
+      <x:c r="I22" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="28" customHeight="1">
+      <x:c r="A23" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B23" s="754" t="str">
+        <x:v>256 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C23" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D23" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E23" s="792" t="n">
+        <x:v>73.6</x:v>
+      </x:c>
+      <x:c r="F23" s="792" t="n">
+        <x:v>98.6</x:v>
+      </x:c>
+      <x:c r="G23" s="757" t="n">
+        <x:f>F23/E23</x:f>
+        <x:v>1.3396739130434783</x:v>
+      </x:c>
+      <x:c r="H23" s="754" t="str">
+        <x:v>output32x64_stage4_adaptive</x:v>
+      </x:c>
+      <x:c r="I23" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="28" customHeight="1">
+      <x:c r="A24" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B24" s="754" t="str">
+        <x:v>512 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C24" s="755" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D24" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E24" s="792" t="n">
+        <x:v>64.7</x:v>
+      </x:c>
+      <x:c r="F24" s="792" t="n">
+        <x:v>97.9</x:v>
+      </x:c>
+      <x:c r="G24" s="757" t="n">
+        <x:f>F24/E24</x:f>
+        <x:v>1.5131375579598145</x:v>
+      </x:c>
+      <x:c r="H24" s="754" t="str">
+        <x:v>output32x64_stage4_adaptive</x:v>
+      </x:c>
+      <x:c r="I24" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="28" customHeight="1">
+      <x:c r="A25" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B25" s="754" t="str">
+        <x:v>1024 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C25" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="D25" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E25" s="792" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="F25" s="792" t="n">
+        <x:v>98.9</x:v>
+      </x:c>
+      <x:c r="G25" s="757" t="n">
+        <x:f>F25/E25</x:f>
+        <x:v>1.5453125</x:v>
+      </x:c>
+      <x:c r="H25" s="754" t="str">
+        <x:v>output32x64_stage4_adaptive</x:v>
+      </x:c>
+      <x:c r="I25" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="28" customHeight="1">
+      <x:c r="A26" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B26" s="754" t="str">
+        <x:v>2048 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C26" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D26" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E26" s="792" t="n">
+        <x:v>85.5</x:v>
+      </x:c>
+      <x:c r="F26" s="792" t="n">
+        <x:v>98.6</x:v>
+      </x:c>
+      <x:c r="G26" s="757" t="n">
+        <x:f>F26/E26</x:f>
+        <x:v>1.1532163742690058</x:v>
+      </x:c>
+      <x:c r="H26" s="754" t="str">
+        <x:v>fixed_stage2_masked_epilogue</x:v>
+      </x:c>
+      <x:c r="I26" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="28" customHeight="1">
+      <x:c r="A27" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B27" s="754" t="str">
+        <x:v>4096 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C27" s="755" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="D27" s="755" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E27" s="792" t="n">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="F27" s="792" t="n">
+        <x:v>188.1</x:v>
+      </x:c>
+      <x:c r="G27" s="757" t="n">
+        <x:f>F27/E27</x:f>
+        <x:v>1.3153846153846154</x:v>
+      </x:c>
+      <x:c r="H27" s="754" t="str">
+        <x:v>output64x64_three_cta_runtime_k</x:v>
+      </x:c>
+      <x:c r="I27" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="28" customHeight="1">
+      <x:c r="A28" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B28" s="754" t="str">
+        <x:v>128 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C28" s="755" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D28" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E28" s="792" t="n">
+        <x:v>91.3</x:v>
+      </x:c>
+      <x:c r="F28" s="792" t="n">
+        <x:v>96.8</x:v>
+      </x:c>
+      <x:c r="G28" s="757" t="n">
+        <x:f>F28/E28</x:f>
+        <x:v>1.0602409638554218</x:v>
+      </x:c>
+      <x:c r="H28" s="754" t="str">
+        <x:v>output64x128_stage2_single_wg</x:v>
+      </x:c>
+      <x:c r="I28" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="28" customHeight="1">
+      <x:c r="A29" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B29" s="754" t="str">
+        <x:v>256 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C29" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D29" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E29" s="792" t="n">
+        <x:v>91.1</x:v>
+      </x:c>
+      <x:c r="F29" s="792" t="n">
+        <x:v>96.7</x:v>
+      </x:c>
+      <x:c r="G29" s="757" t="n">
+        <x:f>F29/E29</x:f>
+        <x:v>1.061470911086718</x:v>
+      </x:c>
+      <x:c r="H29" s="754" t="str">
+        <x:v>output64x128_stage2_single_wg</x:v>
+      </x:c>
+      <x:c r="I29" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="28" customHeight="1">
+      <x:c r="A30" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B30" s="754" t="str">
+        <x:v>512 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C30" s="755" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D30" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E30" s="792" t="n">
+        <x:v>90.7</x:v>
+      </x:c>
+      <x:c r="F30" s="792" t="n">
+        <x:v>96.8</x:v>
+      </x:c>
+      <x:c r="G30" s="757" t="n">
+        <x:f>F30/E30</x:f>
+        <x:v>1.0672546857772878</x:v>
+      </x:c>
+      <x:c r="H30" s="754" t="str">
+        <x:v>output64x128_stage2_single_wg</x:v>
+      </x:c>
+      <x:c r="I30" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="28" customHeight="1">
+      <x:c r="A31" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B31" s="754" t="str">
+        <x:v>1024 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C31" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="D31" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E31" s="792" t="n">
+        <x:v>90.1</x:v>
+      </x:c>
+      <x:c r="F31" s="792" t="n">
+        <x:v>96.5</x:v>
+      </x:c>
+      <x:c r="G31" s="757" t="n">
+        <x:f>F31/E31</x:f>
+        <x:v>1.0710321864594896</x:v>
+      </x:c>
+      <x:c r="H31" s="754" t="str">
+        <x:v>output64x128_stage2_single_wg</x:v>
+      </x:c>
+      <x:c r="I31" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="28" customHeight="1">
+      <x:c r="A32" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B32" s="754" t="str">
+        <x:v>2048 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C32" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D32" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E32" s="792" t="n">
+        <x:v>88.8</x:v>
+      </x:c>
+      <x:c r="F32" s="792" t="n">
+        <x:v>96.8</x:v>
+      </x:c>
+      <x:c r="G32" s="757" t="n">
+        <x:f>F32/E32</x:f>
+        <x:v>1.09009009009009</x:v>
+      </x:c>
+      <x:c r="H32" s="754" t="str">
+        <x:v>output64x128_stage2_single_wg</x:v>
+      </x:c>
+      <x:c r="I32" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="28" customHeight="1">
+      <x:c r="A33" s="761" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B33" s="760" t="str">
+        <x:v>4096 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C33" s="761" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="D33" s="761" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E33" s="793" t="n">
+        <x:v>148.2</x:v>
+      </x:c>
+      <x:c r="F33" s="793" t="n">
+        <x:v>199.5</x:v>
+      </x:c>
+      <x:c r="G33" s="763" t="n">
+        <x:f>F33/E33</x:f>
+        <x:v>1.3461538461538463</x:v>
+      </x:c>
+      <x:c r="H33" s="760" t="str">
+        <x:v>output128x64_output_reuse_handshake</x:v>
+      </x:c>
+      <x:c r="I33" s="761" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="442"/>
+      <x:c r="B34" s="442"/>
+      <x:c r="C34" s="442"/>
+      <x:c r="D34" s="442"/>
+      <x:c r="E34" s="442"/>
+      <x:c r="F34" s="442"/>
+      <x:c r="G34" s="442"/>
+      <x:c r="H34" s="442"/>
+      <x:c r="I34" s="442"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="442"/>
+      <x:c r="B35" s="442"/>
+      <x:c r="C35" s="442"/>
+      <x:c r="D35" s="442"/>
+      <x:c r="E35" s="442"/>
+      <x:c r="F35" s="442"/>
+      <x:c r="G35" s="442"/>
+      <x:c r="H35" s="442"/>
+      <x:c r="I35" s="442"/>
+    </x:row>
+    <x:row r="36" ht="28" customHeight="1">
+      <x:c r="A36" s="840" t="str">
+        <x:v>E64 Contiguous Grouped GEMM - Best Kernel per Shape</x:v>
+      </x:c>
+      <x:c r="B36" s="840"/>
+      <x:c r="C36" s="840"/>
+      <x:c r="D36" s="840"/>
+      <x:c r="E36" s="840"/>
+      <x:c r="F36" s="840"/>
+      <x:c r="G36" s="840"/>
+      <x:c r="H36" s="840"/>
+      <x:c r="I36" s="840"/>
+    </x:row>
+    <x:row r="37" ht="36" customHeight="1">
+      <x:c r="A37" s="841" t="str">
+        <x:v>Num Experts</x:v>
+      </x:c>
+      <x:c r="B37" s="841" t="str">
+        <x:v>Shape (Total M x N x K)</x:v>
+      </x:c>
+      <x:c r="C37" s="841" t="str">
+        <x:v>Tokens / Expert</x:v>
+      </x:c>
+      <x:c r="D37" s="841" t="str">
+        <x:v>Max M</x:v>
+      </x:c>
+      <x:c r="E37" s="841" t="str">
+        <x:v>Hybrid latency (us)</x:v>
+      </x:c>
+      <x:c r="F37" s="841" t="str">
+        <x:v>DeepGEMM latency (us)</x:v>
+      </x:c>
+      <x:c r="G37" s="841" t="str">
+        <x:v>Speedup</x:v>
+      </x:c>
+      <x:c r="H37" s="841" t="str">
+        <x:v>Best kernel version</x:v>
+      </x:c>
+      <x:c r="I37" s="841" t="str">
+        <x:v>Validation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="28" customHeight="1">
+      <x:c r="A38" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B38" s="754" t="str">
+        <x:v>128 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C38" s="755" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D38" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E38" s="792" t="n">
+        <x:v>320.8</x:v>
+      </x:c>
+      <x:c r="F38" s="792" t="n">
+        <x:v>356.2</x:v>
+      </x:c>
+      <x:c r="G38" s="757" t="n">
+        <x:f>F38/E38</x:f>
+        <x:v>1.1103491271820447</x:v>
+      </x:c>
+      <x:c r="H38" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I38" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="28" customHeight="1">
+      <x:c r="A39" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B39" s="754" t="str">
+        <x:v>256 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C39" s="755" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D39" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E39" s="792" t="n">
+        <x:v>320.2</x:v>
+      </x:c>
+      <x:c r="F39" s="792" t="n">
+        <x:v>355.8</x:v>
+      </x:c>
+      <x:c r="G39" s="757" t="n">
+        <x:f>F39/E39</x:f>
+        <x:v>1.1111805121798877</x:v>
+      </x:c>
+      <x:c r="H39" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I39" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="28" customHeight="1">
+      <x:c r="A40" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B40" s="754" t="str">
+        <x:v>512 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C40" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D40" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E40" s="792" t="n">
+        <x:v>319.6</x:v>
+      </x:c>
+      <x:c r="F40" s="792" t="n">
+        <x:v>356.2</x:v>
+      </x:c>
+      <x:c r="G40" s="757" t="n">
+        <x:f>F40/E40</x:f>
+        <x:v>1.1145181476846056</x:v>
+      </x:c>
+      <x:c r="H40" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I40" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="28" customHeight="1">
+      <x:c r="A41" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B41" s="754" t="str">
+        <x:v>1024 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C41" s="755" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D41" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E41" s="792" t="n">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="F41" s="792" t="n">
+        <x:v>356.3</x:v>
+      </x:c>
+      <x:c r="G41" s="757" t="n">
+        <x:f>F41/E41</x:f>
+        <x:v>1.1134375</x:v>
+      </x:c>
+      <x:c r="H41" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I41" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="28" customHeight="1">
+      <x:c r="A42" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B42" s="754" t="str">
+        <x:v>2048 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C42" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="D42" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E42" s="792" t="n">
+        <x:v>319.3</x:v>
+      </x:c>
+      <x:c r="F42" s="792" t="n">
+        <x:v>357.8</x:v>
+      </x:c>
+      <x:c r="G42" s="757" t="n">
+        <x:f>F42/E42</x:f>
+        <x:v>1.120576260569997</x:v>
+      </x:c>
+      <x:c r="H42" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I42" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="28" customHeight="1">
+      <x:c r="A43" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B43" s="754" t="str">
+        <x:v>4096 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C43" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D43" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E43" s="792" t="n">
+        <x:v>312.4</x:v>
+      </x:c>
+      <x:c r="F43" s="792" t="n">
+        <x:v>356.5</x:v>
+      </x:c>
+      <x:c r="G43" s="757" t="n">
+        <x:f>F43/E43</x:f>
+        <x:v>1.1411651728553138</x:v>
+      </x:c>
+      <x:c r="H43" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I43" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="28" customHeight="1">
+      <x:c r="A44" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B44" s="754" t="str">
+        <x:v>128 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C44" s="755" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D44" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E44" s="792" t="n">
+        <x:v>339</x:v>
+      </x:c>
+      <x:c r="F44" s="792" t="n">
+        <x:v>367.1</x:v>
+      </x:c>
+      <x:c r="G44" s="757" t="n">
+        <x:f>F44/E44</x:f>
+        <x:v>1.0828908554572272</x:v>
+      </x:c>
+      <x:c r="H44" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I44" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="28" customHeight="1">
+      <x:c r="A45" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B45" s="754" t="str">
+        <x:v>256 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C45" s="755" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D45" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E45" s="792" t="n">
+        <x:v>339.3</x:v>
+      </x:c>
+      <x:c r="F45" s="792" t="n">
+        <x:v>367</x:v>
+      </x:c>
+      <x:c r="G45" s="757" t="n">
+        <x:f>F45/E45</x:f>
+        <x:v>1.0816386678455643</x:v>
+      </x:c>
+      <x:c r="H45" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I45" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="28" customHeight="1">
+      <x:c r="A46" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B46" s="754" t="str">
+        <x:v>512 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C46" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D46" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E46" s="792" t="n">
+        <x:v>337.9</x:v>
+      </x:c>
+      <x:c r="F46" s="792" t="n">
+        <x:v>367.4</x:v>
+      </x:c>
+      <x:c r="G46" s="757" t="n">
+        <x:f>F46/E46</x:f>
+        <x:v>1.0873039360757621</x:v>
+      </x:c>
+      <x:c r="H46" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I46" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="28" customHeight="1">
+      <x:c r="A47" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B47" s="754" t="str">
+        <x:v>1024 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C47" s="755" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D47" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E47" s="792" t="n">
+        <x:v>337.1</x:v>
+      </x:c>
+      <x:c r="F47" s="792" t="n">
+        <x:v>367.1</x:v>
+      </x:c>
+      <x:c r="G47" s="757" t="n">
+        <x:f>F47/E47</x:f>
+        <x:v>1.0889943636902997</x:v>
+      </x:c>
+      <x:c r="H47" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I47" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="28" customHeight="1">
+      <x:c r="A48" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B48" s="754" t="str">
+        <x:v>2048 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C48" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="D48" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E48" s="792" t="n">
+        <x:v>333.4</x:v>
+      </x:c>
+      <x:c r="F48" s="792" t="n">
+        <x:v>366.6</x:v>
+      </x:c>
+      <x:c r="G48" s="757" t="n">
+        <x:f>F48/E48</x:f>
+        <x:v>1.0995800839832035</x:v>
+      </x:c>
+      <x:c r="H48" s="754" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I48" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="28" customHeight="1">
+      <x:c r="A49" s="761" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B49" s="760" t="str">
+        <x:v>4096 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C49" s="761" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D49" s="761" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E49" s="793" t="n">
+        <x:v>326.6</x:v>
+      </x:c>
+      <x:c r="F49" s="793" t="n">
+        <x:v>368.7</x:v>
+      </x:c>
+      <x:c r="G49" s="763" t="n">
+        <x:f>F49/E49</x:f>
+        <x:v>1.1289038579301898</x:v>
+      </x:c>
+      <x:c r="H49" s="760" t="str">
+        <x:v>output128x64_persistent</x:v>
+      </x:c>
+      <x:c r="I49" s="761" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="442"/>
+      <x:c r="B50" s="442"/>
+      <x:c r="C50" s="442"/>
+      <x:c r="D50" s="442"/>
+      <x:c r="E50" s="442"/>
+      <x:c r="F50" s="442"/>
+      <x:c r="G50" s="442"/>
+      <x:c r="H50" s="442"/>
+      <x:c r="I50" s="442"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="442"/>
+      <x:c r="B51" s="442"/>
+      <x:c r="C51" s="442"/>
+      <x:c r="D51" s="442"/>
+      <x:c r="E51" s="442"/>
+      <x:c r="F51" s="442"/>
+      <x:c r="G51" s="442"/>
+      <x:c r="H51" s="442"/>
+      <x:c r="I51" s="442"/>
+    </x:row>
+    <x:row r="52" ht="28" customHeight="1">
+      <x:c r="A52" s="840" t="str">
+        <x:v>E64 Masked Grouped GEMM - Best Kernel per Shape</x:v>
+      </x:c>
+      <x:c r="B52" s="840"/>
+      <x:c r="C52" s="840"/>
+      <x:c r="D52" s="840"/>
+      <x:c r="E52" s="840"/>
+      <x:c r="F52" s="840"/>
+      <x:c r="G52" s="840"/>
+      <x:c r="H52" s="840"/>
+      <x:c r="I52" s="840"/>
+    </x:row>
+    <x:row r="53" ht="36" customHeight="1">
+      <x:c r="A53" s="841" t="str">
+        <x:v>Num Experts</x:v>
+      </x:c>
+      <x:c r="B53" s="841" t="str">
+        <x:v>Shape (Total M x N x K)</x:v>
+      </x:c>
+      <x:c r="C53" s="841" t="str">
+        <x:v>Tokens / Expert</x:v>
+      </x:c>
+      <x:c r="D53" s="841" t="str">
+        <x:v>Max M</x:v>
+      </x:c>
+      <x:c r="E53" s="841" t="str">
+        <x:v>Hybrid latency (us)</x:v>
+      </x:c>
+      <x:c r="F53" s="841" t="str">
+        <x:v>DeepGEMM latency (us)</x:v>
+      </x:c>
+      <x:c r="G53" s="841" t="str">
+        <x:v>Speedup</x:v>
+      </x:c>
+      <x:c r="H53" s="841" t="str">
+        <x:v>Best kernel version</x:v>
+      </x:c>
+      <x:c r="I53" s="841" t="str">
+        <x:v>Validation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="28" customHeight="1">
+      <x:c r="A54" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B54" s="754" t="str">
+        <x:v>128 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C54" s="755" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D54" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E54" s="792" t="n">
+        <x:v>127.5</x:v>
+      </x:c>
+      <x:c r="F54" s="792" t="n">
+        <x:v>186.4</x:v>
+      </x:c>
+      <x:c r="G54" s="757" t="n">
+        <x:f>F54/E54</x:f>
+        <x:v>1.4619607843137254</x:v>
+      </x:c>
+      <x:c r="H54" s="754" t="str">
+        <x:v>output32x64_stage4_adaptive</x:v>
+      </x:c>
+      <x:c r="I54" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="28" customHeight="1">
+      <x:c r="A55" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B55" s="754" t="str">
+        <x:v>256 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C55" s="755" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D55" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E55" s="792" t="n">
+        <x:v>127.5</x:v>
+      </x:c>
+      <x:c r="F55" s="792" t="n">
+        <x:v>185.8</x:v>
+      </x:c>
+      <x:c r="G55" s="757" t="n">
+        <x:f>F55/E55</x:f>
+        <x:v>1.4572549019607843</x:v>
+      </x:c>
+      <x:c r="H55" s="754" t="str">
+        <x:v>output32x64_stage4_adaptive</x:v>
+      </x:c>
+      <x:c r="I55" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="28" customHeight="1">
+      <x:c r="A56" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B56" s="754" t="str">
+        <x:v>512 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C56" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D56" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E56" s="792" t="n">
+        <x:v>127.3</x:v>
+      </x:c>
+      <x:c r="F56" s="792" t="n">
+        <x:v>186.1</x:v>
+      </x:c>
+      <x:c r="G56" s="757" t="n">
+        <x:f>F56/E56</x:f>
+        <x:v>1.4619010212097407</x:v>
+      </x:c>
+      <x:c r="H56" s="754" t="str">
+        <x:v>output32x64_stage4_adaptive</x:v>
+      </x:c>
+      <x:c r="I56" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="28" customHeight="1">
+      <x:c r="A57" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B57" s="754" t="str">
+        <x:v>1024 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C57" s="755" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D57" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E57" s="792" t="n">
+        <x:v>126.9</x:v>
+      </x:c>
+      <x:c r="F57" s="792" t="n">
+        <x:v>185.7</x:v>
+      </x:c>
+      <x:c r="G57" s="757" t="n">
+        <x:f>F57/E57</x:f>
+        <x:v>1.4633569739952716</x:v>
+      </x:c>
+      <x:c r="H57" s="754" t="str">
+        <x:v>output32x64_stage4_adaptive</x:v>
+      </x:c>
+      <x:c r="I57" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="28" customHeight="1">
+      <x:c r="A58" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B58" s="754" t="str">
+        <x:v>2048 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C58" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="D58" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E58" s="792" t="n">
+        <x:v>125.7</x:v>
+      </x:c>
+      <x:c r="F58" s="792" t="n">
+        <x:v>185.9</x:v>
+      </x:c>
+      <x:c r="G58" s="757" t="n">
+        <x:f>F58/E58</x:f>
+        <x:v>1.4789180588703261</x:v>
+      </x:c>
+      <x:c r="H58" s="754" t="str">
+        <x:v>output32x64_stage4_adaptive</x:v>
+      </x:c>
+      <x:c r="I58" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="28" customHeight="1">
+      <x:c r="A59" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B59" s="754" t="str">
+        <x:v>4096 x 1408 x 2048</x:v>
+      </x:c>
+      <x:c r="C59" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D59" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E59" s="792" t="n">
+        <x:v>160.4</x:v>
+      </x:c>
+      <x:c r="F59" s="792" t="n">
+        <x:v>185.7</x:v>
+      </x:c>
+      <x:c r="G59" s="757" t="n">
+        <x:f>F59/E59</x:f>
+        <x:v>1.157730673316708</x:v>
+      </x:c>
+      <x:c r="H59" s="754" t="str">
+        <x:v>fixed_stage2_masked_epilogue</x:v>
+      </x:c>
+      <x:c r="I59" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="28" customHeight="1">
+      <x:c r="A60" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B60" s="754" t="str">
+        <x:v>128 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C60" s="755" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D60" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E60" s="792" t="n">
+        <x:v>161.6</x:v>
+      </x:c>
+      <x:c r="F60" s="792" t="n">
+        <x:v>190.2</x:v>
+      </x:c>
+      <x:c r="G60" s="757" t="n">
+        <x:f>F60/E60</x:f>
+        <x:v>1.176980198019802</x:v>
+      </x:c>
+      <x:c r="H60" s="754" t="str">
+        <x:v>output64x128_stage2_single_wg</x:v>
+      </x:c>
+      <x:c r="I60" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="28" customHeight="1">
+      <x:c r="A61" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B61" s="754" t="str">
+        <x:v>256 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C61" s="755" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D61" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E61" s="792" t="n">
+        <x:v>161.4</x:v>
+      </x:c>
+      <x:c r="F61" s="792" t="n">
+        <x:v>190.7</x:v>
+      </x:c>
+      <x:c r="G61" s="757" t="n">
+        <x:f>F61/E61</x:f>
+        <x:v>1.181536555142503</x:v>
+      </x:c>
+      <x:c r="H61" s="754" t="str">
+        <x:v>output64x128_stage2_single_wg</x:v>
+      </x:c>
+      <x:c r="I61" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="28" customHeight="1">
+      <x:c r="A62" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B62" s="754" t="str">
+        <x:v>512 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C62" s="755" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D62" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E62" s="792" t="n">
+        <x:v>161.5</x:v>
+      </x:c>
+      <x:c r="F62" s="792" t="n">
+        <x:v>190.4</x:v>
+      </x:c>
+      <x:c r="G62" s="757" t="n">
+        <x:f>F62/E62</x:f>
+        <x:v>1.1789473684210527</x:v>
+      </x:c>
+      <x:c r="H62" s="754" t="str">
+        <x:v>output64x128_stage2_single_wg</x:v>
+      </x:c>
+      <x:c r="I62" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="28" customHeight="1">
+      <x:c r="A63" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B63" s="754" t="str">
+        <x:v>1024 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C63" s="755" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D63" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E63" s="792" t="n">
+        <x:v>160.6</x:v>
+      </x:c>
+      <x:c r="F63" s="792" t="n">
+        <x:v>190.5</x:v>
+      </x:c>
+      <x:c r="G63" s="757" t="n">
+        <x:f>F63/E63</x:f>
+        <x:v>1.1861768368617684</x:v>
+      </x:c>
+      <x:c r="H63" s="754" t="str">
+        <x:v>output64x128_stage2_single_wg</x:v>
+      </x:c>
+      <x:c r="I63" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="28" customHeight="1">
+      <x:c r="A64" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B64" s="754" t="str">
+        <x:v>2048 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C64" s="755" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="D64" s="755" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E64" s="792" t="n">
+        <x:v>159.4</x:v>
+      </x:c>
+      <x:c r="F64" s="792" t="n">
+        <x:v>190.6</x:v>
+      </x:c>
+      <x:c r="G64" s="757" t="n">
+        <x:f>F64/E64</x:f>
+        <x:v>1.1957340025094103</x:v>
+      </x:c>
+      <x:c r="H64" s="754" t="str">
+        <x:v>output64x128_stage2_single_wg</x:v>
+      </x:c>
+      <x:c r="I64" s="755" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="28" customHeight="1">
+      <x:c r="A65" s="761" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B65" s="760" t="str">
+        <x:v>4096 x 2048 x 1408</x:v>
+      </x:c>
+      <x:c r="C65" s="761" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D65" s="761" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E65" s="793" t="n">
+        <x:v>156.7</x:v>
+      </x:c>
+      <x:c r="F65" s="793" t="n">
+        <x:v>190.4</x:v>
+      </x:c>
+      <x:c r="G65" s="763" t="n">
+        <x:f>F65/E65</x:f>
+        <x:v>1.2150606253988514</x:v>
+      </x:c>
+      <x:c r="H65" s="760" t="str">
+        <x:v>output64x128_stage2_single_wg</x:v>
+      </x:c>
+      <x:c r="I65" s="761" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="442"/>
+      <x:c r="B66" s="442"/>
+      <x:c r="C66" s="442"/>
+      <x:c r="D66" s="442"/>
+      <x:c r="E66" s="442"/>
+      <x:c r="F66" s="442"/>
+      <x:c r="G66" s="442"/>
+      <x:c r="H66" s="442"/>
+      <x:c r="I66" s="442"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="442"/>
+      <x:c r="B67" s="442"/>
+      <x:c r="C67" s="442"/>
+      <x:c r="D67" s="442"/>
+      <x:c r="E67" s="442"/>
+      <x:c r="F67" s="442"/>
+      <x:c r="G67" s="442"/>
+      <x:c r="H67" s="442"/>
+      <x:c r="I67" s="442"/>
+    </x:row>
+    <x:row r="68" ht="34" customHeight="1">
+      <x:c r="A68" s="842" t="str">
+        <x:v>Speedup = DeepGEMM latency / hybrid latency. Total valid M is fixed while tokens/expert decreases as expert count grows. Every row uses the best currently dispatched kernel and passed the benchmark output comparison.</x:v>
+      </x:c>
+      <x:c r="B68" s="842"/>
+      <x:c r="C68" s="842"/>
+      <x:c r="D68" s="842"/>
+      <x:c r="E68" s="842"/>
+      <x:c r="F68" s="842"/>
+      <x:c r="G68" s="842"/>
+      <x:c r="H68" s="842"/>
+      <x:c r="I68" s="842"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:I1"/>
+    <x:mergeCell ref="A2:I2"/>
+    <x:mergeCell ref="A4:I4"/>
+    <x:mergeCell ref="A20:I20"/>
+    <x:mergeCell ref="A36:I36"/>
+    <x:mergeCell ref="A52:I52"/>
+    <x:mergeCell ref="A68:I68"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="G6:G17">
+    <x:cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThanOrEqual">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="24" priority="2" operator="lessThan">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G22:G33">
+    <x:cfRule type="cellIs" dxfId="25" priority="3" operator="greaterThanOrEqual">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="26" priority="4" operator="lessThan">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G38:G49">
+    <x:cfRule type="cellIs" dxfId="27" priority="5" operator="greaterThanOrEqual">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="28" priority="6" operator="lessThan">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G54:G65">
+    <x:cfRule type="cellIs" dxfId="29" priority="7" operator="greaterThanOrEqual">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="30" priority="8" operator="lessThan">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>

</xml_diff>